<commit_message>
Complete draft of run reconstruction, 1984-2024
</commit_message>
<xml_diff>
--- a/data-raw/freshwater-catch.xlsx
+++ b/data-raw/freshwater-catch.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\skrunchy2025\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{776C660A-5AA6-438F-BCE2-B9F1306EFBA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4971EBDF-908C-4135-B749-853392DA798D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E0CDEE87-6CC2-4107-81B9-F1AD4EA649A7}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E0CDEE87-6CC2-4107-81B9-F1AD4EA649A7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="34">
   <si>
     <t>Year</t>
   </si>
@@ -133,6 +133,12 @@
   <si>
     <t xml:space="preserve">LW </t>
   </si>
+  <si>
+    <t>LW: 2021-2024 are all place-holders (except for Tyee catch which is correct)</t>
+  </si>
+  <si>
+    <t>LW: Double check rec catch above Terrace for 2002, 2003, 2007</t>
+  </si>
 </sst>
 </file>
 
@@ -179,7 +185,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -222,6 +228,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -248,7 +260,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -304,6 +316,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -326,9 +341,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -366,7 +381,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -472,7 +487,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -614,7 +629,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1301,7 +1316,7 @@
         <v>2007</v>
       </c>
       <c r="M9" s="23">
-        <f t="shared" si="4"/>
+        <f>SUM(J9,K9)</f>
         <v>0</v>
       </c>
       <c r="N9" s="1">
@@ -1443,11 +1458,11 @@
         <v>2197</v>
       </c>
       <c r="G11" s="6">
-        <f t="shared" si="2"/>
+        <f>E11-F11</f>
         <v>1098</v>
       </c>
       <c r="L11" s="7">
-        <f t="shared" si="3"/>
+        <f>SUM(F11,H11,I11)</f>
         <v>2197</v>
       </c>
       <c r="M11" s="23">
@@ -1514,7 +1529,7 @@
         <v>4521</v>
       </c>
       <c r="F12" s="6">
-        <f t="shared" si="1"/>
+        <f>ROUND((E12*2/3),0)</f>
         <v>3014</v>
       </c>
       <c r="G12" s="6">
@@ -1964,7 +1979,7 @@
         <v>2798</v>
       </c>
       <c r="F18" s="6">
-        <f t="shared" si="1"/>
+        <f>ROUND((E18*2/3),0)</f>
         <v>1865</v>
       </c>
       <c r="G18" s="6">
@@ -2194,7 +2209,7 @@
         <v>1000</v>
       </c>
       <c r="L21" s="7">
-        <f t="shared" si="3"/>
+        <f>SUM(F21,H21,I21)</f>
         <v>2500</v>
       </c>
       <c r="M21" s="23">
@@ -2409,7 +2424,7 @@
         <v>5000</v>
       </c>
       <c r="G24" s="11">
-        <f t="shared" si="2"/>
+        <f>E24-F24</f>
         <v>1000</v>
       </c>
       <c r="L24" s="7">
@@ -2480,7 +2495,9 @@
         <v>3962</v>
       </c>
       <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
+      <c r="G25" s="29">
+        <v>0</v>
+      </c>
       <c r="H25" s="1">
         <v>3962</v>
       </c>
@@ -2552,7 +2569,9 @@
         <v>6280</v>
       </c>
       <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
+      <c r="G26" s="29">
+        <v>0</v>
+      </c>
       <c r="H26" s="1">
         <v>5711</v>
       </c>
@@ -2566,11 +2585,11 @@
         <v>97</v>
       </c>
       <c r="L26" s="7">
-        <f t="shared" si="3"/>
+        <f>SUM(F26,H26,I26)</f>
         <v>6280</v>
       </c>
       <c r="M26" s="23">
-        <f t="shared" si="4"/>
+        <f>SUM(J26,K26)</f>
         <v>1092</v>
       </c>
       <c r="N26" s="1">
@@ -2852,7 +2871,9 @@
         <v>500</v>
       </c>
       <c r="F30" s="4"/>
-      <c r="G30" s="4"/>
+      <c r="G30" s="29">
+        <v>0</v>
+      </c>
       <c r="H30" s="1">
         <v>500</v>
       </c>
@@ -3964,11 +3985,26 @@
         <v>482</v>
       </c>
       <c r="E44" s="11"/>
-      <c r="F44" s="4"/>
-      <c r="G44" s="4"/>
-      <c r="L44" s="7"/>
-      <c r="M44" s="23"/>
-      <c r="O44" s="7"/>
+      <c r="F44" s="11"/>
+      <c r="G44" s="1">
+        <f>AVERAGE(G$41:G$43)</f>
+        <v>0</v>
+      </c>
+      <c r="L44" s="7">
+        <v>0</v>
+      </c>
+      <c r="M44" s="7">
+        <f>AVERAGE(M$41:M$43)</f>
+        <v>197.33333333333334</v>
+      </c>
+      <c r="N44" s="7">
+        <f>AVERAGE(N$39:N$43)</f>
+        <v>266.2</v>
+      </c>
+      <c r="O44" s="7">
+        <f>AVERAGE(O$39:O$43)</f>
+        <v>4470.6000000000004</v>
+      </c>
       <c r="P44" s="5" t="s">
         <v>31</v>
       </c>
@@ -4018,11 +4054,25 @@
         <v>903</v>
       </c>
       <c r="E45" s="11"/>
-      <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
-      <c r="L45" s="7"/>
-      <c r="M45" s="23"/>
-      <c r="O45" s="7"/>
+      <c r="F45" s="11"/>
+      <c r="G45" s="11">
+        <v>0</v>
+      </c>
+      <c r="L45" s="1">
+        <v>0</v>
+      </c>
+      <c r="M45" s="7">
+        <f t="shared" ref="M45:M47" si="7">AVERAGE(M$41:M$43)</f>
+        <v>197.33333333333334</v>
+      </c>
+      <c r="N45" s="7">
+        <f t="shared" ref="N45:O47" si="8">AVERAGE(N$39:N$43)</f>
+        <v>266.2</v>
+      </c>
+      <c r="O45" s="7">
+        <f t="shared" si="8"/>
+        <v>4470.6000000000004</v>
+      </c>
       <c r="P45" s="5" t="s">
         <v>31</v>
       </c>
@@ -4072,11 +4122,25 @@
         <v>646</v>
       </c>
       <c r="E46" s="11"/>
-      <c r="F46" s="4"/>
-      <c r="G46" s="4"/>
-      <c r="L46" s="7"/>
-      <c r="M46" s="23"/>
-      <c r="O46" s="7"/>
+      <c r="F46" s="11"/>
+      <c r="G46" s="11">
+        <v>0</v>
+      </c>
+      <c r="L46" s="1">
+        <v>0</v>
+      </c>
+      <c r="M46" s="7">
+        <f t="shared" si="7"/>
+        <v>197.33333333333334</v>
+      </c>
+      <c r="N46" s="7">
+        <f t="shared" si="8"/>
+        <v>266.2</v>
+      </c>
+      <c r="O46" s="7">
+        <f t="shared" si="8"/>
+        <v>4470.6000000000004</v>
+      </c>
       <c r="P46" s="5" t="s">
         <v>31</v>
       </c>
@@ -4126,11 +4190,25 @@
         <v>482</v>
       </c>
       <c r="E47" s="11"/>
-      <c r="F47" s="4"/>
-      <c r="G47" s="4"/>
-      <c r="L47" s="7"/>
-      <c r="M47" s="23"/>
-      <c r="O47" s="7"/>
+      <c r="F47" s="11"/>
+      <c r="G47" s="11">
+        <v>0</v>
+      </c>
+      <c r="L47" s="1">
+        <v>0</v>
+      </c>
+      <c r="M47" s="7">
+        <f t="shared" si="7"/>
+        <v>197.33333333333334</v>
+      </c>
+      <c r="N47" s="7">
+        <f t="shared" si="8"/>
+        <v>266.2</v>
+      </c>
+      <c r="O47" s="7">
+        <f t="shared" si="8"/>
+        <v>4470.6000000000004</v>
+      </c>
       <c r="P47" s="5" t="s">
         <v>31</v>
       </c>
@@ -4330,10 +4408,16 @@
       <c r="BI59" s="7"/>
     </row>
     <row r="60" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="E60" s="1" t="s">
+        <v>32</v>
+      </c>
       <c r="BD60" s="7"/>
       <c r="BI60" s="7"/>
     </row>
     <row r="61" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="E61" s="1" t="s">
+        <v>33</v>
+      </c>
       <c r="BD61" s="7"/>
       <c r="BI61" s="7"/>
     </row>
@@ -4852,5 +4936,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddHeader>&amp;R&amp;"Calibri"&amp;12&amp;K000000 Unclassified - Non-Classifié&amp;1#_x000D_</oddHeader>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update runrecon code, add AFS FSC data for 2021-2025, add kitsumkalum brood fecundity data
</commit_message>
<xml_diff>
--- a/data-raw/freshwater-catch.xlsx
+++ b/data-raw/freshwater-catch.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\skrunchy2025\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4971EBDF-908C-4135-B749-853392DA798D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C58C3C5D-F306-402B-BF1C-1E712D45EF80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E0CDEE87-6CC2-4107-81B9-F1AD4EA649A7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E0CDEE87-6CC2-4107-81B9-F1AD4EA649A7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="34">
   <si>
     <t>Year</t>
   </si>
@@ -131,13 +131,13 @@
     <t>Winther et al. 2024</t>
   </si>
   <si>
-    <t xml:space="preserve">LW </t>
-  </si>
-  <si>
     <t>LW: 2021-2024 are all place-holders (except for Tyee catch which is correct)</t>
   </si>
   <si>
     <t>LW: Double check rec catch above Terrace for 2002, 2003, 2007</t>
+  </si>
+  <si>
+    <t>LW, FN catch above Terrace from AFS</t>
   </si>
 </sst>
 </file>
@@ -305,7 +305,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
@@ -319,6 +318,7 @@
     <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -672,7 +672,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:61" s="4" customFormat="1" ht="72" x14ac:dyDescent="0.2">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
@@ -681,7 +681,7 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="26" t="s">
+      <c r="D1" s="25" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
@@ -690,7 +690,7 @@
       <c r="F1" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="26" t="s">
+      <c r="G1" s="25" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="2" t="s">
@@ -705,16 +705,16 @@
       <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="27" t="s">
+      <c r="L1" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="M1" s="27" t="s">
+      <c r="M1" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="N1" s="26" t="s">
+      <c r="N1" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="O1" s="26" t="s">
+      <c r="O1" s="25" t="s">
         <v>12</v>
       </c>
       <c r="P1" s="2" t="s">
@@ -783,7 +783,7 @@
         <v>940</v>
       </c>
       <c r="G2" s="6">
-        <f t="shared" ref="G2:G24" si="2">E2-F2</f>
+        <f t="shared" ref="G2:G23" si="2">E2-F2</f>
         <v>470</v>
       </c>
       <c r="H2" s="7"/>
@@ -2495,7 +2495,7 @@
         <v>3962</v>
       </c>
       <c r="F25" s="4"/>
-      <c r="G25" s="29">
+      <c r="G25" s="28">
         <v>0</v>
       </c>
       <c r="H25" s="1">
@@ -2569,7 +2569,7 @@
         <v>6280</v>
       </c>
       <c r="F26" s="4"/>
-      <c r="G26" s="29">
+      <c r="G26" s="28">
         <v>0</v>
       </c>
       <c r="H26" s="1">
@@ -2871,7 +2871,7 @@
         <v>500</v>
       </c>
       <c r="F30" s="4"/>
-      <c r="G30" s="29">
+      <c r="G30" s="28">
         <v>0</v>
       </c>
       <c r="H30" s="1">
@@ -3971,7 +3971,7 @@
       <c r="BD43" s="7"/>
       <c r="BI43" s="7"/>
     </row>
-    <row r="44" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:61" ht="15" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>2021</v>
       </c>
@@ -3986,27 +3986,14 @@
       </c>
       <c r="E44" s="11"/>
       <c r="F44" s="11"/>
-      <c r="G44" s="1">
-        <f>AVERAGE(G$41:G$43)</f>
-        <v>0</v>
-      </c>
-      <c r="L44" s="7">
-        <v>0</v>
-      </c>
-      <c r="M44" s="7">
-        <f>AVERAGE(M$41:M$43)</f>
-        <v>197.33333333333334</v>
-      </c>
-      <c r="N44" s="7">
-        <f>AVERAGE(N$39:N$43)</f>
-        <v>266.2</v>
-      </c>
-      <c r="O44" s="7">
-        <f>AVERAGE(O$39:O$43)</f>
-        <v>4470.6000000000004</v>
+      <c r="L44" s="7"/>
+      <c r="M44" s="7"/>
+      <c r="N44" s="7"/>
+      <c r="O44" s="29">
+        <v>4192</v>
       </c>
       <c r="P44" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="Q44" s="5"/>
       <c r="R44" s="5"/>
@@ -4040,7 +4027,7 @@
       <c r="BD44" s="7"/>
       <c r="BI44" s="7"/>
     </row>
-    <row r="45" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:61" ht="15" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>2022</v>
       </c>
@@ -4055,26 +4042,14 @@
       </c>
       <c r="E45" s="11"/>
       <c r="F45" s="11"/>
-      <c r="G45" s="11">
-        <v>0</v>
-      </c>
-      <c r="L45" s="1">
-        <v>0</v>
-      </c>
-      <c r="M45" s="7">
-        <f t="shared" ref="M45:M47" si="7">AVERAGE(M$41:M$43)</f>
-        <v>197.33333333333334</v>
-      </c>
-      <c r="N45" s="7">
-        <f t="shared" ref="N45:O47" si="8">AVERAGE(N$39:N$43)</f>
-        <v>266.2</v>
-      </c>
-      <c r="O45" s="7">
-        <f t="shared" si="8"/>
-        <v>4470.6000000000004</v>
+      <c r="G45" s="11"/>
+      <c r="M45" s="7"/>
+      <c r="N45" s="7"/>
+      <c r="O45" s="29">
+        <v>2959</v>
       </c>
       <c r="P45" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="Q45" s="5"/>
       <c r="R45" s="5"/>
@@ -4108,7 +4083,7 @@
       <c r="BD45" s="7"/>
       <c r="BI45" s="7"/>
     </row>
-    <row r="46" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:61" ht="15" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>2023</v>
       </c>
@@ -4123,26 +4098,14 @@
       </c>
       <c r="E46" s="11"/>
       <c r="F46" s="11"/>
-      <c r="G46" s="11">
-        <v>0</v>
-      </c>
-      <c r="L46" s="1">
-        <v>0</v>
-      </c>
-      <c r="M46" s="7">
-        <f t="shared" si="7"/>
-        <v>197.33333333333334</v>
-      </c>
-      <c r="N46" s="7">
-        <f t="shared" si="8"/>
-        <v>266.2</v>
-      </c>
-      <c r="O46" s="7">
-        <f t="shared" si="8"/>
-        <v>4470.6000000000004</v>
+      <c r="G46" s="11"/>
+      <c r="M46" s="7"/>
+      <c r="N46" s="7"/>
+      <c r="O46" s="29">
+        <v>3369</v>
       </c>
       <c r="P46" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="Q46" s="5"/>
       <c r="R46" s="5"/>
@@ -4176,7 +4139,7 @@
       <c r="BD46" s="7"/>
       <c r="BI46" s="7"/>
     </row>
-    <row r="47" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:61" ht="15" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>2024</v>
       </c>
@@ -4191,26 +4154,14 @@
       </c>
       <c r="E47" s="11"/>
       <c r="F47" s="11"/>
-      <c r="G47" s="11">
-        <v>0</v>
-      </c>
-      <c r="L47" s="1">
-        <v>0</v>
-      </c>
-      <c r="M47" s="7">
-        <f t="shared" si="7"/>
-        <v>197.33333333333334</v>
-      </c>
-      <c r="N47" s="7">
-        <f t="shared" si="8"/>
-        <v>266.2</v>
-      </c>
-      <c r="O47" s="7">
-        <f t="shared" si="8"/>
-        <v>4470.6000000000004</v>
+      <c r="G47" s="11"/>
+      <c r="M47" s="7"/>
+      <c r="N47" s="7"/>
+      <c r="O47" s="29">
+        <v>1860</v>
       </c>
       <c r="P47" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="Q47" s="5"/>
       <c r="R47" s="5"/>
@@ -4244,11 +4195,20 @@
       <c r="BD47" s="7"/>
       <c r="BI47" s="7"/>
     </row>
-    <row r="48" spans="1:61" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:61" ht="15" x14ac:dyDescent="0.25">
+      <c r="A48" s="1">
+        <v>2025</v>
+      </c>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
-      <c r="L48" s="5"/>
-      <c r="M48" s="24"/>
+      <c r="M48" s="7"/>
+      <c r="N48" s="7"/>
+      <c r="O48">
+        <v>3270</v>
+      </c>
+      <c r="P48" s="5" t="s">
+        <v>33</v>
+      </c>
       <c r="R48" s="5"/>
       <c r="S48" s="5"/>
       <c r="T48" s="5"/>
@@ -4278,7 +4238,7 @@
       <c r="A49" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D49" s="28" t="s">
+      <c r="D49" s="27" t="s">
         <v>14</v>
       </c>
       <c r="E49" s="15" t="s">
@@ -4322,9 +4282,9 @@
       <c r="BI50" s="7"/>
     </row>
     <row r="51" spans="1:61" x14ac:dyDescent="0.2">
-      <c r="B51" s="28"/>
-      <c r="C51" s="28"/>
-      <c r="D51" s="28"/>
+      <c r="B51" s="27"/>
+      <c r="C51" s="27"/>
+      <c r="D51" s="27"/>
       <c r="E51" s="10" t="s">
         <v>15</v>
       </c>
@@ -4409,14 +4369,14 @@
     </row>
     <row r="60" spans="1:61" x14ac:dyDescent="0.2">
       <c r="E60" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="BD60" s="7"/>
       <c r="BI60" s="7"/>
     </row>
     <row r="61" spans="1:61" x14ac:dyDescent="0.2">
       <c r="E61" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="BD61" s="7"/>
       <c r="BI61" s="7"/>

</xml_diff>

<commit_message>
Update rr with 2021-2014 fsc nunmbers
</commit_message>
<xml_diff>
--- a/data-raw/freshwater-catch.xlsx
+++ b/data-raw/freshwater-catch.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\skrunchy2025\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C58C3C5D-F306-402B-BF1C-1E712D45EF80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CBA8993-F005-402B-B6D4-14E5E4098EF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E0CDEE87-6CC2-4107-81B9-F1AD4EA649A7}"/>
   </bookViews>
@@ -3986,9 +3986,18 @@
       </c>
       <c r="E44" s="11"/>
       <c r="F44" s="11"/>
-      <c r="L44" s="7"/>
-      <c r="M44" s="7"/>
-      <c r="N44" s="7"/>
+      <c r="G44" s="1">
+        <v>0</v>
+      </c>
+      <c r="L44" s="7">
+        <v>0</v>
+      </c>
+      <c r="M44" s="7">
+        <v>0</v>
+      </c>
+      <c r="N44" s="7">
+        <v>0</v>
+      </c>
       <c r="O44" s="29">
         <v>4192</v>
       </c>
@@ -4042,9 +4051,18 @@
       </c>
       <c r="E45" s="11"/>
       <c r="F45" s="11"/>
-      <c r="G45" s="11"/>
-      <c r="M45" s="7"/>
-      <c r="N45" s="7"/>
+      <c r="G45" s="11">
+        <v>0</v>
+      </c>
+      <c r="L45" s="1">
+        <v>0</v>
+      </c>
+      <c r="M45" s="7">
+        <v>0</v>
+      </c>
+      <c r="N45" s="7">
+        <v>0</v>
+      </c>
       <c r="O45" s="29">
         <v>2959</v>
       </c>
@@ -4098,9 +4116,18 @@
       </c>
       <c r="E46" s="11"/>
       <c r="F46" s="11"/>
-      <c r="G46" s="11"/>
-      <c r="M46" s="7"/>
-      <c r="N46" s="7"/>
+      <c r="G46" s="11">
+        <v>0</v>
+      </c>
+      <c r="L46" s="1">
+        <v>0</v>
+      </c>
+      <c r="M46" s="7">
+        <v>0</v>
+      </c>
+      <c r="N46" s="7">
+        <v>0</v>
+      </c>
       <c r="O46" s="29">
         <v>3369</v>
       </c>
@@ -4154,9 +4181,18 @@
       </c>
       <c r="E47" s="11"/>
       <c r="F47" s="11"/>
-      <c r="G47" s="11"/>
-      <c r="M47" s="7"/>
-      <c r="N47" s="7"/>
+      <c r="G47" s="11">
+        <v>0</v>
+      </c>
+      <c r="L47" s="1">
+        <v>0</v>
+      </c>
+      <c r="M47" s="7">
+        <v>0</v>
+      </c>
+      <c r="N47" s="7">
+        <v>0</v>
+      </c>
       <c r="O47" s="29">
         <v>1860</v>
       </c>

</xml_diff>

<commit_message>
Update freshwater catch raw data file, with creel survey results from 2021-2025, plus some notes
</commit_message>
<xml_diff>
--- a/data-raw/freshwater-catch.xlsx
+++ b/data-raw/freshwater-catch.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\skrunchy2025\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CBA8993-F005-402B-B6D4-14E5E4098EF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE37A6E9-11DD-42FC-A3FF-3D8249269507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E0CDEE87-6CC2-4107-81B9-F1AD4EA649A7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="48">
   <si>
     <t>Year</t>
   </si>
@@ -138,6 +138,48 @@
   </si>
   <si>
     <t>LW, FN catch above Terrace from AFS</t>
+  </si>
+  <si>
+    <t>Creel survey?</t>
+  </si>
+  <si>
+    <t>FN catch below Terrace of 1000 is placeholder</t>
+  </si>
+  <si>
+    <t>Below Terrace, LGL and Kitsumkalum</t>
+  </si>
+  <si>
+    <t>Estimated sport above Terrace = 20% of below Terrace</t>
+  </si>
+  <si>
+    <t>Data notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Robichaud et al. 2020, Tables 13, 15 </t>
+  </si>
+  <si>
+    <t>Robichaud et al. 2018, Tables 15, 17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Robichaud et al. 2021, Tables 13, 15 </t>
+  </si>
+  <si>
+    <t>Robichaud et al. 2022, Tables 13, 15</t>
+  </si>
+  <si>
+    <t>Robichaud et al. 2024, Tables 12, 14</t>
+  </si>
+  <si>
+    <t>Robichaud et al. 2023, Tables 12, 14</t>
+  </si>
+  <si>
+    <t>Robichaud et al. 2025, Tables 13, 15</t>
+  </si>
+  <si>
+    <t>Robichaud et al. 2026, Tables 13. 15</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> FW Sport source details</t>
   </si>
 </sst>
 </file>
@@ -260,7 +302,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -319,6 +361,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="2" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -637,7 +680,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35E3952C-60AA-4AE7-A274-2D9A331D3C7B}">
-  <dimension ref="A1:BI190"/>
+  <dimension ref="A1:BJ190"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.85546875" style="1" customWidth="1"/>
@@ -646,32 +689,35 @@
     <col min="5" max="12" width="8.7109375" style="1"/>
     <col min="13" max="13" width="8.42578125" style="19" customWidth="1"/>
     <col min="14" max="15" width="7.5703125" style="1" customWidth="1"/>
-    <col min="16" max="16" width="20.28515625" style="1" customWidth="1"/>
-    <col min="17" max="22" width="7.5703125" style="1" customWidth="1"/>
-    <col min="23" max="24" width="8.85546875" style="1" customWidth="1"/>
-    <col min="25" max="28" width="7.5703125" style="1" customWidth="1"/>
-    <col min="29" max="29" width="8.140625" style="1" customWidth="1"/>
-    <col min="30" max="43" width="8.7109375" style="1"/>
-    <col min="44" max="44" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="8.7109375" style="1"/>
-    <col min="46" max="46" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="8.7109375" style="1"/>
-    <col min="48" max="48" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="8.7109375" style="1"/>
-    <col min="50" max="50" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="8.7109375" style="1"/>
-    <col min="52" max="53" width="4.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="7.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="56" max="57" width="8.7109375" style="1"/>
-    <col min="58" max="58" width="4.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="3.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="7" style="1" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="7.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="62" max="16384" width="8.7109375" style="1"/>
+    <col min="16" max="16" width="34.42578125" style="1" customWidth="1"/>
+    <col min="17" max="17" width="33.42578125" style="1" customWidth="1"/>
+    <col min="18" max="18" width="32.5703125" style="1" customWidth="1"/>
+    <col min="19" max="19" width="24.140625" style="1" customWidth="1"/>
+    <col min="20" max="23" width="7.5703125" style="1" customWidth="1"/>
+    <col min="24" max="25" width="8.85546875" style="1" customWidth="1"/>
+    <col min="26" max="29" width="7.5703125" style="1" customWidth="1"/>
+    <col min="30" max="30" width="8.140625" style="1" customWidth="1"/>
+    <col min="31" max="44" width="8.7109375" style="1"/>
+    <col min="45" max="45" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="8.7109375" style="1"/>
+    <col min="47" max="47" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="8.7109375" style="1"/>
+    <col min="49" max="49" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="8.7109375" style="1"/>
+    <col min="51" max="51" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="8.7109375" style="1"/>
+    <col min="53" max="54" width="4.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="7.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="57" max="58" width="8.7109375" style="1"/>
+    <col min="59" max="59" width="4.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="3.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="7" style="1" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="7.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="63" max="16384" width="8.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:61" s="4" customFormat="1" ht="72" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:62" s="4" customFormat="1" ht="72" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
@@ -720,15 +766,21 @@
       <c r="P1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="Q1" s="18"/>
-      <c r="R1" s="18"/>
-      <c r="S1" s="18"/>
-      <c r="T1" s="20"/>
-      <c r="U1" s="18"/>
-      <c r="V1" s="20"/>
-      <c r="W1" s="18"/>
-      <c r="X1" s="20"/>
-      <c r="Y1" s="18"/>
+      <c r="Q1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="R1" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="S1" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="T1" s="18"/>
+      <c r="U1" s="20"/>
+      <c r="V1" s="18"/>
+      <c r="W1" s="20"/>
+      <c r="X1" s="18"/>
+      <c r="Y1" s="20"/>
       <c r="Z1" s="18"/>
       <c r="AA1" s="18"/>
       <c r="AB1" s="18"/>
@@ -747,7 +799,7 @@
       <c r="AO1" s="18"/>
       <c r="AP1" s="18"/>
       <c r="AQ1" s="18"/>
-      <c r="AR1" s="21"/>
+      <c r="AR1" s="18"/>
       <c r="AS1" s="21"/>
       <c r="AT1" s="21"/>
       <c r="AU1" s="21"/>
@@ -756,12 +808,13 @@
       <c r="AX1" s="21"/>
       <c r="AY1" s="21"/>
       <c r="AZ1" s="21"/>
-      <c r="BA1" s="19"/>
+      <c r="BA1" s="21"/>
       <c r="BB1" s="19"/>
       <c r="BC1" s="19"/>
-      <c r="BD1" s="1"/>
-    </row>
-    <row r="2" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="BD1" s="19"/>
+      <c r="BE1" s="1"/>
+    </row>
+    <row r="2" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>1979</v>
       </c>
@@ -815,31 +868,32 @@
       <c r="V2" s="7"/>
       <c r="W2" s="7"/>
       <c r="X2" s="7"/>
-      <c r="Y2" s="8"/>
+      <c r="Y2" s="7"/>
       <c r="Z2" s="8"/>
       <c r="AA2" s="8"/>
       <c r="AB2" s="8"/>
       <c r="AC2" s="8"/>
-      <c r="AD2" s="7"/>
+      <c r="AD2" s="8"/>
       <c r="AE2" s="7"/>
       <c r="AF2" s="7"/>
       <c r="AG2" s="7"/>
       <c r="AH2" s="7"/>
       <c r="AI2" s="7"/>
-      <c r="AJ2" s="9"/>
-      <c r="AL2" s="7"/>
+      <c r="AJ2" s="7"/>
+      <c r="AK2" s="9"/>
       <c r="AM2" s="7"/>
       <c r="AN2" s="7"/>
       <c r="AO2" s="7"/>
       <c r="AP2" s="7"/>
       <c r="AQ2" s="7"/>
-      <c r="AS2" s="7"/>
-      <c r="AU2" s="7"/>
-      <c r="AW2" s="7"/>
-      <c r="AY2" s="7"/>
-      <c r="BD2" s="7"/>
-    </row>
-    <row r="3" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR2" s="7"/>
+      <c r="AT2" s="7"/>
+      <c r="AV2" s="7"/>
+      <c r="AX2" s="7"/>
+      <c r="AZ2" s="7"/>
+      <c r="BE2" s="7"/>
+    </row>
+    <row r="3" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>1980</v>
       </c>
@@ -869,7 +923,7 @@
         <v>2417</v>
       </c>
       <c r="M3" s="23">
-        <f t="shared" ref="M3:M43" si="4">SUM(J3,K3)</f>
+        <f t="shared" ref="M3:M47" si="4">SUM(J3,K3)</f>
         <v>0</v>
       </c>
       <c r="N3" s="1">
@@ -881,39 +935,40 @@
       <c r="P3" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q3" s="5"/>
+      <c r="Q3" s="7"/>
       <c r="R3" s="5"/>
       <c r="S3" s="5"/>
-      <c r="T3" s="7"/>
+      <c r="T3" s="5"/>
       <c r="U3" s="7"/>
       <c r="V3" s="7"/>
       <c r="W3" s="7"/>
       <c r="X3" s="7"/>
-      <c r="Y3" s="8"/>
+      <c r="Y3" s="7"/>
       <c r="Z3" s="8"/>
       <c r="AA3" s="8"/>
       <c r="AB3" s="8"/>
       <c r="AC3" s="8"/>
-      <c r="AD3" s="7"/>
+      <c r="AD3" s="8"/>
       <c r="AE3" s="7"/>
       <c r="AF3" s="7"/>
       <c r="AG3" s="7"/>
       <c r="AH3" s="7"/>
       <c r="AI3" s="7"/>
-      <c r="AJ3" s="9"/>
-      <c r="AL3" s="7"/>
+      <c r="AJ3" s="7"/>
+      <c r="AK3" s="9"/>
       <c r="AM3" s="7"/>
       <c r="AN3" s="7"/>
       <c r="AO3" s="7"/>
       <c r="AP3" s="7"/>
       <c r="AQ3" s="7"/>
-      <c r="AS3" s="7"/>
-      <c r="AU3" s="7"/>
-      <c r="AW3" s="7"/>
-      <c r="AY3" s="7"/>
-      <c r="BD3" s="7"/>
-    </row>
-    <row r="4" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR3" s="7"/>
+      <c r="AT3" s="7"/>
+      <c r="AV3" s="7"/>
+      <c r="AX3" s="7"/>
+      <c r="AZ3" s="7"/>
+      <c r="BE3" s="7"/>
+    </row>
+    <row r="4" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>1981</v>
       </c>
@@ -955,39 +1010,40 @@
       <c r="P4" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q4" s="5"/>
+      <c r="Q4" s="7"/>
       <c r="R4" s="5"/>
       <c r="S4" s="5"/>
-      <c r="T4" s="7"/>
+      <c r="T4" s="5"/>
       <c r="U4" s="7"/>
       <c r="V4" s="7"/>
       <c r="W4" s="7"/>
       <c r="X4" s="7"/>
-      <c r="Y4" s="8"/>
+      <c r="Y4" s="7"/>
       <c r="Z4" s="8"/>
       <c r="AA4" s="8"/>
       <c r="AB4" s="8"/>
       <c r="AC4" s="8"/>
-      <c r="AD4" s="7"/>
+      <c r="AD4" s="8"/>
       <c r="AE4" s="7"/>
       <c r="AF4" s="7"/>
       <c r="AG4" s="7"/>
       <c r="AH4" s="7"/>
       <c r="AI4" s="7"/>
-      <c r="AJ4" s="9"/>
-      <c r="AL4" s="7"/>
+      <c r="AJ4" s="7"/>
+      <c r="AK4" s="9"/>
       <c r="AM4" s="7"/>
       <c r="AN4" s="7"/>
       <c r="AO4" s="7"/>
       <c r="AP4" s="7"/>
       <c r="AQ4" s="7"/>
-      <c r="AS4" s="7"/>
-      <c r="AU4" s="7"/>
-      <c r="AW4" s="7"/>
-      <c r="AY4" s="7"/>
-      <c r="BD4" s="7"/>
-    </row>
-    <row r="5" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR4" s="7"/>
+      <c r="AT4" s="7"/>
+      <c r="AV4" s="7"/>
+      <c r="AX4" s="7"/>
+      <c r="AZ4" s="7"/>
+      <c r="BE4" s="7"/>
+    </row>
+    <row r="5" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>1982</v>
       </c>
@@ -1029,39 +1085,40 @@
       <c r="P5" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q5" s="5"/>
+      <c r="Q5" s="7"/>
       <c r="R5" s="5"/>
       <c r="S5" s="5"/>
-      <c r="T5" s="7"/>
+      <c r="T5" s="5"/>
       <c r="U5" s="7"/>
       <c r="V5" s="7"/>
       <c r="W5" s="7"/>
       <c r="X5" s="7"/>
-      <c r="Y5" s="8"/>
+      <c r="Y5" s="7"/>
       <c r="Z5" s="8"/>
       <c r="AA5" s="8"/>
       <c r="AB5" s="8"/>
       <c r="AC5" s="8"/>
-      <c r="AD5" s="7"/>
+      <c r="AD5" s="8"/>
       <c r="AE5" s="7"/>
       <c r="AF5" s="7"/>
       <c r="AG5" s="7"/>
       <c r="AH5" s="7"/>
       <c r="AI5" s="7"/>
-      <c r="AJ5" s="9"/>
-      <c r="AL5" s="7"/>
+      <c r="AJ5" s="7"/>
+      <c r="AK5" s="9"/>
       <c r="AM5" s="7"/>
       <c r="AN5" s="7"/>
       <c r="AO5" s="7"/>
       <c r="AP5" s="7"/>
       <c r="AQ5" s="7"/>
-      <c r="AS5" s="7"/>
-      <c r="AU5" s="7"/>
-      <c r="AW5" s="7"/>
-      <c r="AY5" s="7"/>
-      <c r="BD5" s="7"/>
-    </row>
-    <row r="6" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR5" s="7"/>
+      <c r="AT5" s="7"/>
+      <c r="AV5" s="7"/>
+      <c r="AX5" s="7"/>
+      <c r="AZ5" s="7"/>
+      <c r="BE5" s="7"/>
+    </row>
+    <row r="6" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>1983</v>
       </c>
@@ -1079,7 +1136,7 @@
         <v>4366</v>
       </c>
       <c r="F6" s="6">
-        <f t="shared" si="1"/>
+        <f>ROUND((E6*2/3),0)</f>
         <v>2911</v>
       </c>
       <c r="G6" s="6">
@@ -1103,40 +1160,41 @@
       <c r="P6" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q6" s="5"/>
+      <c r="Q6" s="7"/>
       <c r="R6" s="5"/>
       <c r="S6" s="5"/>
-      <c r="T6" s="7"/>
+      <c r="T6" s="5"/>
       <c r="U6" s="7"/>
       <c r="V6" s="7"/>
       <c r="W6" s="7"/>
       <c r="X6" s="7"/>
-      <c r="Y6" s="8"/>
+      <c r="Y6" s="7"/>
       <c r="Z6" s="8"/>
       <c r="AA6" s="8"/>
       <c r="AB6" s="8"/>
       <c r="AC6" s="8"/>
-      <c r="AD6" s="7"/>
+      <c r="AD6" s="8"/>
       <c r="AE6" s="7"/>
       <c r="AF6" s="7"/>
       <c r="AG6" s="7"/>
       <c r="AH6" s="7"/>
       <c r="AI6" s="7"/>
-      <c r="AJ6" s="9"/>
-      <c r="AL6" s="7"/>
+      <c r="AJ6" s="7"/>
+      <c r="AK6" s="9"/>
       <c r="AM6" s="7"/>
       <c r="AN6" s="7"/>
       <c r="AO6" s="7"/>
       <c r="AP6" s="7"/>
       <c r="AQ6" s="7"/>
-      <c r="AS6" s="7"/>
-      <c r="AU6" s="7"/>
-      <c r="AW6" s="7"/>
-      <c r="AY6" s="7"/>
-      <c r="BD6" s="7"/>
-      <c r="BI6" s="7"/>
-    </row>
-    <row r="7" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR6" s="7"/>
+      <c r="AT6" s="7"/>
+      <c r="AV6" s="7"/>
+      <c r="AX6" s="7"/>
+      <c r="AZ6" s="7"/>
+      <c r="BE6" s="7"/>
+      <c r="BJ6" s="7"/>
+    </row>
+    <row r="7" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>1984</v>
       </c>
@@ -1162,7 +1220,7 @@
         <v>992</v>
       </c>
       <c r="L7" s="7">
-        <f t="shared" si="3"/>
+        <f>SUM(F7,H7,I7)</f>
         <v>1984</v>
       </c>
       <c r="M7" s="23">
@@ -1178,40 +1236,41 @@
       <c r="P7" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q7" s="5"/>
+      <c r="Q7" s="7"/>
       <c r="R7" s="5"/>
       <c r="S7" s="5"/>
-      <c r="T7" s="7"/>
+      <c r="T7" s="5"/>
       <c r="U7" s="7"/>
       <c r="V7" s="7"/>
       <c r="W7" s="7"/>
       <c r="X7" s="7"/>
-      <c r="Y7" s="8"/>
+      <c r="Y7" s="7"/>
       <c r="Z7" s="8"/>
       <c r="AA7" s="8"/>
       <c r="AB7" s="8"/>
       <c r="AC7" s="8"/>
-      <c r="AD7" s="7"/>
+      <c r="AD7" s="8"/>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
       <c r="AG7" s="7"/>
       <c r="AH7" s="7"/>
       <c r="AI7" s="7"/>
-      <c r="AJ7" s="9"/>
-      <c r="AL7" s="7"/>
+      <c r="AJ7" s="7"/>
+      <c r="AK7" s="9"/>
       <c r="AM7" s="7"/>
       <c r="AN7" s="7"/>
       <c r="AO7" s="7"/>
       <c r="AP7" s="7"/>
       <c r="AQ7" s="7"/>
-      <c r="AS7" s="7"/>
-      <c r="AU7" s="7"/>
-      <c r="AW7" s="7"/>
-      <c r="AY7" s="7"/>
-      <c r="BD7" s="7"/>
-      <c r="BI7" s="7"/>
-    </row>
-    <row r="8" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR7" s="7"/>
+      <c r="AT7" s="7"/>
+      <c r="AV7" s="7"/>
+      <c r="AX7" s="7"/>
+      <c r="AZ7" s="7"/>
+      <c r="BE7" s="7"/>
+      <c r="BJ7" s="7"/>
+    </row>
+    <row r="8" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>1985</v>
       </c>
@@ -1253,40 +1312,41 @@
       <c r="P8" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q8" s="5"/>
+      <c r="Q8" s="7"/>
       <c r="R8" s="5"/>
       <c r="S8" s="5"/>
-      <c r="T8" s="7"/>
+      <c r="T8" s="5"/>
       <c r="U8" s="7"/>
       <c r="V8" s="7"/>
       <c r="W8" s="7"/>
       <c r="X8" s="7"/>
-      <c r="Y8" s="8"/>
+      <c r="Y8" s="7"/>
       <c r="Z8" s="8"/>
       <c r="AA8" s="8"/>
       <c r="AB8" s="8"/>
       <c r="AC8" s="8"/>
-      <c r="AD8" s="7"/>
+      <c r="AD8" s="8"/>
       <c r="AE8" s="7"/>
       <c r="AF8" s="7"/>
       <c r="AG8" s="7"/>
       <c r="AH8" s="7"/>
       <c r="AI8" s="7"/>
-      <c r="AJ8" s="9"/>
-      <c r="AL8" s="7"/>
+      <c r="AJ8" s="7"/>
+      <c r="AK8" s="9"/>
       <c r="AM8" s="7"/>
       <c r="AN8" s="7"/>
       <c r="AO8" s="7"/>
       <c r="AP8" s="7"/>
       <c r="AQ8" s="7"/>
-      <c r="AS8" s="7"/>
-      <c r="AU8" s="7"/>
-      <c r="AW8" s="7"/>
-      <c r="AY8" s="7"/>
-      <c r="BD8" s="7"/>
-      <c r="BI8" s="7"/>
-    </row>
-    <row r="9" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR8" s="7"/>
+      <c r="AT8" s="7"/>
+      <c r="AV8" s="7"/>
+      <c r="AX8" s="7"/>
+      <c r="AZ8" s="7"/>
+      <c r="BE8" s="7"/>
+      <c r="BJ8" s="7"/>
+    </row>
+    <row r="9" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>1986</v>
       </c>
@@ -1328,40 +1388,41 @@
       <c r="P9" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q9" s="5"/>
+      <c r="Q9" s="7"/>
       <c r="R9" s="5"/>
       <c r="S9" s="5"/>
-      <c r="T9" s="7"/>
+      <c r="T9" s="5"/>
       <c r="U9" s="7"/>
       <c r="V9" s="7"/>
       <c r="W9" s="7"/>
       <c r="X9" s="7"/>
-      <c r="Y9" s="8"/>
+      <c r="Y9" s="7"/>
       <c r="Z9" s="8"/>
       <c r="AA9" s="8"/>
       <c r="AB9" s="8"/>
       <c r="AC9" s="8"/>
-      <c r="AD9" s="7"/>
+      <c r="AD9" s="8"/>
       <c r="AE9" s="7"/>
       <c r="AF9" s="7"/>
       <c r="AG9" s="7"/>
       <c r="AH9" s="7"/>
       <c r="AI9" s="7"/>
-      <c r="AJ9" s="9"/>
-      <c r="AL9" s="7"/>
+      <c r="AJ9" s="7"/>
+      <c r="AK9" s="9"/>
       <c r="AM9" s="7"/>
       <c r="AN9" s="7"/>
       <c r="AO9" s="7"/>
       <c r="AP9" s="7"/>
       <c r="AQ9" s="7"/>
-      <c r="AS9" s="7"/>
-      <c r="AU9" s="7"/>
-      <c r="AW9" s="7"/>
-      <c r="AY9" s="7"/>
-      <c r="BD9" s="7"/>
-      <c r="BI9" s="7"/>
-    </row>
-    <row r="10" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR9" s="7"/>
+      <c r="AT9" s="7"/>
+      <c r="AV9" s="7"/>
+      <c r="AX9" s="7"/>
+      <c r="AZ9" s="7"/>
+      <c r="BE9" s="7"/>
+      <c r="BJ9" s="7"/>
+    </row>
+    <row r="10" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>1987</v>
       </c>
@@ -1403,40 +1464,41 @@
       <c r="P10" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q10" s="5"/>
+      <c r="Q10" s="7"/>
       <c r="R10" s="5"/>
       <c r="S10" s="5"/>
-      <c r="T10" s="7"/>
+      <c r="T10" s="5"/>
       <c r="U10" s="7"/>
       <c r="V10" s="7"/>
       <c r="W10" s="7"/>
       <c r="X10" s="7"/>
-      <c r="Y10" s="8"/>
+      <c r="Y10" s="7"/>
       <c r="Z10" s="8"/>
       <c r="AA10" s="8"/>
       <c r="AB10" s="8"/>
       <c r="AC10" s="8"/>
-      <c r="AD10" s="7"/>
+      <c r="AD10" s="8"/>
       <c r="AE10" s="7"/>
       <c r="AF10" s="7"/>
       <c r="AG10" s="7"/>
       <c r="AH10" s="7"/>
       <c r="AI10" s="7"/>
-      <c r="AJ10" s="9"/>
-      <c r="AL10" s="7"/>
+      <c r="AJ10" s="7"/>
+      <c r="AK10" s="9"/>
       <c r="AM10" s="7"/>
       <c r="AN10" s="7"/>
       <c r="AO10" s="7"/>
       <c r="AP10" s="7"/>
       <c r="AQ10" s="7"/>
-      <c r="AS10" s="7"/>
-      <c r="AU10" s="7"/>
-      <c r="AW10" s="7"/>
-      <c r="AY10" s="7"/>
-      <c r="BD10" s="7"/>
-      <c r="BI10" s="7"/>
-    </row>
-    <row r="11" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR10" s="7"/>
+      <c r="AT10" s="7"/>
+      <c r="AV10" s="7"/>
+      <c r="AX10" s="7"/>
+      <c r="AZ10" s="7"/>
+      <c r="BE10" s="7"/>
+      <c r="BJ10" s="7"/>
+    </row>
+    <row r="11" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>1988</v>
       </c>
@@ -1478,40 +1540,41 @@
       <c r="P11" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q11" s="5"/>
+      <c r="Q11" s="7"/>
       <c r="R11" s="5"/>
       <c r="S11" s="5"/>
-      <c r="T11" s="7"/>
+      <c r="T11" s="5"/>
       <c r="U11" s="7"/>
       <c r="V11" s="7"/>
       <c r="W11" s="7"/>
       <c r="X11" s="7"/>
-      <c r="Y11" s="8"/>
+      <c r="Y11" s="7"/>
       <c r="Z11" s="8"/>
       <c r="AA11" s="8"/>
       <c r="AB11" s="8"/>
       <c r="AC11" s="8"/>
-      <c r="AD11" s="7"/>
+      <c r="AD11" s="8"/>
       <c r="AE11" s="7"/>
       <c r="AF11" s="7"/>
       <c r="AG11" s="7"/>
       <c r="AH11" s="7"/>
       <c r="AI11" s="7"/>
-      <c r="AJ11" s="9"/>
-      <c r="AL11" s="7"/>
+      <c r="AJ11" s="7"/>
+      <c r="AK11" s="9"/>
       <c r="AM11" s="7"/>
       <c r="AN11" s="7"/>
       <c r="AO11" s="7"/>
       <c r="AP11" s="7"/>
       <c r="AQ11" s="7"/>
-      <c r="AS11" s="7"/>
-      <c r="AU11" s="7"/>
-      <c r="AW11" s="7"/>
-      <c r="AY11" s="7"/>
-      <c r="BD11" s="7"/>
-      <c r="BI11" s="7"/>
-    </row>
-    <row r="12" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR11" s="7"/>
+      <c r="AT11" s="7"/>
+      <c r="AV11" s="7"/>
+      <c r="AX11" s="7"/>
+      <c r="AZ11" s="7"/>
+      <c r="BE11" s="7"/>
+      <c r="BJ11" s="7"/>
+    </row>
+    <row r="12" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>1989</v>
       </c>
@@ -1553,40 +1616,41 @@
       <c r="P12" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q12" s="5"/>
+      <c r="Q12" s="7"/>
       <c r="R12" s="5"/>
       <c r="S12" s="5"/>
-      <c r="T12" s="7"/>
+      <c r="T12" s="5"/>
       <c r="U12" s="7"/>
       <c r="V12" s="7"/>
       <c r="W12" s="7"/>
       <c r="X12" s="7"/>
-      <c r="Y12" s="8"/>
+      <c r="Y12" s="7"/>
       <c r="Z12" s="8"/>
       <c r="AA12" s="8"/>
       <c r="AB12" s="8"/>
       <c r="AC12" s="8"/>
-      <c r="AD12" s="7"/>
+      <c r="AD12" s="8"/>
       <c r="AE12" s="7"/>
       <c r="AF12" s="7"/>
       <c r="AG12" s="7"/>
       <c r="AH12" s="7"/>
       <c r="AI12" s="7"/>
-      <c r="AJ12" s="9"/>
-      <c r="AL12" s="7"/>
+      <c r="AJ12" s="7"/>
+      <c r="AK12" s="9"/>
       <c r="AM12" s="7"/>
       <c r="AN12" s="7"/>
       <c r="AO12" s="7"/>
       <c r="AP12" s="7"/>
       <c r="AQ12" s="7"/>
-      <c r="AS12" s="7"/>
-      <c r="AU12" s="7"/>
-      <c r="AW12" s="7"/>
-      <c r="AY12" s="7"/>
-      <c r="BD12" s="7"/>
-      <c r="BI12" s="7"/>
-    </row>
-    <row r="13" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR12" s="7"/>
+      <c r="AT12" s="7"/>
+      <c r="AV12" s="7"/>
+      <c r="AX12" s="7"/>
+      <c r="AZ12" s="7"/>
+      <c r="BE12" s="7"/>
+      <c r="BJ12" s="7"/>
+    </row>
+    <row r="13" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>1990</v>
       </c>
@@ -1628,40 +1692,41 @@
       <c r="P13" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q13" s="5"/>
+      <c r="Q13" s="7"/>
       <c r="R13" s="5"/>
       <c r="S13" s="5"/>
-      <c r="T13" s="7"/>
+      <c r="T13" s="5"/>
       <c r="U13" s="7"/>
       <c r="V13" s="7"/>
       <c r="W13" s="7"/>
       <c r="X13" s="7"/>
-      <c r="Y13" s="8"/>
+      <c r="Y13" s="7"/>
       <c r="Z13" s="8"/>
       <c r="AA13" s="8"/>
       <c r="AB13" s="8"/>
       <c r="AC13" s="8"/>
-      <c r="AD13" s="7"/>
+      <c r="AD13" s="8"/>
       <c r="AE13" s="7"/>
       <c r="AF13" s="7"/>
       <c r="AG13" s="7"/>
       <c r="AH13" s="7"/>
       <c r="AI13" s="7"/>
-      <c r="AJ13" s="9"/>
-      <c r="AL13" s="7"/>
+      <c r="AJ13" s="7"/>
+      <c r="AK13" s="9"/>
       <c r="AM13" s="7"/>
       <c r="AN13" s="7"/>
       <c r="AO13" s="7"/>
       <c r="AP13" s="7"/>
       <c r="AQ13" s="7"/>
-      <c r="AS13" s="7"/>
-      <c r="AU13" s="7"/>
-      <c r="AW13" s="7"/>
-      <c r="AY13" s="7"/>
-      <c r="BD13" s="7"/>
-      <c r="BI13" s="7"/>
-    </row>
-    <row r="14" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR13" s="7"/>
+      <c r="AT13" s="7"/>
+      <c r="AV13" s="7"/>
+      <c r="AX13" s="7"/>
+      <c r="AZ13" s="7"/>
+      <c r="BE13" s="7"/>
+      <c r="BJ13" s="7"/>
+    </row>
+    <row r="14" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>1991</v>
       </c>
@@ -1703,40 +1768,41 @@
       <c r="P14" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q14" s="5"/>
+      <c r="Q14" s="7"/>
       <c r="R14" s="5"/>
       <c r="S14" s="5"/>
-      <c r="T14" s="7"/>
+      <c r="T14" s="5"/>
       <c r="U14" s="7"/>
       <c r="V14" s="7"/>
       <c r="W14" s="7"/>
       <c r="X14" s="7"/>
-      <c r="Y14" s="8"/>
+      <c r="Y14" s="7"/>
       <c r="Z14" s="8"/>
       <c r="AA14" s="8"/>
       <c r="AB14" s="8"/>
       <c r="AC14" s="8"/>
-      <c r="AD14" s="7"/>
+      <c r="AD14" s="8"/>
       <c r="AE14" s="7"/>
       <c r="AF14" s="7"/>
       <c r="AG14" s="7"/>
       <c r="AH14" s="7"/>
       <c r="AI14" s="7"/>
-      <c r="AJ14" s="9"/>
-      <c r="AL14" s="7"/>
+      <c r="AJ14" s="7"/>
+      <c r="AK14" s="9"/>
       <c r="AM14" s="7"/>
       <c r="AN14" s="7"/>
       <c r="AO14" s="7"/>
       <c r="AP14" s="7"/>
       <c r="AQ14" s="7"/>
-      <c r="AS14" s="7"/>
-      <c r="AU14" s="7"/>
-      <c r="AW14" s="7"/>
-      <c r="AY14" s="7"/>
-      <c r="BD14" s="7"/>
-      <c r="BI14" s="7"/>
-    </row>
-    <row r="15" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR14" s="7"/>
+      <c r="AT14" s="7"/>
+      <c r="AV14" s="7"/>
+      <c r="AX14" s="7"/>
+      <c r="AZ14" s="7"/>
+      <c r="BE14" s="7"/>
+      <c r="BJ14" s="7"/>
+    </row>
+    <row r="15" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>1992</v>
       </c>
@@ -1778,40 +1844,41 @@
       <c r="P15" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q15" s="5"/>
+      <c r="Q15" s="7"/>
       <c r="R15" s="5"/>
       <c r="S15" s="5"/>
-      <c r="T15" s="7"/>
+      <c r="T15" s="5"/>
       <c r="U15" s="7"/>
       <c r="V15" s="7"/>
       <c r="W15" s="7"/>
       <c r="X15" s="7"/>
-      <c r="Y15" s="8"/>
+      <c r="Y15" s="7"/>
       <c r="Z15" s="8"/>
       <c r="AA15" s="8"/>
       <c r="AB15" s="8"/>
       <c r="AC15" s="8"/>
-      <c r="AD15" s="7"/>
+      <c r="AD15" s="8"/>
       <c r="AE15" s="7"/>
       <c r="AF15" s="7"/>
       <c r="AG15" s="7"/>
       <c r="AH15" s="7"/>
       <c r="AI15" s="7"/>
-      <c r="AJ15" s="9"/>
-      <c r="AL15" s="7"/>
+      <c r="AJ15" s="7"/>
+      <c r="AK15" s="9"/>
       <c r="AM15" s="7"/>
       <c r="AN15" s="7"/>
       <c r="AO15" s="7"/>
       <c r="AP15" s="7"/>
       <c r="AQ15" s="7"/>
-      <c r="AS15" s="7"/>
-      <c r="AU15" s="7"/>
-      <c r="AW15" s="7"/>
-      <c r="AY15" s="7"/>
-      <c r="BD15" s="7"/>
-      <c r="BI15" s="7"/>
-    </row>
-    <row r="16" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR15" s="7"/>
+      <c r="AT15" s="7"/>
+      <c r="AV15" s="7"/>
+      <c r="AX15" s="7"/>
+      <c r="AZ15" s="7"/>
+      <c r="BE15" s="7"/>
+      <c r="BJ15" s="7"/>
+    </row>
+    <row r="16" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>1993</v>
       </c>
@@ -1853,40 +1920,41 @@
       <c r="P16" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q16" s="5"/>
+      <c r="Q16" s="7"/>
       <c r="R16" s="5"/>
       <c r="S16" s="5"/>
-      <c r="T16" s="7"/>
+      <c r="T16" s="5"/>
       <c r="U16" s="7"/>
       <c r="V16" s="7"/>
       <c r="W16" s="7"/>
       <c r="X16" s="7"/>
-      <c r="Y16" s="8"/>
+      <c r="Y16" s="7"/>
       <c r="Z16" s="8"/>
       <c r="AA16" s="8"/>
       <c r="AB16" s="8"/>
       <c r="AC16" s="8"/>
-      <c r="AD16" s="7"/>
+      <c r="AD16" s="8"/>
       <c r="AE16" s="7"/>
       <c r="AF16" s="7"/>
       <c r="AG16" s="7"/>
       <c r="AH16" s="7"/>
       <c r="AI16" s="7"/>
-      <c r="AJ16" s="9"/>
-      <c r="AL16" s="7"/>
+      <c r="AJ16" s="7"/>
+      <c r="AK16" s="9"/>
       <c r="AM16" s="7"/>
       <c r="AN16" s="7"/>
       <c r="AO16" s="7"/>
       <c r="AP16" s="7"/>
       <c r="AQ16" s="7"/>
-      <c r="AS16" s="7"/>
-      <c r="AU16" s="7"/>
-      <c r="AW16" s="7"/>
-      <c r="AY16" s="7"/>
-      <c r="BD16" s="7"/>
-      <c r="BI16" s="7"/>
-    </row>
-    <row r="17" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR16" s="7"/>
+      <c r="AT16" s="7"/>
+      <c r="AV16" s="7"/>
+      <c r="AX16" s="7"/>
+      <c r="AZ16" s="7"/>
+      <c r="BE16" s="7"/>
+      <c r="BJ16" s="7"/>
+    </row>
+    <row r="17" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>1994</v>
       </c>
@@ -1912,7 +1980,7 @@
         <v>733</v>
       </c>
       <c r="L17" s="7">
-        <f t="shared" si="3"/>
+        <f>SUM(F17,H17,I17)</f>
         <v>1467</v>
       </c>
       <c r="M17" s="23">
@@ -1928,40 +1996,41 @@
       <c r="P17" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q17" s="5"/>
+      <c r="Q17" s="7"/>
       <c r="R17" s="5"/>
       <c r="S17" s="5"/>
-      <c r="T17" s="7"/>
+      <c r="T17" s="5"/>
       <c r="U17" s="7"/>
       <c r="V17" s="7"/>
       <c r="W17" s="7"/>
       <c r="X17" s="7"/>
-      <c r="Y17" s="8"/>
+      <c r="Y17" s="7"/>
       <c r="Z17" s="8"/>
       <c r="AA17" s="8"/>
       <c r="AB17" s="8"/>
       <c r="AC17" s="8"/>
-      <c r="AD17" s="7"/>
+      <c r="AD17" s="8"/>
       <c r="AE17" s="7"/>
       <c r="AF17" s="7"/>
       <c r="AG17" s="7"/>
       <c r="AH17" s="7"/>
       <c r="AI17" s="7"/>
-      <c r="AJ17" s="9"/>
-      <c r="AL17" s="7"/>
+      <c r="AJ17" s="7"/>
+      <c r="AK17" s="9"/>
       <c r="AM17" s="7"/>
       <c r="AN17" s="7"/>
       <c r="AO17" s="7"/>
       <c r="AP17" s="7"/>
       <c r="AQ17" s="7"/>
-      <c r="AS17" s="7"/>
-      <c r="AU17" s="7"/>
-      <c r="AW17" s="7"/>
-      <c r="AY17" s="7"/>
-      <c r="BD17" s="7"/>
-      <c r="BI17" s="7"/>
-    </row>
-    <row r="18" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR17" s="7"/>
+      <c r="AT17" s="7"/>
+      <c r="AV17" s="7"/>
+      <c r="AX17" s="7"/>
+      <c r="AZ17" s="7"/>
+      <c r="BE17" s="7"/>
+      <c r="BJ17" s="7"/>
+    </row>
+    <row r="18" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>1995</v>
       </c>
@@ -2003,40 +2072,41 @@
       <c r="P18" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q18" s="5"/>
+      <c r="Q18" s="7"/>
       <c r="R18" s="5"/>
       <c r="S18" s="5"/>
-      <c r="T18" s="7"/>
+      <c r="T18" s="5"/>
       <c r="U18" s="7"/>
       <c r="V18" s="7"/>
       <c r="W18" s="7"/>
       <c r="X18" s="7"/>
-      <c r="Y18" s="8"/>
+      <c r="Y18" s="7"/>
       <c r="Z18" s="8"/>
       <c r="AA18" s="8"/>
       <c r="AB18" s="8"/>
       <c r="AC18" s="8"/>
-      <c r="AD18" s="7"/>
+      <c r="AD18" s="8"/>
       <c r="AE18" s="7"/>
       <c r="AF18" s="7"/>
       <c r="AG18" s="7"/>
       <c r="AH18" s="7"/>
       <c r="AI18" s="7"/>
-      <c r="AJ18" s="9"/>
-      <c r="AL18" s="7"/>
+      <c r="AJ18" s="7"/>
+      <c r="AK18" s="9"/>
       <c r="AM18" s="7"/>
       <c r="AN18" s="7"/>
       <c r="AO18" s="7"/>
       <c r="AP18" s="7"/>
       <c r="AQ18" s="7"/>
-      <c r="AS18" s="7"/>
-      <c r="AU18" s="7"/>
-      <c r="AW18" s="7"/>
-      <c r="AY18" s="7"/>
-      <c r="BD18" s="7"/>
-      <c r="BI18" s="7"/>
-    </row>
-    <row r="19" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR18" s="7"/>
+      <c r="AT18" s="7"/>
+      <c r="AV18" s="7"/>
+      <c r="AX18" s="7"/>
+      <c r="AZ18" s="7"/>
+      <c r="BE18" s="7"/>
+      <c r="BJ18" s="7"/>
+    </row>
+    <row r="19" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>1996</v>
       </c>
@@ -2078,40 +2148,41 @@
       <c r="P19" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q19" s="5"/>
+      <c r="Q19" s="7"/>
       <c r="R19" s="5"/>
       <c r="S19" s="5"/>
-      <c r="T19" s="7"/>
+      <c r="T19" s="5"/>
       <c r="U19" s="7"/>
       <c r="V19" s="7"/>
       <c r="W19" s="7"/>
       <c r="X19" s="7"/>
-      <c r="Y19" s="8"/>
+      <c r="Y19" s="7"/>
       <c r="Z19" s="8"/>
       <c r="AA19" s="8"/>
       <c r="AB19" s="8"/>
       <c r="AC19" s="8"/>
-      <c r="AD19" s="7"/>
+      <c r="AD19" s="8"/>
       <c r="AE19" s="7"/>
       <c r="AF19" s="7"/>
       <c r="AG19" s="7"/>
       <c r="AH19" s="7"/>
       <c r="AI19" s="7"/>
-      <c r="AJ19" s="9"/>
-      <c r="AL19" s="7"/>
+      <c r="AJ19" s="7"/>
+      <c r="AK19" s="9"/>
       <c r="AM19" s="7"/>
       <c r="AN19" s="7"/>
       <c r="AO19" s="7"/>
       <c r="AP19" s="7"/>
       <c r="AQ19" s="7"/>
-      <c r="AS19" s="7"/>
-      <c r="AU19" s="7"/>
-      <c r="AW19" s="7"/>
-      <c r="AY19" s="7"/>
-      <c r="BD19" s="7"/>
-      <c r="BI19" s="7"/>
-    </row>
-    <row r="20" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR19" s="7"/>
+      <c r="AT19" s="7"/>
+      <c r="AV19" s="7"/>
+      <c r="AX19" s="7"/>
+      <c r="AZ19" s="7"/>
+      <c r="BE19" s="7"/>
+      <c r="BJ19" s="7"/>
+    </row>
+    <row r="20" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>1997</v>
       </c>
@@ -2136,7 +2207,7 @@
         <v>1000</v>
       </c>
       <c r="L20" s="7">
-        <f t="shared" si="3"/>
+        <f>SUM(F20,H20,I20)</f>
         <v>2500</v>
       </c>
       <c r="M20" s="23">
@@ -2152,39 +2223,40 @@
       <c r="P20" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q20" s="5"/>
+      <c r="Q20" s="7"/>
       <c r="R20" s="5"/>
       <c r="S20" s="5"/>
-      <c r="T20" s="7"/>
+      <c r="T20" s="5"/>
       <c r="U20" s="7"/>
       <c r="V20" s="7"/>
       <c r="W20" s="7"/>
       <c r="X20" s="7"/>
-      <c r="Y20" s="8"/>
+      <c r="Y20" s="7"/>
       <c r="Z20" s="8"/>
       <c r="AA20" s="8"/>
       <c r="AB20" s="8"/>
       <c r="AC20" s="8"/>
-      <c r="AD20" s="7"/>
+      <c r="AD20" s="8"/>
       <c r="AE20" s="7"/>
       <c r="AF20" s="7"/>
       <c r="AG20" s="7"/>
       <c r="AH20" s="7"/>
       <c r="AI20" s="7"/>
-      <c r="AL20" s="7"/>
+      <c r="AJ20" s="7"/>
       <c r="AM20" s="7"/>
       <c r="AN20" s="7"/>
       <c r="AO20" s="7"/>
       <c r="AP20" s="7"/>
       <c r="AQ20" s="7"/>
-      <c r="AS20" s="7"/>
-      <c r="AU20" s="7"/>
-      <c r="AW20" s="7"/>
-      <c r="AY20" s="7"/>
-      <c r="BD20" s="7"/>
-      <c r="BI20" s="7"/>
-    </row>
-    <row r="21" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR20" s="7"/>
+      <c r="AT20" s="7"/>
+      <c r="AV20" s="7"/>
+      <c r="AX20" s="7"/>
+      <c r="AZ20" s="7"/>
+      <c r="BE20" s="7"/>
+      <c r="BJ20" s="7"/>
+    </row>
+    <row r="21" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>1998</v>
       </c>
@@ -2225,39 +2297,40 @@
       <c r="P21" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q21" s="5"/>
+      <c r="Q21" s="7"/>
       <c r="R21" s="5"/>
       <c r="S21" s="5"/>
-      <c r="T21" s="7"/>
+      <c r="T21" s="5"/>
       <c r="U21" s="7"/>
       <c r="V21" s="7"/>
       <c r="W21" s="7"/>
       <c r="X21" s="7"/>
-      <c r="Y21" s="8"/>
+      <c r="Y21" s="7"/>
       <c r="Z21" s="8"/>
       <c r="AA21" s="8"/>
       <c r="AB21" s="8"/>
       <c r="AC21" s="8"/>
-      <c r="AD21" s="7"/>
+      <c r="AD21" s="8"/>
       <c r="AE21" s="7"/>
       <c r="AF21" s="7"/>
       <c r="AG21" s="7"/>
       <c r="AH21" s="7"/>
       <c r="AI21" s="7"/>
-      <c r="AL21" s="7"/>
+      <c r="AJ21" s="7"/>
       <c r="AM21" s="7"/>
       <c r="AN21" s="7"/>
       <c r="AO21" s="7"/>
       <c r="AP21" s="7"/>
       <c r="AQ21" s="7"/>
-      <c r="AS21" s="7"/>
-      <c r="AU21" s="7"/>
-      <c r="AW21" s="7"/>
-      <c r="AY21" s="7"/>
-      <c r="BD21" s="7"/>
-      <c r="BI21" s="7"/>
-    </row>
-    <row r="22" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR21" s="7"/>
+      <c r="AT21" s="7"/>
+      <c r="AV21" s="7"/>
+      <c r="AX21" s="7"/>
+      <c r="AZ21" s="7"/>
+      <c r="BE21" s="7"/>
+      <c r="BJ21" s="7"/>
+    </row>
+    <row r="22" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>1999</v>
       </c>
@@ -2298,39 +2371,40 @@
       <c r="P22" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q22" s="5"/>
+      <c r="Q22" s="7"/>
       <c r="R22" s="5"/>
       <c r="S22" s="5"/>
-      <c r="T22" s="7"/>
+      <c r="T22" s="5"/>
       <c r="U22" s="7"/>
       <c r="V22" s="7"/>
       <c r="W22" s="7"/>
       <c r="X22" s="7"/>
-      <c r="Y22" s="8"/>
+      <c r="Y22" s="7"/>
       <c r="Z22" s="8"/>
       <c r="AA22" s="8"/>
       <c r="AB22" s="8"/>
       <c r="AC22" s="8"/>
-      <c r="AD22" s="7"/>
+      <c r="AD22" s="8"/>
       <c r="AE22" s="7"/>
       <c r="AF22" s="7"/>
       <c r="AG22" s="7"/>
       <c r="AH22" s="7"/>
       <c r="AI22" s="7"/>
-      <c r="AL22" s="7"/>
+      <c r="AJ22" s="7"/>
       <c r="AM22" s="7"/>
       <c r="AN22" s="7"/>
       <c r="AO22" s="7"/>
       <c r="AP22" s="7"/>
       <c r="AQ22" s="7"/>
-      <c r="AS22" s="7"/>
-      <c r="AU22" s="7"/>
-      <c r="AW22" s="7"/>
-      <c r="AY22" s="7"/>
-      <c r="BD22" s="7"/>
-      <c r="BI22" s="7"/>
-    </row>
-    <row r="23" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR22" s="7"/>
+      <c r="AT22" s="7"/>
+      <c r="AV22" s="7"/>
+      <c r="AX22" s="7"/>
+      <c r="AZ22" s="7"/>
+      <c r="BE22" s="7"/>
+      <c r="BJ22" s="7"/>
+    </row>
+    <row r="23" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>2000</v>
       </c>
@@ -2371,39 +2445,40 @@
       <c r="P23" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q23" s="5"/>
+      <c r="Q23" s="7"/>
       <c r="R23" s="5"/>
       <c r="S23" s="5"/>
-      <c r="T23" s="7"/>
+      <c r="T23" s="5"/>
       <c r="U23" s="7"/>
       <c r="V23" s="7"/>
       <c r="W23" s="7"/>
       <c r="X23" s="7"/>
-      <c r="Y23" s="8"/>
+      <c r="Y23" s="7"/>
       <c r="Z23" s="8"/>
       <c r="AA23" s="8"/>
       <c r="AB23" s="8"/>
       <c r="AC23" s="8"/>
-      <c r="AD23" s="7"/>
+      <c r="AD23" s="8"/>
       <c r="AE23" s="7"/>
       <c r="AF23" s="7"/>
       <c r="AG23" s="7"/>
       <c r="AH23" s="7"/>
       <c r="AI23" s="7"/>
-      <c r="AL23" s="7"/>
+      <c r="AJ23" s="7"/>
       <c r="AM23" s="7"/>
       <c r="AN23" s="7"/>
       <c r="AO23" s="7"/>
       <c r="AP23" s="7"/>
       <c r="AQ23" s="7"/>
-      <c r="AS23" s="7"/>
-      <c r="AU23" s="7"/>
-      <c r="AW23" s="7"/>
-      <c r="AY23" s="7"/>
-      <c r="BD23" s="7"/>
-      <c r="BI23" s="7"/>
-    </row>
-    <row r="24" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR23" s="7"/>
+      <c r="AT23" s="7"/>
+      <c r="AV23" s="7"/>
+      <c r="AX23" s="7"/>
+      <c r="AZ23" s="7"/>
+      <c r="BE23" s="7"/>
+      <c r="BJ23" s="7"/>
+    </row>
+    <row r="24" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>2001</v>
       </c>
@@ -2428,7 +2503,7 @@
         <v>1000</v>
       </c>
       <c r="L24" s="7">
-        <f t="shared" si="3"/>
+        <f>SUM(F24,H24,I24)</f>
         <v>5000</v>
       </c>
       <c r="M24" s="23">
@@ -2444,39 +2519,42 @@
       <c r="P24" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q24" s="5"/>
+      <c r="Q24" s="7"/>
       <c r="R24" s="5"/>
-      <c r="S24" s="5"/>
-      <c r="T24" s="7"/>
+      <c r="S24" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="T24" s="5"/>
       <c r="U24" s="7"/>
       <c r="V24" s="7"/>
       <c r="W24" s="7"/>
       <c r="X24" s="7"/>
-      <c r="Y24" s="8"/>
+      <c r="Y24" s="7"/>
       <c r="Z24" s="8"/>
       <c r="AA24" s="8"/>
       <c r="AB24" s="8"/>
       <c r="AC24" s="8"/>
-      <c r="AD24" s="7"/>
+      <c r="AD24" s="8"/>
       <c r="AE24" s="7"/>
       <c r="AF24" s="7"/>
       <c r="AG24" s="7"/>
       <c r="AH24" s="7"/>
       <c r="AI24" s="7"/>
-      <c r="AL24" s="7"/>
+      <c r="AJ24" s="7"/>
       <c r="AM24" s="7"/>
       <c r="AN24" s="7"/>
       <c r="AO24" s="7"/>
       <c r="AP24" s="7"/>
       <c r="AQ24" s="7"/>
-      <c r="AS24" s="7"/>
-      <c r="AU24" s="7"/>
-      <c r="AW24" s="7"/>
-      <c r="AY24" s="7"/>
-      <c r="BD24" s="7"/>
-      <c r="BI24" s="7"/>
-    </row>
-    <row r="25" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR24" s="7"/>
+      <c r="AT24" s="7"/>
+      <c r="AV24" s="7"/>
+      <c r="AX24" s="7"/>
+      <c r="AZ24" s="7"/>
+      <c r="BE24" s="7"/>
+      <c r="BJ24" s="7"/>
+    </row>
+    <row r="25" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>2002</v>
       </c>
@@ -2502,11 +2580,11 @@
         <v>3962</v>
       </c>
       <c r="L25" s="7">
-        <f t="shared" si="3"/>
+        <f>SUM(F25,H25,I25)</f>
         <v>3962</v>
       </c>
       <c r="M25" s="23">
-        <f t="shared" si="4"/>
+        <f>SUM(J25,K25)</f>
         <v>0</v>
       </c>
       <c r="N25" s="1">
@@ -2518,39 +2596,42 @@
       <c r="P25" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q25" s="5"/>
-      <c r="R25" s="5"/>
+      <c r="Q25" s="30"/>
+      <c r="R25" s="5" t="s">
+        <v>36</v>
+      </c>
       <c r="S25" s="5"/>
-      <c r="T25" s="7"/>
+      <c r="T25" s="5"/>
       <c r="U25" s="7"/>
       <c r="V25" s="7"/>
       <c r="W25" s="7"/>
       <c r="X25" s="7"/>
-      <c r="Y25" s="8"/>
+      <c r="Y25" s="7"/>
       <c r="Z25" s="8"/>
       <c r="AA25" s="8"/>
       <c r="AB25" s="8"/>
       <c r="AC25" s="8"/>
-      <c r="AD25" s="7"/>
+      <c r="AD25" s="8"/>
       <c r="AE25" s="7"/>
       <c r="AF25" s="7"/>
       <c r="AG25" s="7"/>
       <c r="AH25" s="7"/>
       <c r="AI25" s="7"/>
-      <c r="AL25" s="7"/>
+      <c r="AJ25" s="7"/>
       <c r="AM25" s="7"/>
       <c r="AN25" s="7"/>
       <c r="AO25" s="7"/>
       <c r="AP25" s="7"/>
       <c r="AQ25" s="7"/>
-      <c r="AS25" s="7"/>
-      <c r="AU25" s="7"/>
-      <c r="AW25" s="7"/>
-      <c r="AY25" s="7"/>
-      <c r="BD25" s="7"/>
-      <c r="BI25" s="7"/>
-    </row>
-    <row r="26" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR25" s="7"/>
+      <c r="AT25" s="7"/>
+      <c r="AV25" s="7"/>
+      <c r="AX25" s="7"/>
+      <c r="AZ25" s="7"/>
+      <c r="BE25" s="7"/>
+      <c r="BJ25" s="7"/>
+    </row>
+    <row r="26" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>2003</v>
       </c>
@@ -2601,39 +2682,42 @@
       <c r="P26" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q26" s="5"/>
-      <c r="R26" s="5"/>
+      <c r="Q26" s="30"/>
+      <c r="R26" s="5" t="s">
+        <v>36</v>
+      </c>
       <c r="S26" s="5"/>
-      <c r="T26" s="7"/>
+      <c r="T26" s="5"/>
       <c r="U26" s="7"/>
       <c r="V26" s="7"/>
       <c r="W26" s="7"/>
       <c r="X26" s="7"/>
-      <c r="Y26" s="8"/>
+      <c r="Y26" s="7"/>
       <c r="Z26" s="8"/>
       <c r="AA26" s="8"/>
       <c r="AB26" s="8"/>
       <c r="AC26" s="8"/>
-      <c r="AD26" s="7"/>
+      <c r="AD26" s="8"/>
       <c r="AE26" s="7"/>
       <c r="AF26" s="7"/>
       <c r="AG26" s="7"/>
       <c r="AH26" s="7"/>
       <c r="AI26" s="7"/>
-      <c r="AL26" s="7"/>
+      <c r="AJ26" s="7"/>
       <c r="AM26" s="7"/>
       <c r="AN26" s="7"/>
       <c r="AO26" s="7"/>
       <c r="AP26" s="7"/>
       <c r="AQ26" s="7"/>
-      <c r="AS26" s="7"/>
-      <c r="AU26" s="7"/>
-      <c r="AW26" s="7"/>
-      <c r="AY26" s="7"/>
-      <c r="BD26" s="7"/>
-      <c r="BI26" s="7"/>
-    </row>
-    <row r="27" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR26" s="7"/>
+      <c r="AT26" s="7"/>
+      <c r="AV26" s="7"/>
+      <c r="AX26" s="7"/>
+      <c r="AZ26" s="7"/>
+      <c r="BE26" s="7"/>
+      <c r="BJ26" s="7"/>
+    </row>
+    <row r="27" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>2004</v>
       </c>
@@ -2658,7 +2742,7 @@
         <v>1000</v>
       </c>
       <c r="L27" s="7">
-        <f t="shared" si="3"/>
+        <f>SUM(F27,H27,I27)</f>
         <v>5000</v>
       </c>
       <c r="M27" s="23">
@@ -2674,39 +2758,40 @@
       <c r="P27" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q27" s="5"/>
+      <c r="Q27" s="7"/>
       <c r="R27" s="5"/>
       <c r="S27" s="5"/>
-      <c r="T27" s="7"/>
+      <c r="T27" s="5"/>
       <c r="U27" s="7"/>
       <c r="V27" s="7"/>
       <c r="W27" s="7"/>
       <c r="X27" s="7"/>
-      <c r="Y27" s="8"/>
+      <c r="Y27" s="7"/>
       <c r="Z27" s="8"/>
       <c r="AA27" s="8"/>
       <c r="AB27" s="8"/>
       <c r="AC27" s="8"/>
-      <c r="AD27" s="7"/>
+      <c r="AD27" s="8"/>
       <c r="AE27" s="7"/>
       <c r="AF27" s="7"/>
       <c r="AG27" s="7"/>
       <c r="AH27" s="7"/>
       <c r="AI27" s="7"/>
-      <c r="AL27" s="7"/>
+      <c r="AJ27" s="7"/>
       <c r="AM27" s="7"/>
       <c r="AN27" s="7"/>
       <c r="AO27" s="7"/>
       <c r="AP27" s="7"/>
       <c r="AQ27" s="7"/>
-      <c r="AS27" s="7"/>
-      <c r="AU27" s="7"/>
-      <c r="AW27" s="7"/>
-      <c r="AY27" s="7"/>
-      <c r="BD27" s="7"/>
-      <c r="BI27" s="7"/>
-    </row>
-    <row r="28" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR27" s="7"/>
+      <c r="AT27" s="7"/>
+      <c r="AV27" s="7"/>
+      <c r="AX27" s="7"/>
+      <c r="AZ27" s="7"/>
+      <c r="BE27" s="7"/>
+      <c r="BJ27" s="7"/>
+    </row>
+    <row r="28" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>2005</v>
       </c>
@@ -2731,7 +2816,7 @@
         <v>1000</v>
       </c>
       <c r="L28" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="L24:L35" si="5">SUM(F28,H28,I28)</f>
         <v>2500</v>
       </c>
       <c r="M28" s="23">
@@ -2747,39 +2832,40 @@
       <c r="P28" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q28" s="5"/>
+      <c r="Q28" s="7"/>
       <c r="R28" s="5"/>
       <c r="S28" s="5"/>
-      <c r="T28" s="7"/>
+      <c r="T28" s="5"/>
       <c r="U28" s="7"/>
       <c r="V28" s="7"/>
       <c r="W28" s="7"/>
       <c r="X28" s="7"/>
-      <c r="Y28" s="8"/>
+      <c r="Y28" s="7"/>
       <c r="Z28" s="8"/>
       <c r="AA28" s="8"/>
       <c r="AB28" s="8"/>
       <c r="AC28" s="8"/>
-      <c r="AD28" s="7"/>
+      <c r="AD28" s="8"/>
       <c r="AE28" s="7"/>
       <c r="AF28" s="7"/>
       <c r="AG28" s="7"/>
       <c r="AH28" s="7"/>
       <c r="AI28" s="7"/>
-      <c r="AL28" s="7"/>
+      <c r="AJ28" s="7"/>
       <c r="AM28" s="7"/>
       <c r="AN28" s="7"/>
       <c r="AO28" s="7"/>
       <c r="AP28" s="7"/>
       <c r="AQ28" s="7"/>
-      <c r="AS28" s="7"/>
-      <c r="AU28" s="7"/>
-      <c r="AW28" s="7"/>
-      <c r="AY28" s="7"/>
-      <c r="BD28" s="7"/>
-      <c r="BI28" s="7"/>
-    </row>
-    <row r="29" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR28" s="7"/>
+      <c r="AT28" s="7"/>
+      <c r="AV28" s="7"/>
+      <c r="AX28" s="7"/>
+      <c r="AZ28" s="7"/>
+      <c r="BE28" s="7"/>
+      <c r="BJ28" s="7"/>
+    </row>
+    <row r="29" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>2006</v>
       </c>
@@ -2804,7 +2890,7 @@
         <v>1000</v>
       </c>
       <c r="L29" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>2500</v>
       </c>
       <c r="M29" s="23">
@@ -2820,39 +2906,40 @@
       <c r="P29" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q29" s="5"/>
+      <c r="Q29" s="7"/>
       <c r="R29" s="5"/>
       <c r="S29" s="5"/>
-      <c r="T29" s="7"/>
+      <c r="T29" s="5"/>
       <c r="U29" s="7"/>
       <c r="V29" s="7"/>
       <c r="W29" s="7"/>
       <c r="X29" s="7"/>
-      <c r="Y29" s="8"/>
+      <c r="Y29" s="7"/>
       <c r="Z29" s="8"/>
       <c r="AA29" s="8"/>
       <c r="AB29" s="8"/>
       <c r="AC29" s="8"/>
-      <c r="AD29" s="7"/>
+      <c r="AD29" s="8"/>
       <c r="AE29" s="7"/>
       <c r="AF29" s="7"/>
       <c r="AG29" s="7"/>
       <c r="AH29" s="7"/>
       <c r="AI29" s="7"/>
-      <c r="AL29" s="7"/>
+      <c r="AJ29" s="7"/>
       <c r="AM29" s="7"/>
       <c r="AN29" s="7"/>
       <c r="AO29" s="7"/>
       <c r="AP29" s="7"/>
       <c r="AQ29" s="7"/>
-      <c r="AS29" s="7"/>
-      <c r="AU29" s="7"/>
-      <c r="AW29" s="7"/>
-      <c r="AY29" s="7"/>
-      <c r="BD29" s="7"/>
-      <c r="BI29" s="7"/>
-    </row>
-    <row r="30" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR29" s="7"/>
+      <c r="AT29" s="7"/>
+      <c r="AV29" s="7"/>
+      <c r="AX29" s="7"/>
+      <c r="AZ29" s="7"/>
+      <c r="BE29" s="7"/>
+      <c r="BJ29" s="7"/>
+    </row>
+    <row r="30" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>2007</v>
       </c>
@@ -2878,7 +2965,7 @@
         <v>500</v>
       </c>
       <c r="L30" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>500</v>
       </c>
       <c r="M30" s="23">
@@ -2894,39 +2981,40 @@
       <c r="P30" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q30" s="5"/>
+      <c r="Q30" s="7"/>
       <c r="R30" s="5"/>
       <c r="S30" s="5"/>
-      <c r="T30" s="7"/>
+      <c r="T30" s="5"/>
       <c r="U30" s="7"/>
       <c r="V30" s="7"/>
       <c r="W30" s="7"/>
       <c r="X30" s="7"/>
-      <c r="Y30" s="8"/>
+      <c r="Y30" s="7"/>
       <c r="Z30" s="8"/>
       <c r="AA30" s="8"/>
       <c r="AB30" s="8"/>
       <c r="AC30" s="8"/>
-      <c r="AD30" s="7"/>
+      <c r="AD30" s="8"/>
       <c r="AE30" s="7"/>
       <c r="AF30" s="7"/>
       <c r="AG30" s="7"/>
       <c r="AH30" s="7"/>
       <c r="AI30" s="7"/>
-      <c r="AL30" s="7"/>
+      <c r="AJ30" s="7"/>
       <c r="AM30" s="7"/>
       <c r="AN30" s="7"/>
       <c r="AO30" s="7"/>
       <c r="AP30" s="7"/>
       <c r="AQ30" s="7"/>
-      <c r="AS30" s="7"/>
-      <c r="AU30" s="7"/>
-      <c r="AW30" s="7"/>
-      <c r="AY30" s="7"/>
-      <c r="BD30" s="7"/>
-      <c r="BI30" s="7"/>
-    </row>
-    <row r="31" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR30" s="7"/>
+      <c r="AT30" s="7"/>
+      <c r="AV30" s="7"/>
+      <c r="AX30" s="7"/>
+      <c r="AZ30" s="7"/>
+      <c r="BE30" s="7"/>
+      <c r="BJ30" s="7"/>
+    </row>
+    <row r="31" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>2008</v>
       </c>
@@ -2951,7 +3039,7 @@
         <v>1000</v>
       </c>
       <c r="L31" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>2500</v>
       </c>
       <c r="M31" s="23">
@@ -2967,39 +3055,40 @@
       <c r="P31" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q31" s="5"/>
+      <c r="Q31" s="7"/>
       <c r="R31" s="5"/>
       <c r="S31" s="5"/>
-      <c r="T31" s="7"/>
+      <c r="T31" s="5"/>
       <c r="U31" s="7"/>
       <c r="V31" s="7"/>
       <c r="W31" s="7"/>
       <c r="X31" s="7"/>
-      <c r="Y31" s="8"/>
+      <c r="Y31" s="7"/>
       <c r="Z31" s="8"/>
       <c r="AA31" s="8"/>
       <c r="AB31" s="8"/>
       <c r="AC31" s="8"/>
-      <c r="AD31" s="7"/>
+      <c r="AD31" s="8"/>
       <c r="AE31" s="7"/>
       <c r="AF31" s="7"/>
       <c r="AG31" s="7"/>
       <c r="AH31" s="7"/>
       <c r="AI31" s="7"/>
-      <c r="AL31" s="7"/>
+      <c r="AJ31" s="7"/>
       <c r="AM31" s="7"/>
       <c r="AN31" s="7"/>
       <c r="AO31" s="7"/>
       <c r="AP31" s="7"/>
       <c r="AQ31" s="7"/>
-      <c r="AS31" s="7"/>
-      <c r="AU31" s="7"/>
-      <c r="AW31" s="7"/>
-      <c r="AY31" s="7"/>
-      <c r="BD31" s="7"/>
-      <c r="BI31" s="7"/>
-    </row>
-    <row r="32" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR31" s="7"/>
+      <c r="AT31" s="7"/>
+      <c r="AV31" s="7"/>
+      <c r="AX31" s="7"/>
+      <c r="AZ31" s="7"/>
+      <c r="BE31" s="7"/>
+      <c r="BJ31" s="7"/>
+    </row>
+    <row r="32" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
         <v>2009</v>
       </c>
@@ -3024,7 +3113,7 @@
         <v>1000</v>
       </c>
       <c r="L32" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>2500</v>
       </c>
       <c r="M32" s="23">
@@ -3040,39 +3129,40 @@
       <c r="P32" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q32" s="5"/>
+      <c r="Q32" s="7"/>
       <c r="R32" s="5"/>
       <c r="S32" s="5"/>
-      <c r="T32" s="7"/>
+      <c r="T32" s="5"/>
       <c r="U32" s="7"/>
       <c r="V32" s="7"/>
       <c r="W32" s="7"/>
       <c r="X32" s="7"/>
-      <c r="Y32" s="8"/>
+      <c r="Y32" s="7"/>
       <c r="Z32" s="8"/>
       <c r="AA32" s="8"/>
       <c r="AB32" s="8"/>
       <c r="AC32" s="8"/>
-      <c r="AD32" s="7"/>
+      <c r="AD32" s="8"/>
       <c r="AE32" s="7"/>
       <c r="AF32" s="7"/>
       <c r="AG32" s="7"/>
       <c r="AH32" s="7"/>
       <c r="AI32" s="7"/>
-      <c r="AL32" s="7"/>
+      <c r="AJ32" s="7"/>
       <c r="AM32" s="7"/>
       <c r="AN32" s="7"/>
       <c r="AO32" s="7"/>
       <c r="AP32" s="7"/>
       <c r="AQ32" s="7"/>
-      <c r="AS32" s="7"/>
-      <c r="AU32" s="7"/>
-      <c r="AW32" s="7"/>
-      <c r="AY32" s="7"/>
-      <c r="BD32" s="7"/>
-      <c r="BI32" s="7"/>
-    </row>
-    <row r="33" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR32" s="7"/>
+      <c r="AT32" s="7"/>
+      <c r="AV32" s="7"/>
+      <c r="AX32" s="7"/>
+      <c r="AZ32" s="7"/>
+      <c r="BE32" s="7"/>
+      <c r="BJ32" s="7"/>
+    </row>
+    <row r="33" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>2010</v>
       </c>
@@ -3087,22 +3177,22 @@
         <v>1043</v>
       </c>
       <c r="E33" s="11">
-        <f t="shared" ref="E33:E43" si="5">SUM(F33:I33)</f>
+        <f t="shared" ref="E33:E45" si="6">SUM(F33:I33)</f>
         <v>2821</v>
       </c>
       <c r="F33" s="11">
         <v>2351</v>
       </c>
       <c r="G33" s="14">
-        <f t="shared" ref="G33:G40" si="6">ROUND(0.2*SUM(F33,H33,I33),0)</f>
+        <f>ROUND(0.2*SUM(F33,H33,I33),0)</f>
         <v>470</v>
       </c>
       <c r="L33" s="7">
-        <f t="shared" si="3"/>
+        <f>SUM(F33,H33,I33)</f>
         <v>2351</v>
       </c>
       <c r="M33" s="23">
-        <f t="shared" si="4"/>
+        <f>SUM(J33,K33)</f>
         <v>0</v>
       </c>
       <c r="N33" s="1">
@@ -3114,39 +3204,42 @@
       <c r="P33" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q33" s="5"/>
+      <c r="Q33" s="7"/>
       <c r="R33" s="5"/>
-      <c r="S33" s="5"/>
-      <c r="T33" s="7"/>
+      <c r="S33" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="T33" s="5"/>
       <c r="U33" s="7"/>
       <c r="V33" s="7"/>
       <c r="W33" s="7"/>
       <c r="X33" s="7"/>
-      <c r="Y33" s="8"/>
+      <c r="Y33" s="7"/>
       <c r="Z33" s="8"/>
       <c r="AA33" s="8"/>
       <c r="AB33" s="8"/>
       <c r="AC33" s="8"/>
-      <c r="AD33" s="7"/>
+      <c r="AD33" s="8"/>
       <c r="AE33" s="7"/>
       <c r="AF33" s="7"/>
       <c r="AG33" s="7"/>
       <c r="AH33" s="7"/>
       <c r="AI33" s="7"/>
-      <c r="AL33" s="7"/>
+      <c r="AJ33" s="7"/>
       <c r="AM33" s="7"/>
       <c r="AN33" s="7"/>
       <c r="AO33" s="7"/>
       <c r="AP33" s="7"/>
       <c r="AQ33" s="7"/>
-      <c r="AS33" s="7"/>
-      <c r="AU33" s="7"/>
-      <c r="AW33" s="7"/>
-      <c r="AY33" s="7"/>
-      <c r="BD33" s="7"/>
-      <c r="BI33" s="7"/>
-    </row>
-    <row r="34" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR33" s="7"/>
+      <c r="AT33" s="7"/>
+      <c r="AV33" s="7"/>
+      <c r="AX33" s="7"/>
+      <c r="AZ33" s="7"/>
+      <c r="BE33" s="7"/>
+      <c r="BJ33" s="7"/>
+    </row>
+    <row r="34" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>2011</v>
       </c>
@@ -3161,18 +3254,18 @@
         <v>1104</v>
       </c>
       <c r="E34" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>2033</v>
       </c>
       <c r="F34" s="11">
         <v>1694</v>
       </c>
       <c r="G34" s="14">
-        <f t="shared" si="6"/>
+        <f>ROUND(0.2*SUM(F34,H34,I34),0)</f>
         <v>339</v>
       </c>
       <c r="L34" s="7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>1694</v>
       </c>
       <c r="M34" s="23">
@@ -3188,39 +3281,42 @@
       <c r="P34" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q34" s="5"/>
+      <c r="Q34" s="7"/>
       <c r="R34" s="5"/>
-      <c r="S34" s="5"/>
-      <c r="T34" s="7"/>
+      <c r="S34" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="T34" s="5"/>
       <c r="U34" s="7"/>
       <c r="V34" s="7"/>
       <c r="W34" s="7"/>
       <c r="X34" s="7"/>
-      <c r="Y34" s="8"/>
+      <c r="Y34" s="7"/>
       <c r="Z34" s="8"/>
       <c r="AA34" s="8"/>
       <c r="AB34" s="8"/>
       <c r="AC34" s="8"/>
-      <c r="AD34" s="7"/>
+      <c r="AD34" s="8"/>
       <c r="AE34" s="7"/>
       <c r="AF34" s="7"/>
       <c r="AG34" s="7"/>
       <c r="AH34" s="7"/>
       <c r="AI34" s="7"/>
-      <c r="AL34" s="7"/>
+      <c r="AJ34" s="7"/>
       <c r="AM34" s="7"/>
       <c r="AN34" s="7"/>
       <c r="AO34" s="7"/>
       <c r="AP34" s="7"/>
       <c r="AQ34" s="7"/>
-      <c r="AS34" s="7"/>
-      <c r="AU34" s="7"/>
-      <c r="AW34" s="7"/>
-      <c r="AY34" s="7"/>
-      <c r="BD34" s="7"/>
-      <c r="BI34" s="7"/>
-    </row>
-    <row r="35" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR34" s="7"/>
+      <c r="AT34" s="7"/>
+      <c r="AV34" s="7"/>
+      <c r="AX34" s="7"/>
+      <c r="AZ34" s="7"/>
+      <c r="BE34" s="7"/>
+      <c r="BJ34" s="7"/>
+    </row>
+    <row r="35" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>2012</v>
       </c>
@@ -3235,12 +3331,12 @@
         <v>645</v>
       </c>
       <c r="E35" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>811</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="14">
-        <f t="shared" si="6"/>
+        <f>ROUND(0.2*SUM(F35,H35,I35),0)</f>
         <v>135</v>
       </c>
       <c r="H35" s="1">
@@ -3250,11 +3346,11 @@
         <v>255</v>
       </c>
       <c r="L35" s="7">
-        <f>SUM(F35,H35,I35)</f>
+        <f t="shared" si="5"/>
         <v>676</v>
       </c>
       <c r="M35" s="23">
-        <f t="shared" si="4"/>
+        <f>SUM(J35,K35)</f>
         <v>0</v>
       </c>
       <c r="N35" s="1">
@@ -3266,39 +3362,44 @@
       <c r="P35" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q35" s="5"/>
-      <c r="R35" s="5"/>
-      <c r="S35" s="5"/>
-      <c r="T35" s="7"/>
+      <c r="Q35" s="30"/>
+      <c r="R35" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="S35" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="T35" s="5"/>
       <c r="U35" s="7"/>
       <c r="V35" s="7"/>
       <c r="W35" s="7"/>
       <c r="X35" s="7"/>
-      <c r="Y35" s="8"/>
+      <c r="Y35" s="7"/>
       <c r="Z35" s="8"/>
       <c r="AA35" s="8"/>
       <c r="AB35" s="8"/>
       <c r="AC35" s="8"/>
-      <c r="AD35" s="7"/>
+      <c r="AD35" s="8"/>
       <c r="AE35" s="7"/>
       <c r="AF35" s="7"/>
       <c r="AG35" s="7"/>
       <c r="AH35" s="7"/>
       <c r="AI35" s="7"/>
-      <c r="AL35" s="7"/>
+      <c r="AJ35" s="7"/>
       <c r="AM35" s="7"/>
       <c r="AN35" s="7"/>
       <c r="AO35" s="7"/>
       <c r="AP35" s="7"/>
       <c r="AQ35" s="7"/>
-      <c r="AS35" s="7"/>
-      <c r="AU35" s="7"/>
-      <c r="AW35" s="7"/>
-      <c r="AY35" s="7"/>
-      <c r="BD35" s="7"/>
-      <c r="BI35" s="7"/>
-    </row>
-    <row r="36" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR35" s="7"/>
+      <c r="AT35" s="7"/>
+      <c r="AV35" s="7"/>
+      <c r="AX35" s="7"/>
+      <c r="AZ35" s="7"/>
+      <c r="BE35" s="7"/>
+      <c r="BJ35" s="7"/>
+    </row>
+    <row r="36" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>2013</v>
       </c>
@@ -3313,12 +3414,12 @@
         <v>642</v>
       </c>
       <c r="E36" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>2868</v>
       </c>
       <c r="F36" s="4"/>
       <c r="G36" s="14">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="G33:G40" si="7">ROUND(0.2*SUM(F36,H36,I36),0)</f>
         <v>478</v>
       </c>
       <c r="H36" s="1">
@@ -3338,7 +3439,7 @@
         <v>2390</v>
       </c>
       <c r="M36" s="23">
-        <f t="shared" si="4"/>
+        <f>SUM(J36,K36)</f>
         <v>958</v>
       </c>
       <c r="N36" s="1">
@@ -3350,39 +3451,44 @@
       <c r="P36" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q36" s="5"/>
-      <c r="R36" s="5"/>
-      <c r="S36" s="5"/>
-      <c r="T36" s="7"/>
+      <c r="Q36" s="30"/>
+      <c r="R36" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="S36" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="T36" s="5"/>
       <c r="U36" s="7"/>
       <c r="V36" s="7"/>
       <c r="W36" s="7"/>
       <c r="X36" s="7"/>
-      <c r="Y36" s="8"/>
+      <c r="Y36" s="7"/>
       <c r="Z36" s="8"/>
       <c r="AA36" s="8"/>
       <c r="AB36" s="8"/>
       <c r="AC36" s="8"/>
-      <c r="AD36" s="7"/>
+      <c r="AD36" s="8"/>
       <c r="AE36" s="7"/>
       <c r="AF36" s="7"/>
       <c r="AG36" s="7"/>
       <c r="AH36" s="7"/>
       <c r="AI36" s="7"/>
-      <c r="AL36" s="7"/>
+      <c r="AJ36" s="7"/>
       <c r="AM36" s="7"/>
       <c r="AN36" s="7"/>
       <c r="AO36" s="7"/>
       <c r="AP36" s="7"/>
       <c r="AQ36" s="7"/>
-      <c r="AS36" s="7"/>
-      <c r="AU36" s="7"/>
-      <c r="AW36" s="7"/>
-      <c r="AY36" s="7"/>
-      <c r="BD36" s="7"/>
-      <c r="BI36" s="7"/>
-    </row>
-    <row r="37" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR36" s="7"/>
+      <c r="AT36" s="7"/>
+      <c r="AV36" s="7"/>
+      <c r="AX36" s="7"/>
+      <c r="AZ36" s="7"/>
+      <c r="BE36" s="7"/>
+      <c r="BJ36" s="7"/>
+    </row>
+    <row r="37" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>2014</v>
       </c>
@@ -3397,12 +3503,12 @@
         <v>604</v>
       </c>
       <c r="E37" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>4638</v>
       </c>
       <c r="F37" s="4"/>
       <c r="G37" s="14">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>773</v>
       </c>
       <c r="H37" s="1">
@@ -3418,11 +3524,11 @@
         <v>250</v>
       </c>
       <c r="L37" s="7">
-        <f t="shared" si="3"/>
+        <f>SUM(F37,H37,I37)</f>
         <v>3865</v>
       </c>
       <c r="M37" s="23">
-        <f t="shared" si="4"/>
+        <f>SUM(J37,K37)</f>
         <v>428</v>
       </c>
       <c r="N37" s="1">
@@ -3434,39 +3540,44 @@
       <c r="P37" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q37" s="5"/>
-      <c r="R37" s="5"/>
-      <c r="S37" s="5"/>
-      <c r="T37" s="7"/>
+      <c r="Q37" s="30"/>
+      <c r="R37" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="S37" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="T37" s="5"/>
       <c r="U37" s="7"/>
       <c r="V37" s="7"/>
       <c r="W37" s="7"/>
       <c r="X37" s="7"/>
-      <c r="Y37" s="8"/>
+      <c r="Y37" s="7"/>
       <c r="Z37" s="8"/>
       <c r="AA37" s="8"/>
       <c r="AB37" s="8"/>
       <c r="AC37" s="8"/>
-      <c r="AD37" s="7"/>
+      <c r="AD37" s="8"/>
       <c r="AE37" s="7"/>
       <c r="AF37" s="7"/>
       <c r="AG37" s="7"/>
       <c r="AH37" s="7"/>
       <c r="AI37" s="7"/>
-      <c r="AL37" s="7"/>
+      <c r="AJ37" s="7"/>
       <c r="AM37" s="7"/>
       <c r="AN37" s="7"/>
       <c r="AO37" s="7"/>
       <c r="AP37" s="7"/>
       <c r="AQ37" s="7"/>
-      <c r="AS37" s="7"/>
-      <c r="AU37" s="7"/>
-      <c r="AW37" s="7"/>
-      <c r="AY37" s="7"/>
-      <c r="BD37" s="7"/>
-      <c r="BI37" s="7"/>
-    </row>
-    <row r="38" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR37" s="7"/>
+      <c r="AT37" s="7"/>
+      <c r="AV37" s="7"/>
+      <c r="AX37" s="7"/>
+      <c r="AZ37" s="7"/>
+      <c r="BE37" s="7"/>
+      <c r="BJ37" s="7"/>
+    </row>
+    <row r="38" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
         <v>2015</v>
       </c>
@@ -3481,12 +3592,12 @@
         <v>852</v>
       </c>
       <c r="E38" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>5897</v>
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="14">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>983</v>
       </c>
       <c r="H38" s="1">
@@ -3502,11 +3613,11 @@
         <v>103</v>
       </c>
       <c r="L38" s="7">
-        <f t="shared" si="3"/>
+        <f>SUM(F38,H38,I38)</f>
         <v>4914</v>
       </c>
       <c r="M38" s="23">
-        <f t="shared" si="4"/>
+        <f>SUM(J38,K38)</f>
         <v>584</v>
       </c>
       <c r="N38" s="1">
@@ -3518,39 +3629,44 @@
       <c r="P38" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q38" s="5"/>
-      <c r="R38" s="5"/>
-      <c r="S38" s="5"/>
-      <c r="T38" s="7"/>
+      <c r="Q38" s="30"/>
+      <c r="R38" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="S38" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="T38" s="5"/>
       <c r="U38" s="7"/>
       <c r="V38" s="7"/>
       <c r="W38" s="7"/>
       <c r="X38" s="7"/>
-      <c r="Y38" s="8"/>
+      <c r="Y38" s="7"/>
       <c r="Z38" s="8"/>
       <c r="AA38" s="8"/>
       <c r="AB38" s="8"/>
       <c r="AC38" s="8"/>
-      <c r="AD38" s="7"/>
+      <c r="AD38" s="8"/>
       <c r="AE38" s="7"/>
       <c r="AF38" s="7"/>
       <c r="AG38" s="7"/>
       <c r="AH38" s="7"/>
       <c r="AI38" s="7"/>
-      <c r="AL38" s="7"/>
+      <c r="AJ38" s="7"/>
       <c r="AM38" s="7"/>
       <c r="AN38" s="7"/>
       <c r="AO38" s="7"/>
       <c r="AP38" s="7"/>
       <c r="AQ38" s="7"/>
-      <c r="AS38" s="7"/>
-      <c r="AU38" s="7"/>
-      <c r="AW38" s="7"/>
-      <c r="AY38" s="7"/>
-      <c r="BD38" s="7"/>
-      <c r="BI38" s="7"/>
-    </row>
-    <row r="39" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR38" s="7"/>
+      <c r="AT38" s="7"/>
+      <c r="AV38" s="7"/>
+      <c r="AX38" s="7"/>
+      <c r="AZ38" s="7"/>
+      <c r="BE38" s="7"/>
+      <c r="BJ38" s="7"/>
+    </row>
+    <row r="39" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>2016</v>
       </c>
@@ -3565,12 +3681,12 @@
         <v>499</v>
       </c>
       <c r="E39" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>3876</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="14">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>646</v>
       </c>
       <c r="H39" s="1">
@@ -3590,7 +3706,7 @@
         <v>3230</v>
       </c>
       <c r="M39" s="23">
-        <f t="shared" si="4"/>
+        <f>SUM(J39,K39)</f>
         <v>1615</v>
       </c>
       <c r="N39" s="1">
@@ -3602,39 +3718,44 @@
       <c r="P39" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q39" s="5"/>
-      <c r="R39" s="5"/>
-      <c r="S39" s="5"/>
-      <c r="T39" s="7"/>
+      <c r="Q39" s="30"/>
+      <c r="R39" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="S39" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="T39" s="5"/>
       <c r="U39" s="7"/>
       <c r="V39" s="7"/>
       <c r="W39" s="7"/>
       <c r="X39" s="7"/>
-      <c r="Y39" s="8"/>
+      <c r="Y39" s="7"/>
       <c r="Z39" s="8"/>
       <c r="AA39" s="8"/>
       <c r="AB39" s="8"/>
       <c r="AC39" s="8"/>
-      <c r="AD39" s="7"/>
+      <c r="AD39" s="8"/>
       <c r="AE39" s="7"/>
       <c r="AF39" s="7"/>
       <c r="AG39" s="7"/>
       <c r="AH39" s="7"/>
       <c r="AI39" s="7"/>
-      <c r="AL39" s="7"/>
+      <c r="AJ39" s="7"/>
       <c r="AM39" s="7"/>
       <c r="AN39" s="7"/>
       <c r="AO39" s="7"/>
       <c r="AP39" s="7"/>
       <c r="AQ39" s="7"/>
-      <c r="AS39" s="7"/>
-      <c r="AU39" s="7"/>
-      <c r="AW39" s="7"/>
-      <c r="AY39" s="7"/>
-      <c r="BD39" s="7"/>
-      <c r="BI39" s="7"/>
-    </row>
-    <row r="40" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR39" s="7"/>
+      <c r="AT39" s="7"/>
+      <c r="AV39" s="7"/>
+      <c r="AX39" s="7"/>
+      <c r="AZ39" s="7"/>
+      <c r="BE39" s="7"/>
+      <c r="BJ39" s="7"/>
+    </row>
+    <row r="40" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>2017</v>
       </c>
@@ -3649,12 +3770,12 @@
         <v>538</v>
       </c>
       <c r="E40" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1488</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="14">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>248</v>
       </c>
       <c r="H40" s="1">
@@ -3664,18 +3785,20 @@
         <v>621</v>
       </c>
       <c r="J40" s="1">
-        <v>808</v>
+        <f>808-H40</f>
+        <v>189</v>
       </c>
       <c r="K40" s="1">
-        <v>1341</v>
+        <f>1341-I40</f>
+        <v>720</v>
       </c>
       <c r="L40" s="7">
-        <f t="shared" si="3"/>
+        <f>SUM(F40,H40,I40)</f>
         <v>1240</v>
       </c>
       <c r="M40" s="23">
-        <f t="shared" si="4"/>
-        <v>2149</v>
+        <f>SUM(J40,K40)</f>
+        <v>909</v>
       </c>
       <c r="N40" s="1">
         <v>239</v>
@@ -3686,39 +3809,46 @@
       <c r="P40" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q40" s="5"/>
-      <c r="R40" s="5"/>
-      <c r="S40" s="5"/>
-      <c r="T40" s="7"/>
+      <c r="Q40" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="R40" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="S40" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="T40" s="5"/>
       <c r="U40" s="7"/>
       <c r="V40" s="7"/>
       <c r="W40" s="7"/>
       <c r="X40" s="7"/>
-      <c r="Y40" s="8"/>
+      <c r="Y40" s="7"/>
       <c r="Z40" s="8"/>
       <c r="AA40" s="8"/>
       <c r="AB40" s="8"/>
       <c r="AC40" s="8"/>
-      <c r="AD40" s="7"/>
+      <c r="AD40" s="8"/>
       <c r="AE40" s="7"/>
       <c r="AF40" s="7"/>
       <c r="AG40" s="7"/>
       <c r="AH40" s="7"/>
       <c r="AI40" s="7"/>
-      <c r="AL40" s="7"/>
+      <c r="AJ40" s="7"/>
       <c r="AM40" s="7"/>
       <c r="AN40" s="7"/>
       <c r="AO40" s="7"/>
       <c r="AP40" s="7"/>
       <c r="AQ40" s="7"/>
-      <c r="AS40" s="7"/>
-      <c r="AU40" s="7"/>
-      <c r="AW40" s="7"/>
-      <c r="AY40" s="7"/>
-      <c r="BD40" s="7"/>
-      <c r="BI40" s="7"/>
-    </row>
-    <row r="41" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR40" s="7"/>
+      <c r="AT40" s="7"/>
+      <c r="AV40" s="7"/>
+      <c r="AX40" s="7"/>
+      <c r="AZ40" s="7"/>
+      <c r="BE40" s="7"/>
+      <c r="BJ40" s="7"/>
+    </row>
+    <row r="41" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
         <v>2018</v>
       </c>
@@ -3733,7 +3863,7 @@
         <v>530</v>
       </c>
       <c r="E41" s="11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="F41" s="4"/>
@@ -3757,7 +3887,7 @@
         <v>0</v>
       </c>
       <c r="M41" s="23">
-        <f t="shared" si="4"/>
+        <f>SUM(J41,K41)</f>
         <v>0</v>
       </c>
       <c r="N41" s="1">
@@ -3769,39 +3899,42 @@
       <c r="P41" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q41" s="5"/>
-      <c r="R41" s="5"/>
+      <c r="Q41" s="30"/>
+      <c r="R41" s="5" t="s">
+        <v>36</v>
+      </c>
       <c r="S41" s="5"/>
-      <c r="T41" s="7"/>
+      <c r="T41" s="5"/>
       <c r="U41" s="7"/>
       <c r="V41" s="7"/>
       <c r="W41" s="7"/>
       <c r="X41" s="7"/>
-      <c r="Y41" s="8"/>
+      <c r="Y41" s="7"/>
       <c r="Z41" s="8"/>
       <c r="AA41" s="8"/>
       <c r="AB41" s="8"/>
       <c r="AC41" s="8"/>
-      <c r="AD41" s="7"/>
+      <c r="AD41" s="8"/>
       <c r="AE41" s="7"/>
       <c r="AF41" s="7"/>
       <c r="AG41" s="7"/>
       <c r="AH41" s="7"/>
       <c r="AI41" s="7"/>
-      <c r="AL41" s="7"/>
+      <c r="AJ41" s="7"/>
       <c r="AM41" s="7"/>
       <c r="AN41" s="7"/>
       <c r="AO41" s="7"/>
       <c r="AP41" s="7"/>
       <c r="AQ41" s="7"/>
-      <c r="AS41" s="7"/>
-      <c r="AU41" s="7"/>
-      <c r="AW41" s="7"/>
-      <c r="AY41" s="7"/>
-      <c r="BD41" s="7"/>
-      <c r="BI41" s="7"/>
-    </row>
-    <row r="42" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR41" s="7"/>
+      <c r="AT41" s="7"/>
+      <c r="AV41" s="7"/>
+      <c r="AX41" s="7"/>
+      <c r="AZ41" s="7"/>
+      <c r="BE41" s="7"/>
+      <c r="BJ41" s="7"/>
+    </row>
+    <row r="42" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>2019</v>
       </c>
@@ -3816,7 +3949,7 @@
         <v>473</v>
       </c>
       <c r="E42" s="11">
-        <f t="shared" si="5"/>
+        <f>SUM(F42:I42)</f>
         <v>762</v>
       </c>
       <c r="F42" s="4"/>
@@ -3842,7 +3975,7 @@
         <v>762</v>
       </c>
       <c r="M42" s="23">
-        <f t="shared" si="4"/>
+        <f>SUM(J42,K42)</f>
         <v>141</v>
       </c>
       <c r="N42" s="1">
@@ -3854,39 +3987,44 @@
       <c r="P42" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q42" s="5"/>
-      <c r="R42" s="5"/>
+      <c r="Q42" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="R42" s="5" t="s">
+        <v>36</v>
+      </c>
       <c r="S42" s="5"/>
-      <c r="T42" s="7"/>
+      <c r="T42" s="5"/>
       <c r="U42" s="7"/>
       <c r="V42" s="7"/>
       <c r="W42" s="7"/>
       <c r="X42" s="7"/>
-      <c r="Y42" s="8"/>
+      <c r="Y42" s="7"/>
       <c r="Z42" s="8"/>
       <c r="AA42" s="8"/>
       <c r="AB42" s="8"/>
       <c r="AC42" s="8"/>
-      <c r="AD42" s="7"/>
+      <c r="AD42" s="8"/>
       <c r="AE42" s="7"/>
       <c r="AF42" s="7"/>
       <c r="AG42" s="7"/>
       <c r="AH42" s="7"/>
       <c r="AI42" s="7"/>
-      <c r="AL42" s="7"/>
+      <c r="AJ42" s="7"/>
       <c r="AM42" s="7"/>
       <c r="AN42" s="7"/>
       <c r="AO42" s="7"/>
       <c r="AP42" s="7"/>
       <c r="AQ42" s="7"/>
-      <c r="AS42" s="7"/>
-      <c r="AU42" s="7"/>
-      <c r="AW42" s="7"/>
-      <c r="AY42" s="7"/>
-      <c r="BD42" s="7"/>
-      <c r="BI42" s="7"/>
-    </row>
-    <row r="43" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR42" s="7"/>
+      <c r="AT42" s="7"/>
+      <c r="AV42" s="7"/>
+      <c r="AX42" s="7"/>
+      <c r="AZ42" s="7"/>
+      <c r="BE42" s="7"/>
+      <c r="BJ42" s="7"/>
+    </row>
+    <row r="43" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>2020</v>
       </c>
@@ -3901,34 +4039,34 @@
         <v>550</v>
       </c>
       <c r="E43" s="11">
-        <f t="shared" si="5"/>
-        <v>1072</v>
+        <f>SUM(F43:I43)</f>
+        <v>1073</v>
       </c>
       <c r="F43" s="4"/>
       <c r="G43" s="4">
         <v>0</v>
       </c>
       <c r="H43" s="1">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="I43" s="1">
         <v>538</v>
       </c>
       <c r="J43" s="1">
-        <f>604-H43</f>
+        <f>605-H43</f>
         <v>70</v>
       </c>
       <c r="K43" s="1">
-        <f>919-I43</f>
-        <v>381</v>
+        <f>920-I43</f>
+        <v>382</v>
       </c>
       <c r="L43" s="7">
         <f>SUM(F43,H43,I43)</f>
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="M43" s="23">
-        <f t="shared" si="4"/>
-        <v>451</v>
+        <f>SUM(J43,K43)</f>
+        <v>452</v>
       </c>
       <c r="N43" s="1">
         <v>329</v>
@@ -3939,39 +4077,44 @@
       <c r="P43" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q43" s="5"/>
-      <c r="R43" s="5"/>
+      <c r="Q43" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="R43" s="5" t="s">
+        <v>36</v>
+      </c>
       <c r="S43" s="5"/>
-      <c r="T43" s="7"/>
+      <c r="T43" s="5"/>
       <c r="U43" s="7"/>
       <c r="V43" s="7"/>
       <c r="W43" s="7"/>
       <c r="X43" s="7"/>
-      <c r="Y43" s="8"/>
+      <c r="Y43" s="7"/>
       <c r="Z43" s="8"/>
       <c r="AA43" s="8"/>
       <c r="AB43" s="8"/>
       <c r="AC43" s="8"/>
-      <c r="AD43" s="7"/>
+      <c r="AD43" s="8"/>
       <c r="AE43" s="7"/>
       <c r="AF43" s="7"/>
       <c r="AG43" s="7"/>
       <c r="AH43" s="7"/>
       <c r="AI43" s="7"/>
-      <c r="AL43" s="7"/>
+      <c r="AJ43" s="7"/>
       <c r="AM43" s="7"/>
       <c r="AN43" s="7"/>
       <c r="AO43" s="7"/>
       <c r="AP43" s="7"/>
       <c r="AQ43" s="7"/>
-      <c r="AS43" s="7"/>
-      <c r="AU43" s="7"/>
-      <c r="AW43" s="7"/>
-      <c r="AY43" s="7"/>
-      <c r="BD43" s="7"/>
-      <c r="BI43" s="7"/>
-    </row>
-    <row r="44" spans="1:61" ht="15" x14ac:dyDescent="0.25">
+      <c r="AR43" s="7"/>
+      <c r="AT43" s="7"/>
+      <c r="AV43" s="7"/>
+      <c r="AX43" s="7"/>
+      <c r="AZ43" s="7"/>
+      <c r="BE43" s="7"/>
+      <c r="BJ43" s="7"/>
+    </row>
+    <row r="44" spans="1:62" ht="15" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>2021</v>
       </c>
@@ -3984,59 +4127,81 @@
       <c r="D44" s="1">
         <v>482</v>
       </c>
-      <c r="E44" s="11"/>
+      <c r="E44" s="11">
+        <f>SUM(F44:I44)</f>
+        <v>0</v>
+      </c>
       <c r="F44" s="11"/>
       <c r="G44" s="1">
         <v>0</v>
       </c>
+      <c r="H44" s="1">
+        <v>0</v>
+      </c>
+      <c r="I44" s="1">
+        <v>0</v>
+      </c>
+      <c r="J44" s="1">
+        <f>0-H44</f>
+        <v>0</v>
+      </c>
+      <c r="K44" s="1">
+        <f>380-I44</f>
+        <v>380</v>
+      </c>
       <c r="L44" s="7">
-        <v>0</v>
-      </c>
-      <c r="M44" s="7">
-        <v>0</v>
-      </c>
-      <c r="N44" s="7">
-        <v>0</v>
-      </c>
+        <f t="shared" ref="L44:L48" si="8">SUM(F44,H44,I44)</f>
+        <v>0</v>
+      </c>
+      <c r="M44" s="23">
+        <f>SUM(J44,K44)</f>
+        <v>380</v>
+      </c>
+      <c r="N44" s="7"/>
       <c r="O44" s="29">
         <v>4192</v>
       </c>
       <c r="P44" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="Q44" s="5"/>
-      <c r="R44" s="5"/>
+      <c r="Q44" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="R44" s="5" t="s">
+        <v>36</v>
+      </c>
       <c r="S44" s="5"/>
-      <c r="T44" s="7"/>
+      <c r="T44" s="5"/>
       <c r="U44" s="7"/>
       <c r="V44" s="7"/>
       <c r="W44" s="7"/>
       <c r="X44" s="7"/>
-      <c r="Y44" s="8"/>
+      <c r="Y44" s="7"/>
       <c r="Z44" s="8"/>
       <c r="AA44" s="8"/>
       <c r="AB44" s="8"/>
       <c r="AC44" s="8"/>
-      <c r="AD44" s="7"/>
+      <c r="AD44" s="8"/>
       <c r="AE44" s="7"/>
       <c r="AF44" s="7"/>
       <c r="AG44" s="7"/>
       <c r="AH44" s="7"/>
       <c r="AI44" s="7"/>
-      <c r="AL44" s="7"/>
+      <c r="AJ44" s="7"/>
       <c r="AM44" s="7"/>
       <c r="AN44" s="7"/>
       <c r="AO44" s="7"/>
       <c r="AP44" s="7"/>
       <c r="AQ44" s="7"/>
-      <c r="AS44" s="7"/>
-      <c r="AU44" s="7"/>
-      <c r="AW44" s="7"/>
-      <c r="AY44" s="7"/>
-      <c r="BD44" s="7"/>
-      <c r="BI44" s="7"/>
-    </row>
-    <row r="45" spans="1:61" ht="15" x14ac:dyDescent="0.25">
+      <c r="AR44" s="7"/>
+      <c r="AT44" s="7"/>
+      <c r="AV44" s="7"/>
+      <c r="AX44" s="7"/>
+      <c r="AZ44" s="7"/>
+      <c r="BE44" s="7"/>
+      <c r="BJ44" s="7"/>
+    </row>
+    <row r="45" spans="1:62" ht="15" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>2022</v>
       </c>
@@ -4049,59 +4214,81 @@
       <c r="D45" s="1">
         <v>903</v>
       </c>
-      <c r="E45" s="11"/>
+      <c r="E45" s="11">
+        <f>SUM(F45:I45)</f>
+        <v>0</v>
+      </c>
       <c r="F45" s="11"/>
       <c r="G45" s="11">
         <v>0</v>
       </c>
-      <c r="L45" s="1">
-        <v>0</v>
-      </c>
-      <c r="M45" s="7">
-        <v>0</v>
-      </c>
-      <c r="N45" s="7">
-        <v>0</v>
-      </c>
+      <c r="H45" s="1">
+        <v>0</v>
+      </c>
+      <c r="I45" s="1">
+        <v>0</v>
+      </c>
+      <c r="J45" s="1">
+        <f>73-H45</f>
+        <v>73</v>
+      </c>
+      <c r="K45" s="1">
+        <f>274-I45</f>
+        <v>274</v>
+      </c>
+      <c r="L45" s="7">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="M45" s="23">
+        <f>SUM(J45,K45)</f>
+        <v>347</v>
+      </c>
+      <c r="N45" s="7"/>
       <c r="O45" s="29">
         <v>2959</v>
       </c>
       <c r="P45" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="Q45" s="5"/>
-      <c r="R45" s="5"/>
+      <c r="Q45" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="R45" s="5" t="s">
+        <v>36</v>
+      </c>
       <c r="S45" s="5"/>
-      <c r="T45" s="7"/>
+      <c r="T45" s="5"/>
       <c r="U45" s="7"/>
       <c r="V45" s="7"/>
       <c r="W45" s="7"/>
       <c r="X45" s="7"/>
-      <c r="Y45" s="8"/>
+      <c r="Y45" s="7"/>
       <c r="Z45" s="8"/>
       <c r="AA45" s="8"/>
       <c r="AB45" s="8"/>
       <c r="AC45" s="8"/>
-      <c r="AD45" s="7"/>
+      <c r="AD45" s="8"/>
       <c r="AE45" s="7"/>
       <c r="AF45" s="7"/>
       <c r="AG45" s="7"/>
       <c r="AH45" s="7"/>
       <c r="AI45" s="7"/>
-      <c r="AL45" s="7"/>
+      <c r="AJ45" s="7"/>
       <c r="AM45" s="7"/>
       <c r="AN45" s="7"/>
       <c r="AO45" s="7"/>
       <c r="AP45" s="7"/>
       <c r="AQ45" s="7"/>
-      <c r="AS45" s="7"/>
-      <c r="AU45" s="7"/>
-      <c r="AW45" s="7"/>
-      <c r="AY45" s="7"/>
-      <c r="BD45" s="7"/>
-      <c r="BI45" s="7"/>
-    </row>
-    <row r="46" spans="1:61" ht="15" x14ac:dyDescent="0.25">
+      <c r="AR45" s="7"/>
+      <c r="AT45" s="7"/>
+      <c r="AV45" s="7"/>
+      <c r="AX45" s="7"/>
+      <c r="AZ45" s="7"/>
+      <c r="BE45" s="7"/>
+      <c r="BJ45" s="7"/>
+    </row>
+    <row r="46" spans="1:62" ht="15" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>2023</v>
       </c>
@@ -4114,59 +4301,81 @@
       <c r="D46" s="1">
         <v>646</v>
       </c>
-      <c r="E46" s="11"/>
+      <c r="E46" s="11">
+        <f t="shared" ref="E46:E48" si="9">SUM(F46:I46)</f>
+        <v>71</v>
+      </c>
       <c r="F46" s="11"/>
       <c r="G46" s="11">
         <v>0</v>
       </c>
-      <c r="L46" s="1">
-        <v>0</v>
-      </c>
-      <c r="M46" s="7">
-        <v>0</v>
-      </c>
-      <c r="N46" s="7">
-        <v>0</v>
-      </c>
+      <c r="H46" s="1">
+        <v>71</v>
+      </c>
+      <c r="I46" s="1">
+        <v>0</v>
+      </c>
+      <c r="J46" s="1">
+        <f>277-H46</f>
+        <v>206</v>
+      </c>
+      <c r="K46" s="1">
+        <f>52-I46</f>
+        <v>52</v>
+      </c>
+      <c r="L46" s="7">
+        <f t="shared" si="8"/>
+        <v>71</v>
+      </c>
+      <c r="M46" s="23">
+        <f t="shared" si="4"/>
+        <v>258</v>
+      </c>
+      <c r="N46" s="7"/>
       <c r="O46" s="29">
         <v>3369</v>
       </c>
       <c r="P46" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="Q46" s="5"/>
-      <c r="R46" s="5"/>
+      <c r="Q46" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="R46" s="5" t="s">
+        <v>36</v>
+      </c>
       <c r="S46" s="5"/>
-      <c r="T46" s="7"/>
+      <c r="T46" s="5"/>
       <c r="U46" s="7"/>
       <c r="V46" s="7"/>
       <c r="W46" s="7"/>
       <c r="X46" s="7"/>
-      <c r="Y46" s="8"/>
+      <c r="Y46" s="7"/>
       <c r="Z46" s="8"/>
       <c r="AA46" s="8"/>
       <c r="AB46" s="8"/>
       <c r="AC46" s="8"/>
-      <c r="AD46" s="7"/>
+      <c r="AD46" s="8"/>
       <c r="AE46" s="7"/>
       <c r="AF46" s="7"/>
       <c r="AG46" s="7"/>
       <c r="AH46" s="7"/>
       <c r="AI46" s="7"/>
-      <c r="AL46" s="7"/>
+      <c r="AJ46" s="7"/>
       <c r="AM46" s="7"/>
       <c r="AN46" s="7"/>
       <c r="AO46" s="7"/>
       <c r="AP46" s="7"/>
       <c r="AQ46" s="7"/>
-      <c r="AS46" s="7"/>
-      <c r="AU46" s="7"/>
-      <c r="AW46" s="7"/>
-      <c r="AY46" s="7"/>
-      <c r="BD46" s="7"/>
-      <c r="BI46" s="7"/>
-    </row>
-    <row r="47" spans="1:61" ht="15" x14ac:dyDescent="0.25">
+      <c r="AR46" s="7"/>
+      <c r="AT46" s="7"/>
+      <c r="AV46" s="7"/>
+      <c r="AX46" s="7"/>
+      <c r="AZ46" s="7"/>
+      <c r="BE46" s="7"/>
+      <c r="BJ46" s="7"/>
+    </row>
+    <row r="47" spans="1:62" ht="15" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>2024</v>
       </c>
@@ -4179,65 +4388,117 @@
       <c r="D47" s="1">
         <v>482</v>
       </c>
-      <c r="E47" s="11"/>
+      <c r="E47" s="11">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
       <c r="F47" s="11"/>
       <c r="G47" s="11">
         <v>0</v>
       </c>
-      <c r="L47" s="1">
-        <v>0</v>
-      </c>
-      <c r="M47" s="7">
-        <v>0</v>
-      </c>
-      <c r="N47" s="7">
-        <v>0</v>
-      </c>
+      <c r="H47" s="1">
+        <v>1</v>
+      </c>
+      <c r="I47" s="1">
+        <v>0</v>
+      </c>
+      <c r="J47" s="1">
+        <f>17 - H47</f>
+        <v>16</v>
+      </c>
+      <c r="K47" s="1">
+        <f>2-I47</f>
+        <v>2</v>
+      </c>
+      <c r="L47" s="7">
+        <f t="shared" si="8"/>
+        <v>1</v>
+      </c>
+      <c r="M47" s="23">
+        <f t="shared" si="4"/>
+        <v>18</v>
+      </c>
+      <c r="N47" s="7"/>
       <c r="O47" s="29">
         <v>1860</v>
       </c>
       <c r="P47" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="Q47" s="5"/>
-      <c r="R47" s="5"/>
+      <c r="Q47" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="R47" s="5" t="s">
+        <v>36</v>
+      </c>
       <c r="S47" s="5"/>
-      <c r="T47" s="7"/>
+      <c r="T47" s="5"/>
       <c r="U47" s="7"/>
       <c r="V47" s="7"/>
       <c r="W47" s="7"/>
       <c r="X47" s="7"/>
-      <c r="Y47" s="8"/>
+      <c r="Y47" s="7"/>
       <c r="Z47" s="8"/>
       <c r="AA47" s="8"/>
       <c r="AB47" s="8"/>
       <c r="AC47" s="8"/>
-      <c r="AD47" s="7"/>
+      <c r="AD47" s="8"/>
       <c r="AE47" s="7"/>
       <c r="AF47" s="7"/>
       <c r="AG47" s="7"/>
       <c r="AH47" s="7"/>
       <c r="AI47" s="7"/>
-      <c r="AL47" s="7"/>
+      <c r="AJ47" s="7"/>
       <c r="AM47" s="7"/>
       <c r="AN47" s="7"/>
       <c r="AO47" s="7"/>
       <c r="AP47" s="7"/>
       <c r="AQ47" s="7"/>
-      <c r="AS47" s="7"/>
-      <c r="AU47" s="7"/>
-      <c r="AW47" s="7"/>
-      <c r="AY47" s="7"/>
-      <c r="BD47" s="7"/>
-      <c r="BI47" s="7"/>
-    </row>
-    <row r="48" spans="1:61" ht="15" x14ac:dyDescent="0.25">
+      <c r="AR47" s="7"/>
+      <c r="AT47" s="7"/>
+      <c r="AV47" s="7"/>
+      <c r="AX47" s="7"/>
+      <c r="AZ47" s="7"/>
+      <c r="BE47" s="7"/>
+      <c r="BJ47" s="7"/>
+    </row>
+    <row r="48" spans="1:62" ht="15" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>2025</v>
       </c>
+      <c r="B48" s="19"/>
+      <c r="C48" s="19"/>
+      <c r="D48" s="19"/>
+      <c r="E48" s="11">
+        <f t="shared" si="9"/>
+        <v>19</v>
+      </c>
       <c r="F48" s="4"/>
-      <c r="G48" s="4"/>
-      <c r="M48" s="7"/>
+      <c r="G48" s="4">
+        <v>0</v>
+      </c>
+      <c r="H48" s="1">
+        <v>14</v>
+      </c>
+      <c r="I48" s="1">
+        <v>5</v>
+      </c>
+      <c r="J48" s="1">
+        <f>105-H48</f>
+        <v>91</v>
+      </c>
+      <c r="K48" s="1">
+        <f>26-I48</f>
+        <v>21</v>
+      </c>
+      <c r="L48" s="7">
+        <f t="shared" si="8"/>
+        <v>19</v>
+      </c>
+      <c r="M48" s="23">
+        <f>SUM(J48,K48)</f>
+        <v>112</v>
+      </c>
       <c r="N48" s="7"/>
       <c r="O48">
         <v>3270</v>
@@ -4245,32 +4506,38 @@
       <c r="P48" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="R48" s="5"/>
+      <c r="Q48" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="R48" s="5" t="s">
+        <v>36</v>
+      </c>
       <c r="S48" s="5"/>
       <c r="T48" s="5"/>
       <c r="U48" s="5"/>
       <c r="V48" s="5"/>
       <c r="W48" s="5"/>
       <c r="X48" s="5"/>
-      <c r="Y48" s="8"/>
+      <c r="Y48" s="5"/>
       <c r="Z48" s="8"/>
       <c r="AA48" s="8"/>
       <c r="AB48" s="8"/>
       <c r="AC48" s="8"/>
-      <c r="AL48" s="7"/>
+      <c r="AD48" s="8"/>
       <c r="AM48" s="7"/>
       <c r="AN48" s="7"/>
       <c r="AO48" s="7"/>
       <c r="AP48" s="7"/>
       <c r="AQ48" s="7"/>
-      <c r="AS48" s="7"/>
-      <c r="AU48" s="7"/>
-      <c r="AW48" s="7"/>
-      <c r="AY48" s="7"/>
-      <c r="BD48" s="7"/>
-      <c r="BI48" s="7"/>
-    </row>
-    <row r="49" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR48" s="7"/>
+      <c r="AT48" s="7"/>
+      <c r="AV48" s="7"/>
+      <c r="AX48" s="7"/>
+      <c r="AZ48" s="7"/>
+      <c r="BE48" s="7"/>
+      <c r="BJ48" s="7"/>
+    </row>
+    <row r="49" spans="1:62" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>28</v>
       </c>
@@ -4285,151 +4552,153 @@
       <c r="N49" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="AL49" s="7"/>
+      <c r="R49" s="5"/>
       <c r="AM49" s="7"/>
       <c r="AN49" s="7"/>
       <c r="AO49" s="7"/>
       <c r="AP49" s="7"/>
       <c r="AQ49" s="7"/>
-      <c r="AS49" s="7"/>
-      <c r="AU49" s="7"/>
-      <c r="AW49" s="7"/>
-      <c r="AY49" s="7"/>
-      <c r="BD49" s="7"/>
-      <c r="BI49" s="7"/>
-    </row>
-    <row r="50" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR49" s="7"/>
+      <c r="AT49" s="7"/>
+      <c r="AV49" s="7"/>
+      <c r="AX49" s="7"/>
+      <c r="AZ49" s="7"/>
+      <c r="BE49" s="7"/>
+      <c r="BJ49" s="7"/>
+    </row>
+    <row r="50" spans="1:62" x14ac:dyDescent="0.2">
       <c r="E50" s="16" t="s">
         <v>18</v>
       </c>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
-      <c r="AL50" s="7"/>
+      <c r="R50" s="5"/>
       <c r="AM50" s="7"/>
       <c r="AN50" s="7"/>
       <c r="AO50" s="7"/>
       <c r="AP50" s="7"/>
       <c r="AQ50" s="7"/>
-      <c r="AS50" s="7"/>
-      <c r="AU50" s="7"/>
-      <c r="AW50" s="7"/>
-      <c r="AY50" s="7"/>
-      <c r="BD50" s="7"/>
-      <c r="BI50" s="7"/>
-    </row>
-    <row r="51" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR50" s="7"/>
+      <c r="AT50" s="7"/>
+      <c r="AV50" s="7"/>
+      <c r="AX50" s="7"/>
+      <c r="AZ50" s="7"/>
+      <c r="BE50" s="7"/>
+      <c r="BJ50" s="7"/>
+    </row>
+    <row r="51" spans="1:62" x14ac:dyDescent="0.2">
       <c r="B51" s="27"/>
       <c r="C51" s="27"/>
       <c r="D51" s="27"/>
       <c r="E51" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="AL51" s="7"/>
       <c r="AM51" s="7"/>
       <c r="AN51" s="7"/>
       <c r="AO51" s="7"/>
       <c r="AP51" s="7"/>
       <c r="AQ51" s="7"/>
-      <c r="AS51" s="7"/>
-      <c r="AU51" s="7"/>
-      <c r="AW51" s="7"/>
-      <c r="AY51" s="7"/>
-      <c r="BD51" s="7"/>
-      <c r="BI51" s="7"/>
-    </row>
-    <row r="52" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR51" s="7"/>
+      <c r="AT51" s="7"/>
+      <c r="AV51" s="7"/>
+      <c r="AX51" s="7"/>
+      <c r="AZ51" s="7"/>
+      <c r="BE51" s="7"/>
+      <c r="BJ51" s="7"/>
+    </row>
+    <row r="52" spans="1:62" x14ac:dyDescent="0.2">
       <c r="E52" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="AL52" s="7"/>
       <c r="AM52" s="7"/>
       <c r="AN52" s="7"/>
       <c r="AO52" s="7"/>
       <c r="AP52" s="7"/>
       <c r="AQ52" s="7"/>
-      <c r="AS52" s="7"/>
-      <c r="AU52" s="7"/>
-      <c r="AW52" s="7"/>
-      <c r="AY52" s="7"/>
-      <c r="BD52" s="7"/>
-      <c r="BI52" s="7"/>
-    </row>
-    <row r="53" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="AR52" s="7"/>
+      <c r="AT52" s="7"/>
+      <c r="AV52" s="7"/>
+      <c r="AX52" s="7"/>
+      <c r="AZ52" s="7"/>
+      <c r="BE52" s="7"/>
+      <c r="BJ52" s="7"/>
+    </row>
+    <row r="53" spans="1:62" x14ac:dyDescent="0.2">
       <c r="E53" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="BD53" s="7"/>
-      <c r="BI53" s="7"/>
-    </row>
-    <row r="54" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="BE53" s="7"/>
+      <c r="BJ53" s="7"/>
+    </row>
+    <row r="54" spans="1:62" x14ac:dyDescent="0.2">
       <c r="E54" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="BD54" s="7"/>
-      <c r="BI54" s="7"/>
-    </row>
-    <row r="55" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="BE54" s="7"/>
+      <c r="BJ54" s="7"/>
+    </row>
+    <row r="55" spans="1:62" x14ac:dyDescent="0.2">
       <c r="E55" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="BD55" s="7"/>
-      <c r="BI55" s="7"/>
-    </row>
-    <row r="56" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="BE55" s="7"/>
+      <c r="BJ55" s="7"/>
+    </row>
+    <row r="56" spans="1:62" x14ac:dyDescent="0.2">
       <c r="E56" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="BD56" s="7"/>
-      <c r="BI56" s="7"/>
-    </row>
-    <row r="57" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="BE56" s="7"/>
+      <c r="BJ56" s="7"/>
+    </row>
+    <row r="57" spans="1:62" x14ac:dyDescent="0.2">
       <c r="E57" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="BD57" s="7"/>
-      <c r="BI57" s="7"/>
-    </row>
-    <row r="58" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="BE57" s="7"/>
+      <c r="BJ57" s="7"/>
+    </row>
+    <row r="58" spans="1:62" x14ac:dyDescent="0.2">
       <c r="E58" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="BD58" s="7"/>
-      <c r="BI58" s="7"/>
-    </row>
-    <row r="59" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="BE58" s="7"/>
+      <c r="BJ58" s="7"/>
+    </row>
+    <row r="59" spans="1:62" x14ac:dyDescent="0.2">
       <c r="E59" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="BD59" s="7"/>
-      <c r="BI59" s="7"/>
-    </row>
-    <row r="60" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="BE59" s="7"/>
+      <c r="BJ59" s="7"/>
+    </row>
+    <row r="60" spans="1:62" x14ac:dyDescent="0.2">
       <c r="E60" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="BD60" s="7"/>
-      <c r="BI60" s="7"/>
-    </row>
-    <row r="61" spans="1:61" x14ac:dyDescent="0.2">
+      <c r="BE60" s="7"/>
+      <c r="BJ60" s="7"/>
+    </row>
+    <row r="61" spans="1:62" x14ac:dyDescent="0.2">
       <c r="E61" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="BD61" s="7"/>
-      <c r="BI61" s="7"/>
-    </row>
-    <row r="62" spans="1:61" x14ac:dyDescent="0.2">
-      <c r="BD62" s="7"/>
-      <c r="BI62" s="7"/>
-    </row>
-    <row r="63" spans="1:61" x14ac:dyDescent="0.2">
-      <c r="BD63" s="7"/>
-      <c r="BI63" s="7"/>
-    </row>
-    <row r="64" spans="1:61" x14ac:dyDescent="0.2">
-      <c r="BD64" s="7"/>
-      <c r="BI64" s="7"/>
-    </row>
-    <row r="65" spans="2:61" x14ac:dyDescent="0.2">
+      <c r="BE61" s="7"/>
+      <c r="BJ61" s="7"/>
+    </row>
+    <row r="62" spans="1:62" x14ac:dyDescent="0.2">
+      <c r="BE62" s="7"/>
+      <c r="BJ62" s="7"/>
+    </row>
+    <row r="63" spans="1:62" x14ac:dyDescent="0.2">
+      <c r="BE63" s="7"/>
+      <c r="BJ63" s="7"/>
+    </row>
+    <row r="64" spans="1:62" x14ac:dyDescent="0.2">
+      <c r="BE64" s="7"/>
+      <c r="BJ64" s="7"/>
+    </row>
+    <row r="65" spans="2:62" x14ac:dyDescent="0.2">
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
       <c r="D65" s="2"/>
@@ -4445,490 +4714,491 @@
       <c r="N65" s="2"/>
       <c r="O65" s="2"/>
       <c r="P65" s="2"/>
-      <c r="S65" s="3"/>
+      <c r="Q65" s="2"/>
       <c r="T65" s="3"/>
       <c r="U65" s="3"/>
-      <c r="W65" s="3"/>
-      <c r="AI65" s="3"/>
-    </row>
-    <row r="66" spans="2:61" x14ac:dyDescent="0.2">
-      <c r="BD66" s="7"/>
-      <c r="BI66" s="7"/>
-    </row>
-    <row r="67" spans="2:61" x14ac:dyDescent="0.2">
-      <c r="BD67" s="7"/>
-      <c r="BI67" s="7"/>
-    </row>
-    <row r="68" spans="2:61" x14ac:dyDescent="0.2">
-      <c r="BD68" s="7"/>
-      <c r="BI68" s="7"/>
-    </row>
-    <row r="69" spans="2:61" x14ac:dyDescent="0.2">
-      <c r="BD69" s="7"/>
-      <c r="BI69" s="7"/>
-    </row>
-    <row r="70" spans="2:61" x14ac:dyDescent="0.2">
-      <c r="BD70" s="7"/>
-      <c r="BI70" s="7"/>
-    </row>
-    <row r="71" spans="2:61" x14ac:dyDescent="0.2">
-      <c r="BD71" s="7"/>
-      <c r="BI71" s="7"/>
-    </row>
-    <row r="72" spans="2:61" x14ac:dyDescent="0.2">
-      <c r="BD72" s="7"/>
-      <c r="BI72" s="7"/>
-    </row>
-    <row r="73" spans="2:61" x14ac:dyDescent="0.2">
-      <c r="BD73" s="7"/>
-      <c r="BI73" s="7"/>
-    </row>
-    <row r="74" spans="2:61" x14ac:dyDescent="0.2">
-      <c r="BD74" s="7"/>
-      <c r="BI74" s="7"/>
-    </row>
-    <row r="75" spans="2:61" x14ac:dyDescent="0.2">
-      <c r="BD75" s="7"/>
-      <c r="BI75" s="7"/>
-    </row>
-    <row r="76" spans="2:61" x14ac:dyDescent="0.2">
-      <c r="BD76" s="7"/>
-      <c r="BI76" s="7"/>
-    </row>
-    <row r="77" spans="2:61" x14ac:dyDescent="0.2">
-      <c r="BD77" s="7"/>
-      <c r="BI77" s="7"/>
-    </row>
-    <row r="78" spans="2:61" x14ac:dyDescent="0.2">
-      <c r="BD78" s="7"/>
-      <c r="BI78" s="7"/>
-    </row>
-    <row r="79" spans="2:61" x14ac:dyDescent="0.2">
-      <c r="BD79" s="7"/>
-      <c r="BI79" s="7"/>
-    </row>
-    <row r="80" spans="2:61" x14ac:dyDescent="0.2">
-      <c r="BD80" s="7"/>
-      <c r="BI80" s="7"/>
-    </row>
-    <row r="81" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD81" s="7"/>
-      <c r="BI81" s="7"/>
-    </row>
-    <row r="82" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD82" s="7"/>
-      <c r="BI82" s="7"/>
-    </row>
-    <row r="83" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD83" s="7"/>
-      <c r="BI83" s="7"/>
-    </row>
-    <row r="84" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD84" s="7"/>
-      <c r="BI84" s="7"/>
-    </row>
-    <row r="85" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD85" s="7"/>
-      <c r="BI85" s="7"/>
-    </row>
-    <row r="86" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD86" s="7"/>
-      <c r="BI86" s="7"/>
-    </row>
-    <row r="87" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD87" s="7"/>
-      <c r="BI87" s="7"/>
-    </row>
-    <row r="88" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD88" s="7"/>
-      <c r="BI88" s="7"/>
-    </row>
-    <row r="89" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD89" s="7"/>
-      <c r="BI89" s="7"/>
-    </row>
-    <row r="90" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD90" s="7"/>
-      <c r="BI90" s="7"/>
-    </row>
-    <row r="91" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD91" s="7"/>
-      <c r="BI91" s="7"/>
-    </row>
-    <row r="92" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD92" s="7"/>
-      <c r="BI92" s="7"/>
-    </row>
-    <row r="93" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD93" s="7"/>
-      <c r="BI93" s="7"/>
-    </row>
-    <row r="94" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD94" s="7"/>
-      <c r="BI94" s="7"/>
-    </row>
-    <row r="95" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD95" s="7"/>
-      <c r="BI95" s="7"/>
-    </row>
-    <row r="96" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD96" s="7"/>
-      <c r="BI96" s="7"/>
-    </row>
-    <row r="97" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD97" s="7"/>
-      <c r="BI97" s="7"/>
-    </row>
-    <row r="98" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD98" s="7"/>
-      <c r="BI98" s="7"/>
-    </row>
-    <row r="99" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD99" s="7"/>
-      <c r="BI99" s="7"/>
-    </row>
-    <row r="100" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD100" s="7"/>
-      <c r="BI100" s="7"/>
-    </row>
-    <row r="101" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD101" s="7"/>
-      <c r="BI101" s="7"/>
-    </row>
-    <row r="102" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD102" s="7"/>
-      <c r="BI102" s="7"/>
-    </row>
-    <row r="103" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD103" s="7"/>
-      <c r="BI103" s="7"/>
-    </row>
-    <row r="104" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD104" s="7"/>
-      <c r="BI104" s="7"/>
-    </row>
-    <row r="105" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD105" s="7"/>
-      <c r="BI105" s="7"/>
-    </row>
-    <row r="106" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD106" s="7"/>
-      <c r="BI106" s="7"/>
-    </row>
-    <row r="107" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD107" s="7"/>
-      <c r="BI107" s="7"/>
-    </row>
-    <row r="108" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD108" s="7"/>
-      <c r="BI108" s="7"/>
-    </row>
-    <row r="109" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD109" s="7"/>
-      <c r="BI109" s="7"/>
-    </row>
-    <row r="110" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD110" s="7"/>
-      <c r="BI110" s="7"/>
-    </row>
-    <row r="111" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD111" s="7"/>
-      <c r="BI111" s="7"/>
-    </row>
-    <row r="112" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD112" s="7"/>
-      <c r="BI112" s="7"/>
-    </row>
-    <row r="113" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD113" s="7"/>
-      <c r="BI113" s="7"/>
-    </row>
-    <row r="114" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD114" s="7"/>
-      <c r="BI114" s="7"/>
-    </row>
-    <row r="115" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD115" s="7"/>
-      <c r="BI115" s="7"/>
-    </row>
-    <row r="116" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD116" s="7"/>
-      <c r="BI116" s="7"/>
-    </row>
-    <row r="117" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD117" s="7"/>
-      <c r="BI117" s="7"/>
-    </row>
-    <row r="118" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD118" s="7"/>
-      <c r="BI118" s="7"/>
-    </row>
-    <row r="119" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD119" s="7"/>
-      <c r="BI119" s="7"/>
-    </row>
-    <row r="120" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD120" s="7"/>
-      <c r="BI120" s="7"/>
-    </row>
-    <row r="121" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD121" s="7"/>
-      <c r="BI121" s="7"/>
-    </row>
-    <row r="122" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD122" s="7"/>
-      <c r="BI122" s="7"/>
-    </row>
-    <row r="123" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD123" s="7"/>
-      <c r="BI123" s="7"/>
-    </row>
-    <row r="124" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD124" s="7"/>
-      <c r="BI124" s="7"/>
-    </row>
-    <row r="125" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD125" s="7"/>
-      <c r="BI125" s="7"/>
-    </row>
-    <row r="126" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD126" s="7"/>
-      <c r="BI126" s="7"/>
-    </row>
-    <row r="127" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD127" s="7"/>
-      <c r="BI127" s="7"/>
-    </row>
-    <row r="128" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD128" s="7"/>
-      <c r="BI128" s="7"/>
-    </row>
-    <row r="129" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD129" s="7"/>
-      <c r="BI129" s="7"/>
-    </row>
-    <row r="130" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD130" s="7"/>
-      <c r="BI130" s="7"/>
-    </row>
-    <row r="131" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD131" s="7"/>
-      <c r="BI131" s="7"/>
-    </row>
-    <row r="132" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD132" s="7"/>
-      <c r="BI132" s="7"/>
-    </row>
-    <row r="133" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD133" s="7"/>
-      <c r="BI133" s="7"/>
-    </row>
-    <row r="134" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD134" s="7"/>
-      <c r="BI134" s="7"/>
-    </row>
-    <row r="135" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD135" s="7"/>
-      <c r="BI135" s="7"/>
-    </row>
-    <row r="136" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD136" s="7"/>
-      <c r="BI136" s="7"/>
-    </row>
-    <row r="137" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD137" s="7"/>
-      <c r="BI137" s="7"/>
-    </row>
-    <row r="138" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD138" s="7"/>
-      <c r="BI138" s="7"/>
-    </row>
-    <row r="139" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD139" s="7"/>
-      <c r="BI139" s="7"/>
-    </row>
-    <row r="140" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD140" s="7"/>
-      <c r="BI140" s="7"/>
-    </row>
-    <row r="141" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD141" s="7"/>
-      <c r="BI141" s="7"/>
-    </row>
-    <row r="142" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD142" s="7"/>
-      <c r="BI142" s="7"/>
-    </row>
-    <row r="143" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD143" s="7"/>
-      <c r="BI143" s="7"/>
-    </row>
-    <row r="144" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD144" s="7"/>
-      <c r="BI144" s="7"/>
-    </row>
-    <row r="145" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD145" s="7"/>
-      <c r="BI145" s="7"/>
-    </row>
-    <row r="146" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD146" s="7"/>
-      <c r="BI146" s="7"/>
-    </row>
-    <row r="147" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD147" s="7"/>
-      <c r="BI147" s="7"/>
-    </row>
-    <row r="148" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD148" s="7"/>
-      <c r="BI148" s="7"/>
-    </row>
-    <row r="149" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD149" s="7"/>
-      <c r="BI149" s="7"/>
-    </row>
-    <row r="150" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD150" s="7"/>
-      <c r="BI150" s="7"/>
-    </row>
-    <row r="151" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD151" s="7"/>
-      <c r="BI151" s="7"/>
-    </row>
-    <row r="152" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD152" s="7"/>
-      <c r="BI152" s="7"/>
-    </row>
-    <row r="153" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD153" s="7"/>
-      <c r="BI153" s="7"/>
-    </row>
-    <row r="154" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD154" s="7"/>
-      <c r="BI154" s="7"/>
-    </row>
-    <row r="155" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD155" s="7"/>
-      <c r="BI155" s="7"/>
-    </row>
-    <row r="156" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD156" s="7"/>
-      <c r="BI156" s="7"/>
-    </row>
-    <row r="157" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD157" s="7"/>
-      <c r="BI157" s="7"/>
-    </row>
-    <row r="158" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD158" s="7"/>
-      <c r="BI158" s="7"/>
-    </row>
-    <row r="159" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD159" s="7"/>
-      <c r="BI159" s="7"/>
-    </row>
-    <row r="160" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD160" s="7"/>
-      <c r="BI160" s="7"/>
-    </row>
-    <row r="161" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD161" s="7"/>
-      <c r="BI161" s="7"/>
-    </row>
-    <row r="162" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD162" s="7"/>
-      <c r="BI162" s="7"/>
-    </row>
-    <row r="163" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD163" s="7"/>
-      <c r="BI163" s="7"/>
-    </row>
-    <row r="164" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD164" s="7"/>
-      <c r="BI164" s="7"/>
-    </row>
-    <row r="165" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD165" s="7"/>
-      <c r="BI165" s="7"/>
-    </row>
-    <row r="166" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD166" s="7"/>
-      <c r="BI166" s="7"/>
-    </row>
-    <row r="167" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD167" s="7"/>
-      <c r="BI167" s="7"/>
-    </row>
-    <row r="168" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD168" s="7"/>
-      <c r="BI168" s="7"/>
-    </row>
-    <row r="169" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD169" s="7"/>
-      <c r="BI169" s="7"/>
-    </row>
-    <row r="170" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD170" s="7"/>
-    </row>
-    <row r="171" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD171" s="7"/>
-    </row>
-    <row r="172" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD172" s="7"/>
-    </row>
-    <row r="173" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD173" s="7"/>
-    </row>
-    <row r="174" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD174" s="7"/>
-    </row>
-    <row r="175" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD175" s="7"/>
-    </row>
-    <row r="176" spans="56:61" x14ac:dyDescent="0.2">
-      <c r="BD176" s="7"/>
-    </row>
-    <row r="177" spans="56:56" x14ac:dyDescent="0.2">
-      <c r="BD177" s="7"/>
-    </row>
-    <row r="178" spans="56:56" x14ac:dyDescent="0.2">
-      <c r="BD178" s="7"/>
-    </row>
-    <row r="179" spans="56:56" x14ac:dyDescent="0.2">
-      <c r="BD179" s="7"/>
-    </row>
-    <row r="180" spans="56:56" x14ac:dyDescent="0.2">
-      <c r="BD180" s="7"/>
-    </row>
-    <row r="181" spans="56:56" x14ac:dyDescent="0.2">
-      <c r="BD181" s="7"/>
-    </row>
-    <row r="182" spans="56:56" x14ac:dyDescent="0.2">
-      <c r="BD182" s="7"/>
-    </row>
-    <row r="183" spans="56:56" x14ac:dyDescent="0.2">
-      <c r="BD183" s="7"/>
-    </row>
-    <row r="184" spans="56:56" x14ac:dyDescent="0.2">
-      <c r="BD184" s="7"/>
-    </row>
-    <row r="185" spans="56:56" x14ac:dyDescent="0.2">
-      <c r="BD185" s="7"/>
-    </row>
-    <row r="186" spans="56:56" x14ac:dyDescent="0.2">
-      <c r="BD186" s="7"/>
-    </row>
-    <row r="187" spans="56:56" x14ac:dyDescent="0.2">
-      <c r="BD187" s="7"/>
-    </row>
-    <row r="188" spans="56:56" x14ac:dyDescent="0.2">
-      <c r="BD188" s="7"/>
-    </row>
-    <row r="189" spans="56:56" x14ac:dyDescent="0.2">
-      <c r="BD189" s="7"/>
-    </row>
-    <row r="190" spans="56:56" x14ac:dyDescent="0.2">
-      <c r="BD190" s="7"/>
+      <c r="V65" s="3"/>
+      <c r="X65" s="3"/>
+      <c r="AJ65" s="3"/>
+    </row>
+    <row r="66" spans="2:62" x14ac:dyDescent="0.2">
+      <c r="BE66" s="7"/>
+      <c r="BJ66" s="7"/>
+    </row>
+    <row r="67" spans="2:62" x14ac:dyDescent="0.2">
+      <c r="BE67" s="7"/>
+      <c r="BJ67" s="7"/>
+    </row>
+    <row r="68" spans="2:62" x14ac:dyDescent="0.2">
+      <c r="BE68" s="7"/>
+      <c r="BJ68" s="7"/>
+    </row>
+    <row r="69" spans="2:62" x14ac:dyDescent="0.2">
+      <c r="BE69" s="7"/>
+      <c r="BJ69" s="7"/>
+    </row>
+    <row r="70" spans="2:62" x14ac:dyDescent="0.2">
+      <c r="BE70" s="7"/>
+      <c r="BJ70" s="7"/>
+    </row>
+    <row r="71" spans="2:62" x14ac:dyDescent="0.2">
+      <c r="BE71" s="7"/>
+      <c r="BJ71" s="7"/>
+    </row>
+    <row r="72" spans="2:62" x14ac:dyDescent="0.2">
+      <c r="BE72" s="7"/>
+      <c r="BJ72" s="7"/>
+    </row>
+    <row r="73" spans="2:62" x14ac:dyDescent="0.2">
+      <c r="BE73" s="7"/>
+      <c r="BJ73" s="7"/>
+    </row>
+    <row r="74" spans="2:62" x14ac:dyDescent="0.2">
+      <c r="BE74" s="7"/>
+      <c r="BJ74" s="7"/>
+    </row>
+    <row r="75" spans="2:62" x14ac:dyDescent="0.2">
+      <c r="BE75" s="7"/>
+      <c r="BJ75" s="7"/>
+    </row>
+    <row r="76" spans="2:62" x14ac:dyDescent="0.2">
+      <c r="BE76" s="7"/>
+      <c r="BJ76" s="7"/>
+    </row>
+    <row r="77" spans="2:62" x14ac:dyDescent="0.2">
+      <c r="BE77" s="7"/>
+      <c r="BJ77" s="7"/>
+    </row>
+    <row r="78" spans="2:62" x14ac:dyDescent="0.2">
+      <c r="BE78" s="7"/>
+      <c r="BJ78" s="7"/>
+    </row>
+    <row r="79" spans="2:62" x14ac:dyDescent="0.2">
+      <c r="BE79" s="7"/>
+      <c r="BJ79" s="7"/>
+    </row>
+    <row r="80" spans="2:62" x14ac:dyDescent="0.2">
+      <c r="BE80" s="7"/>
+      <c r="BJ80" s="7"/>
+    </row>
+    <row r="81" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE81" s="7"/>
+      <c r="BJ81" s="7"/>
+    </row>
+    <row r="82" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE82" s="7"/>
+      <c r="BJ82" s="7"/>
+    </row>
+    <row r="83" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE83" s="7"/>
+      <c r="BJ83" s="7"/>
+    </row>
+    <row r="84" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE84" s="7"/>
+      <c r="BJ84" s="7"/>
+    </row>
+    <row r="85" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE85" s="7"/>
+      <c r="BJ85" s="7"/>
+    </row>
+    <row r="86" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE86" s="7"/>
+      <c r="BJ86" s="7"/>
+    </row>
+    <row r="87" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE87" s="7"/>
+      <c r="BJ87" s="7"/>
+    </row>
+    <row r="88" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE88" s="7"/>
+      <c r="BJ88" s="7"/>
+    </row>
+    <row r="89" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE89" s="7"/>
+      <c r="BJ89" s="7"/>
+    </row>
+    <row r="90" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE90" s="7"/>
+      <c r="BJ90" s="7"/>
+    </row>
+    <row r="91" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE91" s="7"/>
+      <c r="BJ91" s="7"/>
+    </row>
+    <row r="92" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE92" s="7"/>
+      <c r="BJ92" s="7"/>
+    </row>
+    <row r="93" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE93" s="7"/>
+      <c r="BJ93" s="7"/>
+    </row>
+    <row r="94" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE94" s="7"/>
+      <c r="BJ94" s="7"/>
+    </row>
+    <row r="95" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE95" s="7"/>
+      <c r="BJ95" s="7"/>
+    </row>
+    <row r="96" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE96" s="7"/>
+      <c r="BJ96" s="7"/>
+    </row>
+    <row r="97" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE97" s="7"/>
+      <c r="BJ97" s="7"/>
+    </row>
+    <row r="98" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE98" s="7"/>
+      <c r="BJ98" s="7"/>
+    </row>
+    <row r="99" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE99" s="7"/>
+      <c r="BJ99" s="7"/>
+    </row>
+    <row r="100" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE100" s="7"/>
+      <c r="BJ100" s="7"/>
+    </row>
+    <row r="101" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE101" s="7"/>
+      <c r="BJ101" s="7"/>
+    </row>
+    <row r="102" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE102" s="7"/>
+      <c r="BJ102" s="7"/>
+    </row>
+    <row r="103" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE103" s="7"/>
+      <c r="BJ103" s="7"/>
+    </row>
+    <row r="104" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE104" s="7"/>
+      <c r="BJ104" s="7"/>
+    </row>
+    <row r="105" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE105" s="7"/>
+      <c r="BJ105" s="7"/>
+    </row>
+    <row r="106" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE106" s="7"/>
+      <c r="BJ106" s="7"/>
+    </row>
+    <row r="107" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE107" s="7"/>
+      <c r="BJ107" s="7"/>
+    </row>
+    <row r="108" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE108" s="7"/>
+      <c r="BJ108" s="7"/>
+    </row>
+    <row r="109" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE109" s="7"/>
+      <c r="BJ109" s="7"/>
+    </row>
+    <row r="110" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE110" s="7"/>
+      <c r="BJ110" s="7"/>
+    </row>
+    <row r="111" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE111" s="7"/>
+      <c r="BJ111" s="7"/>
+    </row>
+    <row r="112" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE112" s="7"/>
+      <c r="BJ112" s="7"/>
+    </row>
+    <row r="113" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE113" s="7"/>
+      <c r="BJ113" s="7"/>
+    </row>
+    <row r="114" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE114" s="7"/>
+      <c r="BJ114" s="7"/>
+    </row>
+    <row r="115" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE115" s="7"/>
+      <c r="BJ115" s="7"/>
+    </row>
+    <row r="116" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE116" s="7"/>
+      <c r="BJ116" s="7"/>
+    </row>
+    <row r="117" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE117" s="7"/>
+      <c r="BJ117" s="7"/>
+    </row>
+    <row r="118" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE118" s="7"/>
+      <c r="BJ118" s="7"/>
+    </row>
+    <row r="119" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE119" s="7"/>
+      <c r="BJ119" s="7"/>
+    </row>
+    <row r="120" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE120" s="7"/>
+      <c r="BJ120" s="7"/>
+    </row>
+    <row r="121" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE121" s="7"/>
+      <c r="BJ121" s="7"/>
+    </row>
+    <row r="122" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE122" s="7"/>
+      <c r="BJ122" s="7"/>
+    </row>
+    <row r="123" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE123" s="7"/>
+      <c r="BJ123" s="7"/>
+    </row>
+    <row r="124" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE124" s="7"/>
+      <c r="BJ124" s="7"/>
+    </row>
+    <row r="125" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE125" s="7"/>
+      <c r="BJ125" s="7"/>
+    </row>
+    <row r="126" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE126" s="7"/>
+      <c r="BJ126" s="7"/>
+    </row>
+    <row r="127" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE127" s="7"/>
+      <c r="BJ127" s="7"/>
+    </row>
+    <row r="128" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE128" s="7"/>
+      <c r="BJ128" s="7"/>
+    </row>
+    <row r="129" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE129" s="7"/>
+      <c r="BJ129" s="7"/>
+    </row>
+    <row r="130" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE130" s="7"/>
+      <c r="BJ130" s="7"/>
+    </row>
+    <row r="131" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE131" s="7"/>
+      <c r="BJ131" s="7"/>
+    </row>
+    <row r="132" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE132" s="7"/>
+      <c r="BJ132" s="7"/>
+    </row>
+    <row r="133" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE133" s="7"/>
+      <c r="BJ133" s="7"/>
+    </row>
+    <row r="134" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE134" s="7"/>
+      <c r="BJ134" s="7"/>
+    </row>
+    <row r="135" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE135" s="7"/>
+      <c r="BJ135" s="7"/>
+    </row>
+    <row r="136" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE136" s="7"/>
+      <c r="BJ136" s="7"/>
+    </row>
+    <row r="137" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE137" s="7"/>
+      <c r="BJ137" s="7"/>
+    </row>
+    <row r="138" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE138" s="7"/>
+      <c r="BJ138" s="7"/>
+    </row>
+    <row r="139" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE139" s="7"/>
+      <c r="BJ139" s="7"/>
+    </row>
+    <row r="140" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE140" s="7"/>
+      <c r="BJ140" s="7"/>
+    </row>
+    <row r="141" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE141" s="7"/>
+      <c r="BJ141" s="7"/>
+    </row>
+    <row r="142" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE142" s="7"/>
+      <c r="BJ142" s="7"/>
+    </row>
+    <row r="143" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE143" s="7"/>
+      <c r="BJ143" s="7"/>
+    </row>
+    <row r="144" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE144" s="7"/>
+      <c r="BJ144" s="7"/>
+    </row>
+    <row r="145" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE145" s="7"/>
+      <c r="BJ145" s="7"/>
+    </row>
+    <row r="146" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE146" s="7"/>
+      <c r="BJ146" s="7"/>
+    </row>
+    <row r="147" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE147" s="7"/>
+      <c r="BJ147" s="7"/>
+    </row>
+    <row r="148" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE148" s="7"/>
+      <c r="BJ148" s="7"/>
+    </row>
+    <row r="149" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE149" s="7"/>
+      <c r="BJ149" s="7"/>
+    </row>
+    <row r="150" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE150" s="7"/>
+      <c r="BJ150" s="7"/>
+    </row>
+    <row r="151" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE151" s="7"/>
+      <c r="BJ151" s="7"/>
+    </row>
+    <row r="152" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE152" s="7"/>
+      <c r="BJ152" s="7"/>
+    </row>
+    <row r="153" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE153" s="7"/>
+      <c r="BJ153" s="7"/>
+    </row>
+    <row r="154" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE154" s="7"/>
+      <c r="BJ154" s="7"/>
+    </row>
+    <row r="155" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE155" s="7"/>
+      <c r="BJ155" s="7"/>
+    </row>
+    <row r="156" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE156" s="7"/>
+      <c r="BJ156" s="7"/>
+    </row>
+    <row r="157" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE157" s="7"/>
+      <c r="BJ157" s="7"/>
+    </row>
+    <row r="158" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE158" s="7"/>
+      <c r="BJ158" s="7"/>
+    </row>
+    <row r="159" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE159" s="7"/>
+      <c r="BJ159" s="7"/>
+    </row>
+    <row r="160" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE160" s="7"/>
+      <c r="BJ160" s="7"/>
+    </row>
+    <row r="161" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE161" s="7"/>
+      <c r="BJ161" s="7"/>
+    </row>
+    <row r="162" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE162" s="7"/>
+      <c r="BJ162" s="7"/>
+    </row>
+    <row r="163" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE163" s="7"/>
+      <c r="BJ163" s="7"/>
+    </row>
+    <row r="164" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE164" s="7"/>
+      <c r="BJ164" s="7"/>
+    </row>
+    <row r="165" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE165" s="7"/>
+      <c r="BJ165" s="7"/>
+    </row>
+    <row r="166" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE166" s="7"/>
+      <c r="BJ166" s="7"/>
+    </row>
+    <row r="167" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE167" s="7"/>
+      <c r="BJ167" s="7"/>
+    </row>
+    <row r="168" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE168" s="7"/>
+      <c r="BJ168" s="7"/>
+    </row>
+    <row r="169" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE169" s="7"/>
+      <c r="BJ169" s="7"/>
+    </row>
+    <row r="170" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE170" s="7"/>
+    </row>
+    <row r="171" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE171" s="7"/>
+    </row>
+    <row r="172" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE172" s="7"/>
+    </row>
+    <row r="173" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE173" s="7"/>
+    </row>
+    <row r="174" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE174" s="7"/>
+    </row>
+    <row r="175" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE175" s="7"/>
+    </row>
+    <row r="176" spans="57:62" x14ac:dyDescent="0.2">
+      <c r="BE176" s="7"/>
+    </row>
+    <row r="177" spans="57:57" x14ac:dyDescent="0.2">
+      <c r="BE177" s="7"/>
+    </row>
+    <row r="178" spans="57:57" x14ac:dyDescent="0.2">
+      <c r="BE178" s="7"/>
+    </row>
+    <row r="179" spans="57:57" x14ac:dyDescent="0.2">
+      <c r="BE179" s="7"/>
+    </row>
+    <row r="180" spans="57:57" x14ac:dyDescent="0.2">
+      <c r="BE180" s="7"/>
+    </row>
+    <row r="181" spans="57:57" x14ac:dyDescent="0.2">
+      <c r="BE181" s="7"/>
+    </row>
+    <row r="182" spans="57:57" x14ac:dyDescent="0.2">
+      <c r="BE182" s="7"/>
+    </row>
+    <row r="183" spans="57:57" x14ac:dyDescent="0.2">
+      <c r="BE183" s="7"/>
+    </row>
+    <row r="184" spans="57:57" x14ac:dyDescent="0.2">
+      <c r="BE184" s="7"/>
+    </row>
+    <row r="185" spans="57:57" x14ac:dyDescent="0.2">
+      <c r="BE185" s="7"/>
+    </row>
+    <row r="186" spans="57:57" x14ac:dyDescent="0.2">
+      <c r="BE186" s="7"/>
+    </row>
+    <row r="187" spans="57:57" x14ac:dyDescent="0.2">
+      <c r="BE187" s="7"/>
+    </row>
+    <row r="188" spans="57:57" x14ac:dyDescent="0.2">
+      <c r="BE188" s="7"/>
+    </row>
+    <row r="189" spans="57:57" x14ac:dyDescent="0.2">
+      <c r="BE189" s="7"/>
+    </row>
+    <row r="190" spans="57:57" x14ac:dyDescent="0.2">
+      <c r="BE190" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update freshwater catch data, fig of spawners and total run
</commit_message>
<xml_diff>
--- a/data-raw/freshwater-catch.xlsx
+++ b/data-raw/freshwater-catch.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\skrunchy2025\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE37A6E9-11DD-42FC-A3FF-3D8249269507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1649AC2B-2634-4801-9A7A-60FFFF04D40F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E0CDEE87-6CC2-4107-81B9-F1AD4EA649A7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="48">
   <si>
     <t>Year</t>
   </si>
@@ -302,7 +302,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -361,7 +361,18 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="3" fontId="2" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -690,7 +701,7 @@
     <col min="13" max="13" width="8.42578125" style="19" customWidth="1"/>
     <col min="14" max="15" width="7.5703125" style="1" customWidth="1"/>
     <col min="16" max="16" width="34.42578125" style="1" customWidth="1"/>
-    <col min="17" max="17" width="33.42578125" style="1" customWidth="1"/>
+    <col min="17" max="17" width="33.42578125" style="3" customWidth="1"/>
     <col min="18" max="18" width="32.5703125" style="1" customWidth="1"/>
     <col min="19" max="19" width="24.140625" style="1" customWidth="1"/>
     <col min="20" max="23" width="7.5703125" style="1" customWidth="1"/>
@@ -814,7 +825,7 @@
       <c r="BD1" s="19"/>
       <c r="BE1" s="1"/>
     </row>
-    <row r="2" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>1979</v>
       </c>
@@ -860,7 +871,9 @@
       <c r="P2" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q2" s="7"/>
+      <c r="Q2" s="30" t="s">
+        <v>27</v>
+      </c>
       <c r="R2" s="7"/>
       <c r="S2" s="7"/>
       <c r="T2" s="7"/>
@@ -893,7 +906,7 @@
       <c r="AZ2" s="7"/>
       <c r="BE2" s="7"/>
     </row>
-    <row r="3" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>1980</v>
       </c>
@@ -935,7 +948,9 @@
       <c r="P3" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q3" s="7"/>
+      <c r="Q3" s="30" t="s">
+        <v>27</v>
+      </c>
       <c r="R3" s="5"/>
       <c r="S3" s="5"/>
       <c r="T3" s="5"/>
@@ -968,7 +983,7 @@
       <c r="AZ3" s="7"/>
       <c r="BE3" s="7"/>
     </row>
-    <row r="4" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>1981</v>
       </c>
@@ -1010,7 +1025,9 @@
       <c r="P4" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q4" s="7"/>
+      <c r="Q4" s="30" t="s">
+        <v>27</v>
+      </c>
       <c r="R4" s="5"/>
       <c r="S4" s="5"/>
       <c r="T4" s="5"/>
@@ -1043,7 +1060,7 @@
       <c r="AZ4" s="7"/>
       <c r="BE4" s="7"/>
     </row>
-    <row r="5" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>1982</v>
       </c>
@@ -1085,7 +1102,9 @@
       <c r="P5" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q5" s="7"/>
+      <c r="Q5" s="30" t="s">
+        <v>27</v>
+      </c>
       <c r="R5" s="5"/>
       <c r="S5" s="5"/>
       <c r="T5" s="5"/>
@@ -1118,7 +1137,7 @@
       <c r="AZ5" s="7"/>
       <c r="BE5" s="7"/>
     </row>
-    <row r="6" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>1983</v>
       </c>
@@ -1160,7 +1179,9 @@
       <c r="P6" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q6" s="7"/>
+      <c r="Q6" s="30" t="s">
+        <v>27</v>
+      </c>
       <c r="R6" s="5"/>
       <c r="S6" s="5"/>
       <c r="T6" s="5"/>
@@ -1194,7 +1215,7 @@
       <c r="BE6" s="7"/>
       <c r="BJ6" s="7"/>
     </row>
-    <row r="7" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>1984</v>
       </c>
@@ -1236,7 +1257,9 @@
       <c r="P7" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q7" s="7"/>
+      <c r="Q7" s="30" t="s">
+        <v>27</v>
+      </c>
       <c r="R7" s="5"/>
       <c r="S7" s="5"/>
       <c r="T7" s="5"/>
@@ -1270,7 +1293,7 @@
       <c r="BE7" s="7"/>
       <c r="BJ7" s="7"/>
     </row>
-    <row r="8" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>1985</v>
       </c>
@@ -1312,7 +1335,9 @@
       <c r="P8" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q8" s="7"/>
+      <c r="Q8" s="30" t="s">
+        <v>27</v>
+      </c>
       <c r="R8" s="5"/>
       <c r="S8" s="5"/>
       <c r="T8" s="5"/>
@@ -1346,7 +1371,7 @@
       <c r="BE8" s="7"/>
       <c r="BJ8" s="7"/>
     </row>
-    <row r="9" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>1986</v>
       </c>
@@ -1388,7 +1413,9 @@
       <c r="P9" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q9" s="7"/>
+      <c r="Q9" s="30" t="s">
+        <v>27</v>
+      </c>
       <c r="R9" s="5"/>
       <c r="S9" s="5"/>
       <c r="T9" s="5"/>
@@ -1422,7 +1449,7 @@
       <c r="BE9" s="7"/>
       <c r="BJ9" s="7"/>
     </row>
-    <row r="10" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>1987</v>
       </c>
@@ -1464,7 +1491,9 @@
       <c r="P10" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q10" s="7"/>
+      <c r="Q10" s="30" t="s">
+        <v>27</v>
+      </c>
       <c r="R10" s="5"/>
       <c r="S10" s="5"/>
       <c r="T10" s="5"/>
@@ -1498,7 +1527,7 @@
       <c r="BE10" s="7"/>
       <c r="BJ10" s="7"/>
     </row>
-    <row r="11" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>1988</v>
       </c>
@@ -1540,7 +1569,9 @@
       <c r="P11" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q11" s="7"/>
+      <c r="Q11" s="30" t="s">
+        <v>27</v>
+      </c>
       <c r="R11" s="5"/>
       <c r="S11" s="5"/>
       <c r="T11" s="5"/>
@@ -1574,7 +1605,7 @@
       <c r="BE11" s="7"/>
       <c r="BJ11" s="7"/>
     </row>
-    <row r="12" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>1989</v>
       </c>
@@ -1616,7 +1647,9 @@
       <c r="P12" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q12" s="7"/>
+      <c r="Q12" s="30" t="s">
+        <v>27</v>
+      </c>
       <c r="R12" s="5"/>
       <c r="S12" s="5"/>
       <c r="T12" s="5"/>
@@ -1650,7 +1683,7 @@
       <c r="BE12" s="7"/>
       <c r="BJ12" s="7"/>
     </row>
-    <row r="13" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>1990</v>
       </c>
@@ -1692,7 +1725,9 @@
       <c r="P13" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q13" s="7"/>
+      <c r="Q13" s="30" t="s">
+        <v>27</v>
+      </c>
       <c r="R13" s="5"/>
       <c r="S13" s="5"/>
       <c r="T13" s="5"/>
@@ -1726,7 +1761,7 @@
       <c r="BE13" s="7"/>
       <c r="BJ13" s="7"/>
     </row>
-    <row r="14" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>1991</v>
       </c>
@@ -1768,7 +1803,9 @@
       <c r="P14" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q14" s="7"/>
+      <c r="Q14" s="30" t="s">
+        <v>27</v>
+      </c>
       <c r="R14" s="5"/>
       <c r="S14" s="5"/>
       <c r="T14" s="5"/>
@@ -1802,7 +1839,7 @@
       <c r="BE14" s="7"/>
       <c r="BJ14" s="7"/>
     </row>
-    <row r="15" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>1992</v>
       </c>
@@ -1844,7 +1881,9 @@
       <c r="P15" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q15" s="7"/>
+      <c r="Q15" s="30" t="s">
+        <v>27</v>
+      </c>
       <c r="R15" s="5"/>
       <c r="S15" s="5"/>
       <c r="T15" s="5"/>
@@ -1878,7 +1917,7 @@
       <c r="BE15" s="7"/>
       <c r="BJ15" s="7"/>
     </row>
-    <row r="16" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>1993</v>
       </c>
@@ -1920,7 +1959,9 @@
       <c r="P16" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q16" s="7"/>
+      <c r="Q16" s="30" t="s">
+        <v>27</v>
+      </c>
       <c r="R16" s="5"/>
       <c r="S16" s="5"/>
       <c r="T16" s="5"/>
@@ -1954,7 +1995,7 @@
       <c r="BE16" s="7"/>
       <c r="BJ16" s="7"/>
     </row>
-    <row r="17" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>1994</v>
       </c>
@@ -1996,7 +2037,9 @@
       <c r="P17" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q17" s="7"/>
+      <c r="Q17" s="30" t="s">
+        <v>27</v>
+      </c>
       <c r="R17" s="5"/>
       <c r="S17" s="5"/>
       <c r="T17" s="5"/>
@@ -2030,7 +2073,7 @@
       <c r="BE17" s="7"/>
       <c r="BJ17" s="7"/>
     </row>
-    <row r="18" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>1995</v>
       </c>
@@ -2072,7 +2115,9 @@
       <c r="P18" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q18" s="7"/>
+      <c r="Q18" s="30" t="s">
+        <v>27</v>
+      </c>
       <c r="R18" s="5"/>
       <c r="S18" s="5"/>
       <c r="T18" s="5"/>
@@ -2106,7 +2151,7 @@
       <c r="BE18" s="7"/>
       <c r="BJ18" s="7"/>
     </row>
-    <row r="19" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>1996</v>
       </c>
@@ -2148,7 +2193,9 @@
       <c r="P19" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q19" s="7"/>
+      <c r="Q19" s="30" t="s">
+        <v>27</v>
+      </c>
       <c r="R19" s="5"/>
       <c r="S19" s="5"/>
       <c r="T19" s="5"/>
@@ -2182,7 +2229,7 @@
       <c r="BE19" s="7"/>
       <c r="BJ19" s="7"/>
     </row>
-    <row r="20" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>1997</v>
       </c>
@@ -2223,7 +2270,7 @@
       <c r="P20" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q20" s="7"/>
+      <c r="Q20" s="31"/>
       <c r="R20" s="5"/>
       <c r="S20" s="5"/>
       <c r="T20" s="5"/>
@@ -2256,7 +2303,7 @@
       <c r="BE20" s="7"/>
       <c r="BJ20" s="7"/>
     </row>
-    <row r="21" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>1998</v>
       </c>
@@ -2297,7 +2344,7 @@
       <c r="P21" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q21" s="7"/>
+      <c r="Q21" s="31"/>
       <c r="R21" s="5"/>
       <c r="S21" s="5"/>
       <c r="T21" s="5"/>
@@ -2330,7 +2377,7 @@
       <c r="BE21" s="7"/>
       <c r="BJ21" s="7"/>
     </row>
-    <row r="22" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>1999</v>
       </c>
@@ -2371,7 +2418,7 @@
       <c r="P22" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q22" s="7"/>
+      <c r="Q22" s="31"/>
       <c r="R22" s="5"/>
       <c r="S22" s="5"/>
       <c r="T22" s="5"/>
@@ -2404,7 +2451,7 @@
       <c r="BE22" s="7"/>
       <c r="BJ22" s="7"/>
     </row>
-    <row r="23" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>2000</v>
       </c>
@@ -2445,7 +2492,7 @@
       <c r="P23" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q23" s="7"/>
+      <c r="Q23" s="31"/>
       <c r="R23" s="5"/>
       <c r="S23" s="5"/>
       <c r="T23" s="5"/>
@@ -2478,7 +2525,7 @@
       <c r="BE23" s="7"/>
       <c r="BJ23" s="7"/>
     </row>
-    <row r="24" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>2001</v>
       </c>
@@ -2519,7 +2566,7 @@
       <c r="P24" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q24" s="7"/>
+      <c r="Q24" s="31"/>
       <c r="R24" s="5"/>
       <c r="S24" s="5" t="s">
         <v>35</v>
@@ -2596,7 +2643,7 @@
       <c r="P25" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q25" s="30"/>
+      <c r="Q25" s="32"/>
       <c r="R25" s="5" t="s">
         <v>36</v>
       </c>
@@ -2631,7 +2678,7 @@
       <c r="BE25" s="7"/>
       <c r="BJ25" s="7"/>
     </row>
-    <row r="26" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>2003</v>
       </c>
@@ -2682,7 +2729,7 @@
       <c r="P26" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q26" s="30"/>
+      <c r="Q26" s="32"/>
       <c r="R26" s="5" t="s">
         <v>36</v>
       </c>
@@ -2717,7 +2764,7 @@
       <c r="BE26" s="7"/>
       <c r="BJ26" s="7"/>
     </row>
-    <row r="27" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>2004</v>
       </c>
@@ -2758,7 +2805,7 @@
       <c r="P27" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q27" s="7"/>
+      <c r="Q27" s="31"/>
       <c r="R27" s="5"/>
       <c r="S27" s="5"/>
       <c r="T27" s="5"/>
@@ -2791,7 +2838,7 @@
       <c r="BE27" s="7"/>
       <c r="BJ27" s="7"/>
     </row>
-    <row r="28" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>2005</v>
       </c>
@@ -2832,7 +2879,7 @@
       <c r="P28" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q28" s="7"/>
+      <c r="Q28" s="31"/>
       <c r="R28" s="5"/>
       <c r="S28" s="5"/>
       <c r="T28" s="5"/>
@@ -2865,7 +2912,7 @@
       <c r="BE28" s="7"/>
       <c r="BJ28" s="7"/>
     </row>
-    <row r="29" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>2006</v>
       </c>
@@ -2906,7 +2953,7 @@
       <c r="P29" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q29" s="7"/>
+      <c r="Q29" s="31"/>
       <c r="R29" s="5"/>
       <c r="S29" s="5"/>
       <c r="T29" s="5"/>
@@ -2939,7 +2986,7 @@
       <c r="BE29" s="7"/>
       <c r="BJ29" s="7"/>
     </row>
-    <row r="30" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>2007</v>
       </c>
@@ -2981,7 +3028,7 @@
       <c r="P30" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q30" s="7"/>
+      <c r="Q30" s="31"/>
       <c r="R30" s="5"/>
       <c r="S30" s="5"/>
       <c r="T30" s="5"/>
@@ -3014,7 +3061,7 @@
       <c r="BE30" s="7"/>
       <c r="BJ30" s="7"/>
     </row>
-    <row r="31" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>2008</v>
       </c>
@@ -3055,7 +3102,7 @@
       <c r="P31" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q31" s="7"/>
+      <c r="Q31" s="31"/>
       <c r="R31" s="5"/>
       <c r="S31" s="5"/>
       <c r="T31" s="5"/>
@@ -3088,7 +3135,7 @@
       <c r="BE31" s="7"/>
       <c r="BJ31" s="7"/>
     </row>
-    <row r="32" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
         <v>2009</v>
       </c>
@@ -3129,7 +3176,7 @@
       <c r="P32" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q32" s="7"/>
+      <c r="Q32" s="31"/>
       <c r="R32" s="5"/>
       <c r="S32" s="5"/>
       <c r="T32" s="5"/>
@@ -3162,7 +3209,7 @@
       <c r="BE32" s="7"/>
       <c r="BJ32" s="7"/>
     </row>
-    <row r="33" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>2010</v>
       </c>
@@ -3204,7 +3251,7 @@
       <c r="P33" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q33" s="7"/>
+      <c r="Q33" s="31"/>
       <c r="R33" s="5"/>
       <c r="S33" s="5" t="s">
         <v>37</v>
@@ -3239,7 +3286,7 @@
       <c r="BE33" s="7"/>
       <c r="BJ33" s="7"/>
     </row>
-    <row r="34" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>2011</v>
       </c>
@@ -3281,7 +3328,7 @@
       <c r="P34" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q34" s="7"/>
+      <c r="Q34" s="31"/>
       <c r="R34" s="5"/>
       <c r="S34" s="5" t="s">
         <v>37</v>
@@ -3316,7 +3363,7 @@
       <c r="BE34" s="7"/>
       <c r="BJ34" s="7"/>
     </row>
-    <row r="35" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>2012</v>
       </c>
@@ -3362,7 +3409,7 @@
       <c r="P35" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q35" s="30"/>
+      <c r="Q35" s="32"/>
       <c r="R35" s="5" t="s">
         <v>36</v>
       </c>
@@ -3399,7 +3446,7 @@
       <c r="BE35" s="7"/>
       <c r="BJ35" s="7"/>
     </row>
-    <row r="36" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>2013</v>
       </c>
@@ -3419,7 +3466,7 @@
       </c>
       <c r="F36" s="4"/>
       <c r="G36" s="14">
-        <f t="shared" ref="G33:G40" si="7">ROUND(0.2*SUM(F36,H36,I36),0)</f>
+        <f>ROUND(0.2*SUM(F36,H36,I36),0)</f>
         <v>478</v>
       </c>
       <c r="H36" s="1">
@@ -3451,7 +3498,7 @@
       <c r="P36" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q36" s="30"/>
+      <c r="Q36" s="32"/>
       <c r="R36" s="5" t="s">
         <v>36</v>
       </c>
@@ -3488,7 +3535,7 @@
       <c r="BE36" s="7"/>
       <c r="BJ36" s="7"/>
     </row>
-    <row r="37" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>2014</v>
       </c>
@@ -3508,7 +3555,7 @@
       </c>
       <c r="F37" s="4"/>
       <c r="G37" s="14">
-        <f t="shared" si="7"/>
+        <f>ROUND(0.2*SUM(F37,H37,I37),0)</f>
         <v>773</v>
       </c>
       <c r="H37" s="1">
@@ -3540,7 +3587,7 @@
       <c r="P37" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q37" s="30"/>
+      <c r="Q37" s="32"/>
       <c r="R37" s="5" t="s">
         <v>36</v>
       </c>
@@ -3577,7 +3624,7 @@
       <c r="BE37" s="7"/>
       <c r="BJ37" s="7"/>
     </row>
-    <row r="38" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
         <v>2015</v>
       </c>
@@ -3597,7 +3644,7 @@
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="14">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="G33:G40" si="7">ROUND(0.2*SUM(F38,H38,I38),0)</f>
         <v>983</v>
       </c>
       <c r="H38" s="1">
@@ -3629,7 +3676,7 @@
       <c r="P38" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q38" s="30"/>
+      <c r="Q38" s="32"/>
       <c r="R38" s="5" t="s">
         <v>36</v>
       </c>
@@ -3666,7 +3713,7 @@
       <c r="BE38" s="7"/>
       <c r="BJ38" s="7"/>
     </row>
-    <row r="39" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>2016</v>
       </c>
@@ -3718,7 +3765,7 @@
       <c r="P39" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q39" s="30"/>
+      <c r="Q39" s="32"/>
       <c r="R39" s="5" t="s">
         <v>36</v>
       </c>
@@ -3755,7 +3802,7 @@
       <c r="BE39" s="7"/>
       <c r="BJ39" s="7"/>
     </row>
-    <row r="40" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>2017</v>
       </c>
@@ -3809,7 +3856,7 @@
       <c r="P40" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q40" s="7" t="s">
+      <c r="Q40" s="31" t="s">
         <v>40</v>
       </c>
       <c r="R40" s="5" t="s">
@@ -3848,7 +3895,7 @@
       <c r="BE40" s="7"/>
       <c r="BJ40" s="7"/>
     </row>
-    <row r="41" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
         <v>2018</v>
       </c>
@@ -3899,7 +3946,7 @@
       <c r="P41" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q41" s="30"/>
+      <c r="Q41" s="32"/>
       <c r="R41" s="5" t="s">
         <v>36</v>
       </c>
@@ -3934,7 +3981,7 @@
       <c r="BE41" s="7"/>
       <c r="BJ41" s="7"/>
     </row>
-    <row r="42" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>2019</v>
       </c>
@@ -3987,7 +4034,7 @@
       <c r="P42" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q42" s="7" t="s">
+      <c r="Q42" s="31" t="s">
         <v>39</v>
       </c>
       <c r="R42" s="5" t="s">
@@ -4024,7 +4071,7 @@
       <c r="BE42" s="7"/>
       <c r="BJ42" s="7"/>
     </row>
-    <row r="43" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>2020</v>
       </c>
@@ -4077,7 +4124,7 @@
       <c r="P43" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q43" s="7" t="s">
+      <c r="Q43" s="31" t="s">
         <v>41</v>
       </c>
       <c r="R43" s="5" t="s">
@@ -4114,7 +4161,7 @@
       <c r="BE43" s="7"/>
       <c r="BJ43" s="7"/>
     </row>
-    <row r="44" spans="1:62" ht="15" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>2021</v>
       </c>
@@ -4164,7 +4211,7 @@
       <c r="P44" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="Q44" s="5" t="s">
+      <c r="Q44" s="33" t="s">
         <v>42</v>
       </c>
       <c r="R44" s="5" t="s">
@@ -4201,7 +4248,7 @@
       <c r="BE44" s="7"/>
       <c r="BJ44" s="7"/>
     </row>
-    <row r="45" spans="1:62" ht="15" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>2022</v>
       </c>
@@ -4251,7 +4298,7 @@
       <c r="P45" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="Q45" s="5" t="s">
+      <c r="Q45" s="33" t="s">
         <v>44</v>
       </c>
       <c r="R45" s="5" t="s">
@@ -4288,7 +4335,7 @@
       <c r="BE45" s="7"/>
       <c r="BJ45" s="7"/>
     </row>
-    <row r="46" spans="1:62" ht="15" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>2023</v>
       </c>
@@ -4338,7 +4385,7 @@
       <c r="P46" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="Q46" s="5" t="s">
+      <c r="Q46" s="33" t="s">
         <v>43</v>
       </c>
       <c r="R46" s="5" t="s">
@@ -4375,7 +4422,7 @@
       <c r="BE46" s="7"/>
       <c r="BJ46" s="7"/>
     </row>
-    <row r="47" spans="1:62" ht="15" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>2024</v>
       </c>
@@ -4425,7 +4472,7 @@
       <c r="P47" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="Q47" s="5" t="s">
+      <c r="Q47" s="33" t="s">
         <v>45</v>
       </c>
       <c r="R47" s="5" t="s">
@@ -4462,7 +4509,7 @@
       <c r="BE47" s="7"/>
       <c r="BJ47" s="7"/>
     </row>
-    <row r="48" spans="1:62" ht="15" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>2025</v>
       </c>
@@ -4506,7 +4553,7 @@
       <c r="P48" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="Q48" s="5" t="s">
+      <c r="Q48" s="33" t="s">
         <v>46</v>
       </c>
       <c r="R48" s="5" t="s">

</xml_diff>

<commit_message>
Update freshwater rec catch numbers based on LGL creel reports
</commit_message>
<xml_diff>
--- a/data-raw/freshwater-catch.xlsx
+++ b/data-raw/freshwater-catch.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\skrunchy2025\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1649AC2B-2634-4801-9A7A-60FFFF04D40F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FCE902D-13F1-481D-8064-DF2B457AEE42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E0CDEE87-6CC2-4107-81B9-F1AD4EA649A7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="56">
   <si>
     <t>Year</t>
   </si>
@@ -180,6 +180,30 @@
   </si>
   <si>
     <t xml:space="preserve"> FW Sport source details</t>
+  </si>
+  <si>
+    <t>No creel survey in 2018</t>
+  </si>
+  <si>
+    <t>FSC data source</t>
+  </si>
+  <si>
+    <t>Robichaud &amp; English 2012, Tables 11, 13</t>
+  </si>
+  <si>
+    <t>Robichaud &amp; English 2011, Tables 13,15</t>
+  </si>
+  <si>
+    <t>Robichaud et al. 2013, Tables 11, 13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Robichaud et al. 2014, Tables 12, 14 </t>
+  </si>
+  <si>
+    <t>Robichaud et al. 2015, Tables 12, 14</t>
+  </si>
+  <si>
+    <t>Robichaud et al. 2016, Tables 12, 14</t>
   </si>
 </sst>
 </file>
@@ -302,7 +326,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -373,6 +397,11 @@
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -392,6 +421,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -691,7 +724,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35E3952C-60AA-4AE7-A274-2D9A331D3C7B}">
-  <dimension ref="A1:BJ190"/>
+  <dimension ref="A1:BK191"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.85546875" style="1" customWidth="1"/>
@@ -701,34 +734,34 @@
     <col min="13" max="13" width="8.42578125" style="19" customWidth="1"/>
     <col min="14" max="15" width="7.5703125" style="1" customWidth="1"/>
     <col min="16" max="16" width="34.42578125" style="1" customWidth="1"/>
-    <col min="17" max="17" width="33.42578125" style="3" customWidth="1"/>
-    <col min="18" max="18" width="32.5703125" style="1" customWidth="1"/>
-    <col min="19" max="19" width="24.140625" style="1" customWidth="1"/>
-    <col min="20" max="23" width="7.5703125" style="1" customWidth="1"/>
-    <col min="24" max="25" width="8.85546875" style="1" customWidth="1"/>
-    <col min="26" max="29" width="7.5703125" style="1" customWidth="1"/>
-    <col min="30" max="30" width="8.140625" style="1" customWidth="1"/>
-    <col min="31" max="44" width="8.7109375" style="1"/>
-    <col min="45" max="45" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="8.7109375" style="1"/>
-    <col min="47" max="47" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="8.7109375" style="1"/>
-    <col min="49" max="49" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="8.7109375" style="1"/>
-    <col min="51" max="51" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="8.7109375" style="1"/>
-    <col min="53" max="54" width="4.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="7.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="57" max="58" width="8.7109375" style="1"/>
-    <col min="59" max="59" width="4.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="3.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="7" style="1" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="7.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="63" max="16384" width="8.7109375" style="1"/>
+    <col min="17" max="17" width="37.7109375" style="3" customWidth="1"/>
+    <col min="18" max="19" width="32.5703125" style="1" customWidth="1"/>
+    <col min="20" max="20" width="24.140625" style="1" customWidth="1"/>
+    <col min="21" max="24" width="7.5703125" style="1" customWidth="1"/>
+    <col min="25" max="26" width="8.85546875" style="1" customWidth="1"/>
+    <col min="27" max="30" width="7.5703125" style="1" customWidth="1"/>
+    <col min="31" max="31" width="8.140625" style="1" customWidth="1"/>
+    <col min="32" max="45" width="8.7109375" style="1"/>
+    <col min="46" max="46" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="8.7109375" style="1"/>
+    <col min="48" max="48" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="8.7109375" style="1"/>
+    <col min="50" max="50" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="8.7109375" style="1"/>
+    <col min="52" max="52" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="8.7109375" style="1"/>
+    <col min="54" max="55" width="4.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="7.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="58" max="59" width="8.7109375" style="1"/>
+    <col min="60" max="60" width="4.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="3.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="7" style="1" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="7.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="64" max="16384" width="8.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:62" s="4" customFormat="1" ht="72" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:63" s="4" customFormat="1" ht="72" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
@@ -784,15 +817,17 @@
         <v>34</v>
       </c>
       <c r="S1" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="T1" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="T1" s="18"/>
-      <c r="U1" s="20"/>
-      <c r="V1" s="18"/>
-      <c r="W1" s="20"/>
-      <c r="X1" s="18"/>
-      <c r="Y1" s="20"/>
-      <c r="Z1" s="18"/>
+      <c r="U1" s="18"/>
+      <c r="V1" s="20"/>
+      <c r="W1" s="18"/>
+      <c r="X1" s="20"/>
+      <c r="Y1" s="18"/>
+      <c r="Z1" s="20"/>
       <c r="AA1" s="18"/>
       <c r="AB1" s="18"/>
       <c r="AC1" s="18"/>
@@ -811,7 +846,7 @@
       <c r="AP1" s="18"/>
       <c r="AQ1" s="18"/>
       <c r="AR1" s="18"/>
-      <c r="AS1" s="21"/>
+      <c r="AS1" s="18"/>
       <c r="AT1" s="21"/>
       <c r="AU1" s="21"/>
       <c r="AV1" s="21"/>
@@ -820,12 +855,13 @@
       <c r="AY1" s="21"/>
       <c r="AZ1" s="21"/>
       <c r="BA1" s="21"/>
-      <c r="BB1" s="19"/>
+      <c r="BB1" s="21"/>
       <c r="BC1" s="19"/>
       <c r="BD1" s="19"/>
-      <c r="BE1" s="1"/>
-    </row>
-    <row r="2" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="BE1" s="19"/>
+      <c r="BF1" s="1"/>
+    </row>
+    <row r="2" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>1979</v>
       </c>
@@ -882,31 +918,32 @@
       <c r="W2" s="7"/>
       <c r="X2" s="7"/>
       <c r="Y2" s="7"/>
-      <c r="Z2" s="8"/>
+      <c r="Z2" s="7"/>
       <c r="AA2" s="8"/>
       <c r="AB2" s="8"/>
       <c r="AC2" s="8"/>
       <c r="AD2" s="8"/>
-      <c r="AE2" s="7"/>
+      <c r="AE2" s="8"/>
       <c r="AF2" s="7"/>
       <c r="AG2" s="7"/>
       <c r="AH2" s="7"/>
       <c r="AI2" s="7"/>
       <c r="AJ2" s="7"/>
-      <c r="AK2" s="9"/>
-      <c r="AM2" s="7"/>
+      <c r="AK2" s="7"/>
+      <c r="AL2" s="9"/>
       <c r="AN2" s="7"/>
       <c r="AO2" s="7"/>
       <c r="AP2" s="7"/>
       <c r="AQ2" s="7"/>
       <c r="AR2" s="7"/>
-      <c r="AT2" s="7"/>
-      <c r="AV2" s="7"/>
-      <c r="AX2" s="7"/>
-      <c r="AZ2" s="7"/>
-      <c r="BE2" s="7"/>
-    </row>
-    <row r="3" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS2" s="7"/>
+      <c r="AU2" s="7"/>
+      <c r="AW2" s="7"/>
+      <c r="AY2" s="7"/>
+      <c r="BA2" s="7"/>
+      <c r="BF2" s="7"/>
+    </row>
+    <row r="3" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>1980</v>
       </c>
@@ -954,36 +991,37 @@
       <c r="R3" s="5"/>
       <c r="S3" s="5"/>
       <c r="T3" s="5"/>
-      <c r="U3" s="7"/>
+      <c r="U3" s="5"/>
       <c r="V3" s="7"/>
       <c r="W3" s="7"/>
       <c r="X3" s="7"/>
       <c r="Y3" s="7"/>
-      <c r="Z3" s="8"/>
+      <c r="Z3" s="7"/>
       <c r="AA3" s="8"/>
       <c r="AB3" s="8"/>
       <c r="AC3" s="8"/>
       <c r="AD3" s="8"/>
-      <c r="AE3" s="7"/>
+      <c r="AE3" s="8"/>
       <c r="AF3" s="7"/>
       <c r="AG3" s="7"/>
       <c r="AH3" s="7"/>
       <c r="AI3" s="7"/>
       <c r="AJ3" s="7"/>
-      <c r="AK3" s="9"/>
-      <c r="AM3" s="7"/>
+      <c r="AK3" s="7"/>
+      <c r="AL3" s="9"/>
       <c r="AN3" s="7"/>
       <c r="AO3" s="7"/>
       <c r="AP3" s="7"/>
       <c r="AQ3" s="7"/>
       <c r="AR3" s="7"/>
-      <c r="AT3" s="7"/>
-      <c r="AV3" s="7"/>
-      <c r="AX3" s="7"/>
-      <c r="AZ3" s="7"/>
-      <c r="BE3" s="7"/>
-    </row>
-    <row r="4" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS3" s="7"/>
+      <c r="AU3" s="7"/>
+      <c r="AW3" s="7"/>
+      <c r="AY3" s="7"/>
+      <c r="BA3" s="7"/>
+      <c r="BF3" s="7"/>
+    </row>
+    <row r="4" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>1981</v>
       </c>
@@ -1031,36 +1069,37 @@
       <c r="R4" s="5"/>
       <c r="S4" s="5"/>
       <c r="T4" s="5"/>
-      <c r="U4" s="7"/>
+      <c r="U4" s="5"/>
       <c r="V4" s="7"/>
       <c r="W4" s="7"/>
       <c r="X4" s="7"/>
       <c r="Y4" s="7"/>
-      <c r="Z4" s="8"/>
+      <c r="Z4" s="7"/>
       <c r="AA4" s="8"/>
       <c r="AB4" s="8"/>
       <c r="AC4" s="8"/>
       <c r="AD4" s="8"/>
-      <c r="AE4" s="7"/>
+      <c r="AE4" s="8"/>
       <c r="AF4" s="7"/>
       <c r="AG4" s="7"/>
       <c r="AH4" s="7"/>
       <c r="AI4" s="7"/>
       <c r="AJ4" s="7"/>
-      <c r="AK4" s="9"/>
-      <c r="AM4" s="7"/>
+      <c r="AK4" s="7"/>
+      <c r="AL4" s="9"/>
       <c r="AN4" s="7"/>
       <c r="AO4" s="7"/>
       <c r="AP4" s="7"/>
       <c r="AQ4" s="7"/>
       <c r="AR4" s="7"/>
-      <c r="AT4" s="7"/>
-      <c r="AV4" s="7"/>
-      <c r="AX4" s="7"/>
-      <c r="AZ4" s="7"/>
-      <c r="BE4" s="7"/>
-    </row>
-    <row r="5" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS4" s="7"/>
+      <c r="AU4" s="7"/>
+      <c r="AW4" s="7"/>
+      <c r="AY4" s="7"/>
+      <c r="BA4" s="7"/>
+      <c r="BF4" s="7"/>
+    </row>
+    <row r="5" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>1982</v>
       </c>
@@ -1108,36 +1147,37 @@
       <c r="R5" s="5"/>
       <c r="S5" s="5"/>
       <c r="T5" s="5"/>
-      <c r="U5" s="7"/>
+      <c r="U5" s="5"/>
       <c r="V5" s="7"/>
       <c r="W5" s="7"/>
       <c r="X5" s="7"/>
       <c r="Y5" s="7"/>
-      <c r="Z5" s="8"/>
+      <c r="Z5" s="7"/>
       <c r="AA5" s="8"/>
       <c r="AB5" s="8"/>
       <c r="AC5" s="8"/>
       <c r="AD5" s="8"/>
-      <c r="AE5" s="7"/>
+      <c r="AE5" s="8"/>
       <c r="AF5" s="7"/>
       <c r="AG5" s="7"/>
       <c r="AH5" s="7"/>
       <c r="AI5" s="7"/>
       <c r="AJ5" s="7"/>
-      <c r="AK5" s="9"/>
-      <c r="AM5" s="7"/>
+      <c r="AK5" s="7"/>
+      <c r="AL5" s="9"/>
       <c r="AN5" s="7"/>
       <c r="AO5" s="7"/>
       <c r="AP5" s="7"/>
       <c r="AQ5" s="7"/>
       <c r="AR5" s="7"/>
-      <c r="AT5" s="7"/>
-      <c r="AV5" s="7"/>
-      <c r="AX5" s="7"/>
-      <c r="AZ5" s="7"/>
-      <c r="BE5" s="7"/>
-    </row>
-    <row r="6" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS5" s="7"/>
+      <c r="AU5" s="7"/>
+      <c r="AW5" s="7"/>
+      <c r="AY5" s="7"/>
+      <c r="BA5" s="7"/>
+      <c r="BF5" s="7"/>
+    </row>
+    <row r="6" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>1983</v>
       </c>
@@ -1185,37 +1225,38 @@
       <c r="R6" s="5"/>
       <c r="S6" s="5"/>
       <c r="T6" s="5"/>
-      <c r="U6" s="7"/>
+      <c r="U6" s="5"/>
       <c r="V6" s="7"/>
       <c r="W6" s="7"/>
       <c r="X6" s="7"/>
       <c r="Y6" s="7"/>
-      <c r="Z6" s="8"/>
+      <c r="Z6" s="7"/>
       <c r="AA6" s="8"/>
       <c r="AB6" s="8"/>
       <c r="AC6" s="8"/>
       <c r="AD6" s="8"/>
-      <c r="AE6" s="7"/>
+      <c r="AE6" s="8"/>
       <c r="AF6" s="7"/>
       <c r="AG6" s="7"/>
       <c r="AH6" s="7"/>
       <c r="AI6" s="7"/>
       <c r="AJ6" s="7"/>
-      <c r="AK6" s="9"/>
-      <c r="AM6" s="7"/>
+      <c r="AK6" s="7"/>
+      <c r="AL6" s="9"/>
       <c r="AN6" s="7"/>
       <c r="AO6" s="7"/>
       <c r="AP6" s="7"/>
       <c r="AQ6" s="7"/>
       <c r="AR6" s="7"/>
-      <c r="AT6" s="7"/>
-      <c r="AV6" s="7"/>
-      <c r="AX6" s="7"/>
-      <c r="AZ6" s="7"/>
-      <c r="BE6" s="7"/>
-      <c r="BJ6" s="7"/>
-    </row>
-    <row r="7" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS6" s="7"/>
+      <c r="AU6" s="7"/>
+      <c r="AW6" s="7"/>
+      <c r="AY6" s="7"/>
+      <c r="BA6" s="7"/>
+      <c r="BF6" s="7"/>
+      <c r="BK6" s="7"/>
+    </row>
+    <row r="7" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>1984</v>
       </c>
@@ -1263,37 +1304,38 @@
       <c r="R7" s="5"/>
       <c r="S7" s="5"/>
       <c r="T7" s="5"/>
-      <c r="U7" s="7"/>
+      <c r="U7" s="5"/>
       <c r="V7" s="7"/>
       <c r="W7" s="7"/>
       <c r="X7" s="7"/>
       <c r="Y7" s="7"/>
-      <c r="Z7" s="8"/>
+      <c r="Z7" s="7"/>
       <c r="AA7" s="8"/>
       <c r="AB7" s="8"/>
       <c r="AC7" s="8"/>
       <c r="AD7" s="8"/>
-      <c r="AE7" s="7"/>
+      <c r="AE7" s="8"/>
       <c r="AF7" s="7"/>
       <c r="AG7" s="7"/>
       <c r="AH7" s="7"/>
       <c r="AI7" s="7"/>
       <c r="AJ7" s="7"/>
-      <c r="AK7" s="9"/>
-      <c r="AM7" s="7"/>
+      <c r="AK7" s="7"/>
+      <c r="AL7" s="9"/>
       <c r="AN7" s="7"/>
       <c r="AO7" s="7"/>
       <c r="AP7" s="7"/>
       <c r="AQ7" s="7"/>
       <c r="AR7" s="7"/>
-      <c r="AT7" s="7"/>
-      <c r="AV7" s="7"/>
-      <c r="AX7" s="7"/>
-      <c r="AZ7" s="7"/>
-      <c r="BE7" s="7"/>
-      <c r="BJ7" s="7"/>
-    </row>
-    <row r="8" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS7" s="7"/>
+      <c r="AU7" s="7"/>
+      <c r="AW7" s="7"/>
+      <c r="AY7" s="7"/>
+      <c r="BA7" s="7"/>
+      <c r="BF7" s="7"/>
+      <c r="BK7" s="7"/>
+    </row>
+    <row r="8" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>1985</v>
       </c>
@@ -1341,37 +1383,38 @@
       <c r="R8" s="5"/>
       <c r="S8" s="5"/>
       <c r="T8" s="5"/>
-      <c r="U8" s="7"/>
+      <c r="U8" s="5"/>
       <c r="V8" s="7"/>
       <c r="W8" s="7"/>
       <c r="X8" s="7"/>
       <c r="Y8" s="7"/>
-      <c r="Z8" s="8"/>
+      <c r="Z8" s="7"/>
       <c r="AA8" s="8"/>
       <c r="AB8" s="8"/>
       <c r="AC8" s="8"/>
       <c r="AD8" s="8"/>
-      <c r="AE8" s="7"/>
+      <c r="AE8" s="8"/>
       <c r="AF8" s="7"/>
       <c r="AG8" s="7"/>
       <c r="AH8" s="7"/>
       <c r="AI8" s="7"/>
       <c r="AJ8" s="7"/>
-      <c r="AK8" s="9"/>
-      <c r="AM8" s="7"/>
+      <c r="AK8" s="7"/>
+      <c r="AL8" s="9"/>
       <c r="AN8" s="7"/>
       <c r="AO8" s="7"/>
       <c r="AP8" s="7"/>
       <c r="AQ8" s="7"/>
       <c r="AR8" s="7"/>
-      <c r="AT8" s="7"/>
-      <c r="AV8" s="7"/>
-      <c r="AX8" s="7"/>
-      <c r="AZ8" s="7"/>
-      <c r="BE8" s="7"/>
-      <c r="BJ8" s="7"/>
-    </row>
-    <row r="9" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS8" s="7"/>
+      <c r="AU8" s="7"/>
+      <c r="AW8" s="7"/>
+      <c r="AY8" s="7"/>
+      <c r="BA8" s="7"/>
+      <c r="BF8" s="7"/>
+      <c r="BK8" s="7"/>
+    </row>
+    <row r="9" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>1986</v>
       </c>
@@ -1419,37 +1462,38 @@
       <c r="R9" s="5"/>
       <c r="S9" s="5"/>
       <c r="T9" s="5"/>
-      <c r="U9" s="7"/>
+      <c r="U9" s="5"/>
       <c r="V9" s="7"/>
       <c r="W9" s="7"/>
       <c r="X9" s="7"/>
       <c r="Y9" s="7"/>
-      <c r="Z9" s="8"/>
+      <c r="Z9" s="7"/>
       <c r="AA9" s="8"/>
       <c r="AB9" s="8"/>
       <c r="AC9" s="8"/>
       <c r="AD9" s="8"/>
-      <c r="AE9" s="7"/>
+      <c r="AE9" s="8"/>
       <c r="AF9" s="7"/>
       <c r="AG9" s="7"/>
       <c r="AH9" s="7"/>
       <c r="AI9" s="7"/>
       <c r="AJ9" s="7"/>
-      <c r="AK9" s="9"/>
-      <c r="AM9" s="7"/>
+      <c r="AK9" s="7"/>
+      <c r="AL9" s="9"/>
       <c r="AN9" s="7"/>
       <c r="AO9" s="7"/>
       <c r="AP9" s="7"/>
       <c r="AQ9" s="7"/>
       <c r="AR9" s="7"/>
-      <c r="AT9" s="7"/>
-      <c r="AV9" s="7"/>
-      <c r="AX9" s="7"/>
-      <c r="AZ9" s="7"/>
-      <c r="BE9" s="7"/>
-      <c r="BJ9" s="7"/>
-    </row>
-    <row r="10" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS9" s="7"/>
+      <c r="AU9" s="7"/>
+      <c r="AW9" s="7"/>
+      <c r="AY9" s="7"/>
+      <c r="BA9" s="7"/>
+      <c r="BF9" s="7"/>
+      <c r="BK9" s="7"/>
+    </row>
+    <row r="10" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>1987</v>
       </c>
@@ -1497,37 +1541,38 @@
       <c r="R10" s="5"/>
       <c r="S10" s="5"/>
       <c r="T10" s="5"/>
-      <c r="U10" s="7"/>
+      <c r="U10" s="5"/>
       <c r="V10" s="7"/>
       <c r="W10" s="7"/>
       <c r="X10" s="7"/>
       <c r="Y10" s="7"/>
-      <c r="Z10" s="8"/>
+      <c r="Z10" s="7"/>
       <c r="AA10" s="8"/>
       <c r="AB10" s="8"/>
       <c r="AC10" s="8"/>
       <c r="AD10" s="8"/>
-      <c r="AE10" s="7"/>
+      <c r="AE10" s="8"/>
       <c r="AF10" s="7"/>
       <c r="AG10" s="7"/>
       <c r="AH10" s="7"/>
       <c r="AI10" s="7"/>
       <c r="AJ10" s="7"/>
-      <c r="AK10" s="9"/>
-      <c r="AM10" s="7"/>
+      <c r="AK10" s="7"/>
+      <c r="AL10" s="9"/>
       <c r="AN10" s="7"/>
       <c r="AO10" s="7"/>
       <c r="AP10" s="7"/>
       <c r="AQ10" s="7"/>
       <c r="AR10" s="7"/>
-      <c r="AT10" s="7"/>
-      <c r="AV10" s="7"/>
-      <c r="AX10" s="7"/>
-      <c r="AZ10" s="7"/>
-      <c r="BE10" s="7"/>
-      <c r="BJ10" s="7"/>
-    </row>
-    <row r="11" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS10" s="7"/>
+      <c r="AU10" s="7"/>
+      <c r="AW10" s="7"/>
+      <c r="AY10" s="7"/>
+      <c r="BA10" s="7"/>
+      <c r="BF10" s="7"/>
+      <c r="BK10" s="7"/>
+    </row>
+    <row r="11" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>1988</v>
       </c>
@@ -1575,37 +1620,38 @@
       <c r="R11" s="5"/>
       <c r="S11" s="5"/>
       <c r="T11" s="5"/>
-      <c r="U11" s="7"/>
+      <c r="U11" s="5"/>
       <c r="V11" s="7"/>
       <c r="W11" s="7"/>
       <c r="X11" s="7"/>
       <c r="Y11" s="7"/>
-      <c r="Z11" s="8"/>
+      <c r="Z11" s="7"/>
       <c r="AA11" s="8"/>
       <c r="AB11" s="8"/>
       <c r="AC11" s="8"/>
       <c r="AD11" s="8"/>
-      <c r="AE11" s="7"/>
+      <c r="AE11" s="8"/>
       <c r="AF11" s="7"/>
       <c r="AG11" s="7"/>
       <c r="AH11" s="7"/>
       <c r="AI11" s="7"/>
       <c r="AJ11" s="7"/>
-      <c r="AK11" s="9"/>
-      <c r="AM11" s="7"/>
+      <c r="AK11" s="7"/>
+      <c r="AL11" s="9"/>
       <c r="AN11" s="7"/>
       <c r="AO11" s="7"/>
       <c r="AP11" s="7"/>
       <c r="AQ11" s="7"/>
       <c r="AR11" s="7"/>
-      <c r="AT11" s="7"/>
-      <c r="AV11" s="7"/>
-      <c r="AX11" s="7"/>
-      <c r="AZ11" s="7"/>
-      <c r="BE11" s="7"/>
-      <c r="BJ11" s="7"/>
-    </row>
-    <row r="12" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS11" s="7"/>
+      <c r="AU11" s="7"/>
+      <c r="AW11" s="7"/>
+      <c r="AY11" s="7"/>
+      <c r="BA11" s="7"/>
+      <c r="BF11" s="7"/>
+      <c r="BK11" s="7"/>
+    </row>
+    <row r="12" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>1989</v>
       </c>
@@ -1653,37 +1699,38 @@
       <c r="R12" s="5"/>
       <c r="S12" s="5"/>
       <c r="T12" s="5"/>
-      <c r="U12" s="7"/>
+      <c r="U12" s="5"/>
       <c r="V12" s="7"/>
       <c r="W12" s="7"/>
       <c r="X12" s="7"/>
       <c r="Y12" s="7"/>
-      <c r="Z12" s="8"/>
+      <c r="Z12" s="7"/>
       <c r="AA12" s="8"/>
       <c r="AB12" s="8"/>
       <c r="AC12" s="8"/>
       <c r="AD12" s="8"/>
-      <c r="AE12" s="7"/>
+      <c r="AE12" s="8"/>
       <c r="AF12" s="7"/>
       <c r="AG12" s="7"/>
       <c r="AH12" s="7"/>
       <c r="AI12" s="7"/>
       <c r="AJ12" s="7"/>
-      <c r="AK12" s="9"/>
-      <c r="AM12" s="7"/>
+      <c r="AK12" s="7"/>
+      <c r="AL12" s="9"/>
       <c r="AN12" s="7"/>
       <c r="AO12" s="7"/>
       <c r="AP12" s="7"/>
       <c r="AQ12" s="7"/>
       <c r="AR12" s="7"/>
-      <c r="AT12" s="7"/>
-      <c r="AV12" s="7"/>
-      <c r="AX12" s="7"/>
-      <c r="AZ12" s="7"/>
-      <c r="BE12" s="7"/>
-      <c r="BJ12" s="7"/>
-    </row>
-    <row r="13" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS12" s="7"/>
+      <c r="AU12" s="7"/>
+      <c r="AW12" s="7"/>
+      <c r="AY12" s="7"/>
+      <c r="BA12" s="7"/>
+      <c r="BF12" s="7"/>
+      <c r="BK12" s="7"/>
+    </row>
+    <row r="13" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>1990</v>
       </c>
@@ -1731,37 +1778,38 @@
       <c r="R13" s="5"/>
       <c r="S13" s="5"/>
       <c r="T13" s="5"/>
-      <c r="U13" s="7"/>
+      <c r="U13" s="5"/>
       <c r="V13" s="7"/>
       <c r="W13" s="7"/>
       <c r="X13" s="7"/>
       <c r="Y13" s="7"/>
-      <c r="Z13" s="8"/>
+      <c r="Z13" s="7"/>
       <c r="AA13" s="8"/>
       <c r="AB13" s="8"/>
       <c r="AC13" s="8"/>
       <c r="AD13" s="8"/>
-      <c r="AE13" s="7"/>
+      <c r="AE13" s="8"/>
       <c r="AF13" s="7"/>
       <c r="AG13" s="7"/>
       <c r="AH13" s="7"/>
       <c r="AI13" s="7"/>
       <c r="AJ13" s="7"/>
-      <c r="AK13" s="9"/>
-      <c r="AM13" s="7"/>
+      <c r="AK13" s="7"/>
+      <c r="AL13" s="9"/>
       <c r="AN13" s="7"/>
       <c r="AO13" s="7"/>
       <c r="AP13" s="7"/>
       <c r="AQ13" s="7"/>
       <c r="AR13" s="7"/>
-      <c r="AT13" s="7"/>
-      <c r="AV13" s="7"/>
-      <c r="AX13" s="7"/>
-      <c r="AZ13" s="7"/>
-      <c r="BE13" s="7"/>
-      <c r="BJ13" s="7"/>
-    </row>
-    <row r="14" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS13" s="7"/>
+      <c r="AU13" s="7"/>
+      <c r="AW13" s="7"/>
+      <c r="AY13" s="7"/>
+      <c r="BA13" s="7"/>
+      <c r="BF13" s="7"/>
+      <c r="BK13" s="7"/>
+    </row>
+    <row r="14" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>1991</v>
       </c>
@@ -1809,37 +1857,38 @@
       <c r="R14" s="5"/>
       <c r="S14" s="5"/>
       <c r="T14" s="5"/>
-      <c r="U14" s="7"/>
+      <c r="U14" s="5"/>
       <c r="V14" s="7"/>
       <c r="W14" s="7"/>
       <c r="X14" s="7"/>
       <c r="Y14" s="7"/>
-      <c r="Z14" s="8"/>
+      <c r="Z14" s="7"/>
       <c r="AA14" s="8"/>
       <c r="AB14" s="8"/>
       <c r="AC14" s="8"/>
       <c r="AD14" s="8"/>
-      <c r="AE14" s="7"/>
+      <c r="AE14" s="8"/>
       <c r="AF14" s="7"/>
       <c r="AG14" s="7"/>
       <c r="AH14" s="7"/>
       <c r="AI14" s="7"/>
       <c r="AJ14" s="7"/>
-      <c r="AK14" s="9"/>
-      <c r="AM14" s="7"/>
+      <c r="AK14" s="7"/>
+      <c r="AL14" s="9"/>
       <c r="AN14" s="7"/>
       <c r="AO14" s="7"/>
       <c r="AP14" s="7"/>
       <c r="AQ14" s="7"/>
       <c r="AR14" s="7"/>
-      <c r="AT14" s="7"/>
-      <c r="AV14" s="7"/>
-      <c r="AX14" s="7"/>
-      <c r="AZ14" s="7"/>
-      <c r="BE14" s="7"/>
-      <c r="BJ14" s="7"/>
-    </row>
-    <row r="15" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS14" s="7"/>
+      <c r="AU14" s="7"/>
+      <c r="AW14" s="7"/>
+      <c r="AY14" s="7"/>
+      <c r="BA14" s="7"/>
+      <c r="BF14" s="7"/>
+      <c r="BK14" s="7"/>
+    </row>
+    <row r="15" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>1992</v>
       </c>
@@ -1872,8 +1921,8 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N15" s="1">
-        <v>0</v>
+      <c r="N15" s="36">
+        <v>3405</v>
       </c>
       <c r="O15" s="7">
         <v>11361</v>
@@ -1887,37 +1936,38 @@
       <c r="R15" s="5"/>
       <c r="S15" s="5"/>
       <c r="T15" s="5"/>
-      <c r="U15" s="7"/>
+      <c r="U15" s="5"/>
       <c r="V15" s="7"/>
       <c r="W15" s="7"/>
       <c r="X15" s="7"/>
       <c r="Y15" s="7"/>
-      <c r="Z15" s="8"/>
+      <c r="Z15" s="7"/>
       <c r="AA15" s="8"/>
       <c r="AB15" s="8"/>
       <c r="AC15" s="8"/>
       <c r="AD15" s="8"/>
-      <c r="AE15" s="7"/>
+      <c r="AE15" s="8"/>
       <c r="AF15" s="7"/>
       <c r="AG15" s="7"/>
       <c r="AH15" s="7"/>
       <c r="AI15" s="7"/>
       <c r="AJ15" s="7"/>
-      <c r="AK15" s="9"/>
-      <c r="AM15" s="7"/>
+      <c r="AK15" s="7"/>
+      <c r="AL15" s="9"/>
       <c r="AN15" s="7"/>
       <c r="AO15" s="7"/>
       <c r="AP15" s="7"/>
       <c r="AQ15" s="7"/>
       <c r="AR15" s="7"/>
-      <c r="AT15" s="7"/>
-      <c r="AV15" s="7"/>
-      <c r="AX15" s="7"/>
-      <c r="AZ15" s="7"/>
-      <c r="BE15" s="7"/>
-      <c r="BJ15" s="7"/>
-    </row>
-    <row r="16" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS15" s="7"/>
+      <c r="AU15" s="7"/>
+      <c r="AW15" s="7"/>
+      <c r="AY15" s="7"/>
+      <c r="BA15" s="7"/>
+      <c r="BF15" s="7"/>
+      <c r="BK15" s="7"/>
+    </row>
+    <row r="16" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>1993</v>
       </c>
@@ -1965,37 +2015,38 @@
       <c r="R16" s="5"/>
       <c r="S16" s="5"/>
       <c r="T16" s="5"/>
-      <c r="U16" s="7"/>
+      <c r="U16" s="5"/>
       <c r="V16" s="7"/>
       <c r="W16" s="7"/>
       <c r="X16" s="7"/>
       <c r="Y16" s="7"/>
-      <c r="Z16" s="8"/>
+      <c r="Z16" s="7"/>
       <c r="AA16" s="8"/>
       <c r="AB16" s="8"/>
       <c r="AC16" s="8"/>
       <c r="AD16" s="8"/>
-      <c r="AE16" s="7"/>
+      <c r="AE16" s="8"/>
       <c r="AF16" s="7"/>
       <c r="AG16" s="7"/>
       <c r="AH16" s="7"/>
       <c r="AI16" s="7"/>
       <c r="AJ16" s="7"/>
-      <c r="AK16" s="9"/>
-      <c r="AM16" s="7"/>
+      <c r="AK16" s="7"/>
+      <c r="AL16" s="9"/>
       <c r="AN16" s="7"/>
       <c r="AO16" s="7"/>
       <c r="AP16" s="7"/>
       <c r="AQ16" s="7"/>
       <c r="AR16" s="7"/>
-      <c r="AT16" s="7"/>
-      <c r="AV16" s="7"/>
-      <c r="AX16" s="7"/>
-      <c r="AZ16" s="7"/>
-      <c r="BE16" s="7"/>
-      <c r="BJ16" s="7"/>
-    </row>
-    <row r="17" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS16" s="7"/>
+      <c r="AU16" s="7"/>
+      <c r="AW16" s="7"/>
+      <c r="AY16" s="7"/>
+      <c r="BA16" s="7"/>
+      <c r="BF16" s="7"/>
+      <c r="BK16" s="7"/>
+    </row>
+    <row r="17" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>1994</v>
       </c>
@@ -2043,37 +2094,38 @@
       <c r="R17" s="5"/>
       <c r="S17" s="5"/>
       <c r="T17" s="5"/>
-      <c r="U17" s="7"/>
+      <c r="U17" s="5"/>
       <c r="V17" s="7"/>
       <c r="W17" s="7"/>
       <c r="X17" s="7"/>
       <c r="Y17" s="7"/>
-      <c r="Z17" s="8"/>
+      <c r="Z17" s="7"/>
       <c r="AA17" s="8"/>
       <c r="AB17" s="8"/>
       <c r="AC17" s="8"/>
       <c r="AD17" s="8"/>
-      <c r="AE17" s="7"/>
+      <c r="AE17" s="8"/>
       <c r="AF17" s="7"/>
       <c r="AG17" s="7"/>
       <c r="AH17" s="7"/>
       <c r="AI17" s="7"/>
       <c r="AJ17" s="7"/>
-      <c r="AK17" s="9"/>
-      <c r="AM17" s="7"/>
+      <c r="AK17" s="7"/>
+      <c r="AL17" s="9"/>
       <c r="AN17" s="7"/>
       <c r="AO17" s="7"/>
       <c r="AP17" s="7"/>
       <c r="AQ17" s="7"/>
       <c r="AR17" s="7"/>
-      <c r="AT17" s="7"/>
-      <c r="AV17" s="7"/>
-      <c r="AX17" s="7"/>
-      <c r="AZ17" s="7"/>
-      <c r="BE17" s="7"/>
-      <c r="BJ17" s="7"/>
-    </row>
-    <row r="18" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS17" s="7"/>
+      <c r="AU17" s="7"/>
+      <c r="AW17" s="7"/>
+      <c r="AY17" s="7"/>
+      <c r="BA17" s="7"/>
+      <c r="BF17" s="7"/>
+      <c r="BK17" s="7"/>
+    </row>
+    <row r="18" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>1995</v>
       </c>
@@ -2121,37 +2173,38 @@
       <c r="R18" s="5"/>
       <c r="S18" s="5"/>
       <c r="T18" s="5"/>
-      <c r="U18" s="7"/>
+      <c r="U18" s="5"/>
       <c r="V18" s="7"/>
       <c r="W18" s="7"/>
       <c r="X18" s="7"/>
       <c r="Y18" s="7"/>
-      <c r="Z18" s="8"/>
+      <c r="Z18" s="7"/>
       <c r="AA18" s="8"/>
       <c r="AB18" s="8"/>
       <c r="AC18" s="8"/>
       <c r="AD18" s="8"/>
-      <c r="AE18" s="7"/>
+      <c r="AE18" s="8"/>
       <c r="AF18" s="7"/>
       <c r="AG18" s="7"/>
       <c r="AH18" s="7"/>
       <c r="AI18" s="7"/>
       <c r="AJ18" s="7"/>
-      <c r="AK18" s="9"/>
-      <c r="AM18" s="7"/>
+      <c r="AK18" s="7"/>
+      <c r="AL18" s="9"/>
       <c r="AN18" s="7"/>
       <c r="AO18" s="7"/>
       <c r="AP18" s="7"/>
       <c r="AQ18" s="7"/>
       <c r="AR18" s="7"/>
-      <c r="AT18" s="7"/>
-      <c r="AV18" s="7"/>
-      <c r="AX18" s="7"/>
-      <c r="AZ18" s="7"/>
-      <c r="BE18" s="7"/>
-      <c r="BJ18" s="7"/>
-    </row>
-    <row r="19" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS18" s="7"/>
+      <c r="AU18" s="7"/>
+      <c r="AW18" s="7"/>
+      <c r="AY18" s="7"/>
+      <c r="BA18" s="7"/>
+      <c r="BF18" s="7"/>
+      <c r="BK18" s="7"/>
+    </row>
+    <row r="19" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>1996</v>
       </c>
@@ -2199,37 +2252,38 @@
       <c r="R19" s="5"/>
       <c r="S19" s="5"/>
       <c r="T19" s="5"/>
-      <c r="U19" s="7"/>
+      <c r="U19" s="5"/>
       <c r="V19" s="7"/>
       <c r="W19" s="7"/>
       <c r="X19" s="7"/>
       <c r="Y19" s="7"/>
-      <c r="Z19" s="8"/>
+      <c r="Z19" s="7"/>
       <c r="AA19" s="8"/>
       <c r="AB19" s="8"/>
       <c r="AC19" s="8"/>
       <c r="AD19" s="8"/>
-      <c r="AE19" s="7"/>
+      <c r="AE19" s="8"/>
       <c r="AF19" s="7"/>
       <c r="AG19" s="7"/>
       <c r="AH19" s="7"/>
       <c r="AI19" s="7"/>
       <c r="AJ19" s="7"/>
-      <c r="AK19" s="9"/>
-      <c r="AM19" s="7"/>
+      <c r="AK19" s="7"/>
+      <c r="AL19" s="9"/>
       <c r="AN19" s="7"/>
       <c r="AO19" s="7"/>
       <c r="AP19" s="7"/>
       <c r="AQ19" s="7"/>
       <c r="AR19" s="7"/>
-      <c r="AT19" s="7"/>
-      <c r="AV19" s="7"/>
-      <c r="AX19" s="7"/>
-      <c r="AZ19" s="7"/>
-      <c r="BE19" s="7"/>
-      <c r="BJ19" s="7"/>
-    </row>
-    <row r="20" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS19" s="7"/>
+      <c r="AU19" s="7"/>
+      <c r="AW19" s="7"/>
+      <c r="AY19" s="7"/>
+      <c r="BA19" s="7"/>
+      <c r="BF19" s="7"/>
+      <c r="BK19" s="7"/>
+    </row>
+    <row r="20" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>1997</v>
       </c>
@@ -2274,36 +2328,37 @@
       <c r="R20" s="5"/>
       <c r="S20" s="5"/>
       <c r="T20" s="5"/>
-      <c r="U20" s="7"/>
+      <c r="U20" s="5"/>
       <c r="V20" s="7"/>
       <c r="W20" s="7"/>
       <c r="X20" s="7"/>
       <c r="Y20" s="7"/>
-      <c r="Z20" s="8"/>
+      <c r="Z20" s="7"/>
       <c r="AA20" s="8"/>
       <c r="AB20" s="8"/>
       <c r="AC20" s="8"/>
       <c r="AD20" s="8"/>
-      <c r="AE20" s="7"/>
+      <c r="AE20" s="8"/>
       <c r="AF20" s="7"/>
       <c r="AG20" s="7"/>
       <c r="AH20" s="7"/>
       <c r="AI20" s="7"/>
       <c r="AJ20" s="7"/>
-      <c r="AM20" s="7"/>
+      <c r="AK20" s="7"/>
       <c r="AN20" s="7"/>
       <c r="AO20" s="7"/>
       <c r="AP20" s="7"/>
       <c r="AQ20" s="7"/>
       <c r="AR20" s="7"/>
-      <c r="AT20" s="7"/>
-      <c r="AV20" s="7"/>
-      <c r="AX20" s="7"/>
-      <c r="AZ20" s="7"/>
-      <c r="BE20" s="7"/>
-      <c r="BJ20" s="7"/>
-    </row>
-    <row r="21" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS20" s="7"/>
+      <c r="AU20" s="7"/>
+      <c r="AW20" s="7"/>
+      <c r="AY20" s="7"/>
+      <c r="BA20" s="7"/>
+      <c r="BF20" s="7"/>
+      <c r="BK20" s="7"/>
+    </row>
+    <row r="21" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>1998</v>
       </c>
@@ -2348,36 +2403,37 @@
       <c r="R21" s="5"/>
       <c r="S21" s="5"/>
       <c r="T21" s="5"/>
-      <c r="U21" s="7"/>
+      <c r="U21" s="5"/>
       <c r="V21" s="7"/>
       <c r="W21" s="7"/>
       <c r="X21" s="7"/>
       <c r="Y21" s="7"/>
-      <c r="Z21" s="8"/>
+      <c r="Z21" s="7"/>
       <c r="AA21" s="8"/>
       <c r="AB21" s="8"/>
       <c r="AC21" s="8"/>
       <c r="AD21" s="8"/>
-      <c r="AE21" s="7"/>
+      <c r="AE21" s="8"/>
       <c r="AF21" s="7"/>
       <c r="AG21" s="7"/>
       <c r="AH21" s="7"/>
       <c r="AI21" s="7"/>
       <c r="AJ21" s="7"/>
-      <c r="AM21" s="7"/>
+      <c r="AK21" s="7"/>
       <c r="AN21" s="7"/>
       <c r="AO21" s="7"/>
       <c r="AP21" s="7"/>
       <c r="AQ21" s="7"/>
       <c r="AR21" s="7"/>
-      <c r="AT21" s="7"/>
-      <c r="AV21" s="7"/>
-      <c r="AX21" s="7"/>
-      <c r="AZ21" s="7"/>
-      <c r="BE21" s="7"/>
-      <c r="BJ21" s="7"/>
-    </row>
-    <row r="22" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS21" s="7"/>
+      <c r="AU21" s="7"/>
+      <c r="AW21" s="7"/>
+      <c r="AY21" s="7"/>
+      <c r="BA21" s="7"/>
+      <c r="BF21" s="7"/>
+      <c r="BK21" s="7"/>
+    </row>
+    <row r="22" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>1999</v>
       </c>
@@ -2422,36 +2478,37 @@
       <c r="R22" s="5"/>
       <c r="S22" s="5"/>
       <c r="T22" s="5"/>
-      <c r="U22" s="7"/>
+      <c r="U22" s="5"/>
       <c r="V22" s="7"/>
       <c r="W22" s="7"/>
       <c r="X22" s="7"/>
       <c r="Y22" s="7"/>
-      <c r="Z22" s="8"/>
+      <c r="Z22" s="7"/>
       <c r="AA22" s="8"/>
       <c r="AB22" s="8"/>
       <c r="AC22" s="8"/>
       <c r="AD22" s="8"/>
-      <c r="AE22" s="7"/>
+      <c r="AE22" s="8"/>
       <c r="AF22" s="7"/>
       <c r="AG22" s="7"/>
       <c r="AH22" s="7"/>
       <c r="AI22" s="7"/>
       <c r="AJ22" s="7"/>
-      <c r="AM22" s="7"/>
+      <c r="AK22" s="7"/>
       <c r="AN22" s="7"/>
       <c r="AO22" s="7"/>
       <c r="AP22" s="7"/>
       <c r="AQ22" s="7"/>
       <c r="AR22" s="7"/>
-      <c r="AT22" s="7"/>
-      <c r="AV22" s="7"/>
-      <c r="AX22" s="7"/>
-      <c r="AZ22" s="7"/>
-      <c r="BE22" s="7"/>
-      <c r="BJ22" s="7"/>
-    </row>
-    <row r="23" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS22" s="7"/>
+      <c r="AU22" s="7"/>
+      <c r="AW22" s="7"/>
+      <c r="AY22" s="7"/>
+      <c r="BA22" s="7"/>
+      <c r="BF22" s="7"/>
+      <c r="BK22" s="7"/>
+    </row>
+    <row r="23" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>2000</v>
       </c>
@@ -2496,36 +2553,37 @@
       <c r="R23" s="5"/>
       <c r="S23" s="5"/>
       <c r="T23" s="5"/>
-      <c r="U23" s="7"/>
+      <c r="U23" s="5"/>
       <c r="V23" s="7"/>
       <c r="W23" s="7"/>
       <c r="X23" s="7"/>
       <c r="Y23" s="7"/>
-      <c r="Z23" s="8"/>
+      <c r="Z23" s="7"/>
       <c r="AA23" s="8"/>
       <c r="AB23" s="8"/>
       <c r="AC23" s="8"/>
       <c r="AD23" s="8"/>
-      <c r="AE23" s="7"/>
+      <c r="AE23" s="8"/>
       <c r="AF23" s="7"/>
       <c r="AG23" s="7"/>
       <c r="AH23" s="7"/>
       <c r="AI23" s="7"/>
       <c r="AJ23" s="7"/>
-      <c r="AM23" s="7"/>
+      <c r="AK23" s="7"/>
       <c r="AN23" s="7"/>
       <c r="AO23" s="7"/>
       <c r="AP23" s="7"/>
       <c r="AQ23" s="7"/>
       <c r="AR23" s="7"/>
-      <c r="AT23" s="7"/>
-      <c r="AV23" s="7"/>
-      <c r="AX23" s="7"/>
-      <c r="AZ23" s="7"/>
-      <c r="BE23" s="7"/>
-      <c r="BJ23" s="7"/>
-    </row>
-    <row r="24" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS23" s="7"/>
+      <c r="AU23" s="7"/>
+      <c r="AW23" s="7"/>
+      <c r="AY23" s="7"/>
+      <c r="BA23" s="7"/>
+      <c r="BF23" s="7"/>
+      <c r="BK23" s="7"/>
+    </row>
+    <row r="24" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>2001</v>
       </c>
@@ -2568,40 +2626,41 @@
       </c>
       <c r="Q24" s="31"/>
       <c r="R24" s="5"/>
-      <c r="S24" s="5" t="s">
+      <c r="S24" s="5"/>
+      <c r="T24" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="T24" s="5"/>
-      <c r="U24" s="7"/>
+      <c r="U24" s="5"/>
       <c r="V24" s="7"/>
       <c r="W24" s="7"/>
       <c r="X24" s="7"/>
       <c r="Y24" s="7"/>
-      <c r="Z24" s="8"/>
+      <c r="Z24" s="7"/>
       <c r="AA24" s="8"/>
       <c r="AB24" s="8"/>
       <c r="AC24" s="8"/>
       <c r="AD24" s="8"/>
-      <c r="AE24" s="7"/>
+      <c r="AE24" s="8"/>
       <c r="AF24" s="7"/>
       <c r="AG24" s="7"/>
       <c r="AH24" s="7"/>
       <c r="AI24" s="7"/>
       <c r="AJ24" s="7"/>
-      <c r="AM24" s="7"/>
+      <c r="AK24" s="7"/>
       <c r="AN24" s="7"/>
       <c r="AO24" s="7"/>
       <c r="AP24" s="7"/>
       <c r="AQ24" s="7"/>
       <c r="AR24" s="7"/>
-      <c r="AT24" s="7"/>
-      <c r="AV24" s="7"/>
-      <c r="AX24" s="7"/>
-      <c r="AZ24" s="7"/>
-      <c r="BE24" s="7"/>
-      <c r="BJ24" s="7"/>
-    </row>
-    <row r="25" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS24" s="7"/>
+      <c r="AU24" s="7"/>
+      <c r="AW24" s="7"/>
+      <c r="AY24" s="7"/>
+      <c r="BA24" s="7"/>
+      <c r="BF24" s="7"/>
+      <c r="BK24" s="7"/>
+    </row>
+    <row r="25" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>2002</v>
       </c>
@@ -2649,36 +2708,37 @@
       </c>
       <c r="S25" s="5"/>
       <c r="T25" s="5"/>
-      <c r="U25" s="7"/>
+      <c r="U25" s="5"/>
       <c r="V25" s="7"/>
       <c r="W25" s="7"/>
       <c r="X25" s="7"/>
       <c r="Y25" s="7"/>
-      <c r="Z25" s="8"/>
+      <c r="Z25" s="7"/>
       <c r="AA25" s="8"/>
       <c r="AB25" s="8"/>
       <c r="AC25" s="8"/>
       <c r="AD25" s="8"/>
-      <c r="AE25" s="7"/>
+      <c r="AE25" s="8"/>
       <c r="AF25" s="7"/>
       <c r="AG25" s="7"/>
       <c r="AH25" s="7"/>
       <c r="AI25" s="7"/>
       <c r="AJ25" s="7"/>
-      <c r="AM25" s="7"/>
+      <c r="AK25" s="7"/>
       <c r="AN25" s="7"/>
       <c r="AO25" s="7"/>
       <c r="AP25" s="7"/>
       <c r="AQ25" s="7"/>
       <c r="AR25" s="7"/>
-      <c r="AT25" s="7"/>
-      <c r="AV25" s="7"/>
-      <c r="AX25" s="7"/>
-      <c r="AZ25" s="7"/>
-      <c r="BE25" s="7"/>
-      <c r="BJ25" s="7"/>
-    </row>
-    <row r="26" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS25" s="7"/>
+      <c r="AU25" s="7"/>
+      <c r="AW25" s="7"/>
+      <c r="AY25" s="7"/>
+      <c r="BA25" s="7"/>
+      <c r="BF25" s="7"/>
+      <c r="BK25" s="7"/>
+    </row>
+    <row r="26" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>2003</v>
       </c>
@@ -2735,36 +2795,37 @@
       </c>
       <c r="S26" s="5"/>
       <c r="T26" s="5"/>
-      <c r="U26" s="7"/>
+      <c r="U26" s="5"/>
       <c r="V26" s="7"/>
       <c r="W26" s="7"/>
       <c r="X26" s="7"/>
       <c r="Y26" s="7"/>
-      <c r="Z26" s="8"/>
+      <c r="Z26" s="7"/>
       <c r="AA26" s="8"/>
       <c r="AB26" s="8"/>
       <c r="AC26" s="8"/>
       <c r="AD26" s="8"/>
-      <c r="AE26" s="7"/>
+      <c r="AE26" s="8"/>
       <c r="AF26" s="7"/>
       <c r="AG26" s="7"/>
       <c r="AH26" s="7"/>
       <c r="AI26" s="7"/>
       <c r="AJ26" s="7"/>
-      <c r="AM26" s="7"/>
+      <c r="AK26" s="7"/>
       <c r="AN26" s="7"/>
       <c r="AO26" s="7"/>
       <c r="AP26" s="7"/>
       <c r="AQ26" s="7"/>
       <c r="AR26" s="7"/>
-      <c r="AT26" s="7"/>
-      <c r="AV26" s="7"/>
-      <c r="AX26" s="7"/>
-      <c r="AZ26" s="7"/>
-      <c r="BE26" s="7"/>
-      <c r="BJ26" s="7"/>
-    </row>
-    <row r="27" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS26" s="7"/>
+      <c r="AU26" s="7"/>
+      <c r="AW26" s="7"/>
+      <c r="AY26" s="7"/>
+      <c r="BA26" s="7"/>
+      <c r="BF26" s="7"/>
+      <c r="BK26" s="7"/>
+    </row>
+    <row r="27" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>2004</v>
       </c>
@@ -2809,36 +2870,37 @@
       <c r="R27" s="5"/>
       <c r="S27" s="5"/>
       <c r="T27" s="5"/>
-      <c r="U27" s="7"/>
+      <c r="U27" s="5"/>
       <c r="V27" s="7"/>
       <c r="W27" s="7"/>
       <c r="X27" s="7"/>
       <c r="Y27" s="7"/>
-      <c r="Z27" s="8"/>
+      <c r="Z27" s="7"/>
       <c r="AA27" s="8"/>
       <c r="AB27" s="8"/>
       <c r="AC27" s="8"/>
       <c r="AD27" s="8"/>
-      <c r="AE27" s="7"/>
+      <c r="AE27" s="8"/>
       <c r="AF27" s="7"/>
       <c r="AG27" s="7"/>
       <c r="AH27" s="7"/>
       <c r="AI27" s="7"/>
       <c r="AJ27" s="7"/>
-      <c r="AM27" s="7"/>
+      <c r="AK27" s="7"/>
       <c r="AN27" s="7"/>
       <c r="AO27" s="7"/>
       <c r="AP27" s="7"/>
       <c r="AQ27" s="7"/>
       <c r="AR27" s="7"/>
-      <c r="AT27" s="7"/>
-      <c r="AV27" s="7"/>
-      <c r="AX27" s="7"/>
-      <c r="AZ27" s="7"/>
-      <c r="BE27" s="7"/>
-      <c r="BJ27" s="7"/>
-    </row>
-    <row r="28" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS27" s="7"/>
+      <c r="AU27" s="7"/>
+      <c r="AW27" s="7"/>
+      <c r="AY27" s="7"/>
+      <c r="BA27" s="7"/>
+      <c r="BF27" s="7"/>
+      <c r="BK27" s="7"/>
+    </row>
+    <row r="28" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>2005</v>
       </c>
@@ -2863,7 +2925,7 @@
         <v>1000</v>
       </c>
       <c r="L28" s="7">
-        <f t="shared" ref="L24:L35" si="5">SUM(F28,H28,I28)</f>
+        <f t="shared" ref="L28:L32" si="5">SUM(F28,H28,I28)</f>
         <v>2500</v>
       </c>
       <c r="M28" s="23">
@@ -2883,36 +2945,37 @@
       <c r="R28" s="5"/>
       <c r="S28" s="5"/>
       <c r="T28" s="5"/>
-      <c r="U28" s="7"/>
+      <c r="U28" s="5"/>
       <c r="V28" s="7"/>
       <c r="W28" s="7"/>
       <c r="X28" s="7"/>
       <c r="Y28" s="7"/>
-      <c r="Z28" s="8"/>
+      <c r="Z28" s="7"/>
       <c r="AA28" s="8"/>
       <c r="AB28" s="8"/>
       <c r="AC28" s="8"/>
       <c r="AD28" s="8"/>
-      <c r="AE28" s="7"/>
+      <c r="AE28" s="8"/>
       <c r="AF28" s="7"/>
       <c r="AG28" s="7"/>
       <c r="AH28" s="7"/>
       <c r="AI28" s="7"/>
       <c r="AJ28" s="7"/>
-      <c r="AM28" s="7"/>
+      <c r="AK28" s="7"/>
       <c r="AN28" s="7"/>
       <c r="AO28" s="7"/>
       <c r="AP28" s="7"/>
       <c r="AQ28" s="7"/>
       <c r="AR28" s="7"/>
-      <c r="AT28" s="7"/>
-      <c r="AV28" s="7"/>
-      <c r="AX28" s="7"/>
-      <c r="AZ28" s="7"/>
-      <c r="BE28" s="7"/>
-      <c r="BJ28" s="7"/>
-    </row>
-    <row r="29" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS28" s="7"/>
+      <c r="AU28" s="7"/>
+      <c r="AW28" s="7"/>
+      <c r="AY28" s="7"/>
+      <c r="BA28" s="7"/>
+      <c r="BF28" s="7"/>
+      <c r="BK28" s="7"/>
+    </row>
+    <row r="29" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>2006</v>
       </c>
@@ -2957,36 +3020,37 @@
       <c r="R29" s="5"/>
       <c r="S29" s="5"/>
       <c r="T29" s="5"/>
-      <c r="U29" s="7"/>
+      <c r="U29" s="5"/>
       <c r="V29" s="7"/>
       <c r="W29" s="7"/>
       <c r="X29" s="7"/>
       <c r="Y29" s="7"/>
-      <c r="Z29" s="8"/>
+      <c r="Z29" s="7"/>
       <c r="AA29" s="8"/>
       <c r="AB29" s="8"/>
       <c r="AC29" s="8"/>
       <c r="AD29" s="8"/>
-      <c r="AE29" s="7"/>
+      <c r="AE29" s="8"/>
       <c r="AF29" s="7"/>
       <c r="AG29" s="7"/>
       <c r="AH29" s="7"/>
       <c r="AI29" s="7"/>
       <c r="AJ29" s="7"/>
-      <c r="AM29" s="7"/>
+      <c r="AK29" s="7"/>
       <c r="AN29" s="7"/>
       <c r="AO29" s="7"/>
       <c r="AP29" s="7"/>
       <c r="AQ29" s="7"/>
       <c r="AR29" s="7"/>
-      <c r="AT29" s="7"/>
-      <c r="AV29" s="7"/>
-      <c r="AX29" s="7"/>
-      <c r="AZ29" s="7"/>
-      <c r="BE29" s="7"/>
-      <c r="BJ29" s="7"/>
-    </row>
-    <row r="30" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS29" s="7"/>
+      <c r="AU29" s="7"/>
+      <c r="AW29" s="7"/>
+      <c r="AY29" s="7"/>
+      <c r="BA29" s="7"/>
+      <c r="BF29" s="7"/>
+      <c r="BK29" s="7"/>
+    </row>
+    <row r="30" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>2007</v>
       </c>
@@ -3012,7 +3076,7 @@
         <v>500</v>
       </c>
       <c r="L30" s="7">
-        <f t="shared" si="5"/>
+        <f>SUM(F30,H30,I30)</f>
         <v>500</v>
       </c>
       <c r="M30" s="23">
@@ -3032,36 +3096,37 @@
       <c r="R30" s="5"/>
       <c r="S30" s="5"/>
       <c r="T30" s="5"/>
-      <c r="U30" s="7"/>
+      <c r="U30" s="5"/>
       <c r="V30" s="7"/>
       <c r="W30" s="7"/>
       <c r="X30" s="7"/>
       <c r="Y30" s="7"/>
-      <c r="Z30" s="8"/>
+      <c r="Z30" s="7"/>
       <c r="AA30" s="8"/>
       <c r="AB30" s="8"/>
       <c r="AC30" s="8"/>
       <c r="AD30" s="8"/>
-      <c r="AE30" s="7"/>
+      <c r="AE30" s="8"/>
       <c r="AF30" s="7"/>
       <c r="AG30" s="7"/>
       <c r="AH30" s="7"/>
       <c r="AI30" s="7"/>
       <c r="AJ30" s="7"/>
-      <c r="AM30" s="7"/>
+      <c r="AK30" s="7"/>
       <c r="AN30" s="7"/>
       <c r="AO30" s="7"/>
       <c r="AP30" s="7"/>
       <c r="AQ30" s="7"/>
       <c r="AR30" s="7"/>
-      <c r="AT30" s="7"/>
-      <c r="AV30" s="7"/>
-      <c r="AX30" s="7"/>
-      <c r="AZ30" s="7"/>
-      <c r="BE30" s="7"/>
-      <c r="BJ30" s="7"/>
-    </row>
-    <row r="31" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS30" s="7"/>
+      <c r="AU30" s="7"/>
+      <c r="AW30" s="7"/>
+      <c r="AY30" s="7"/>
+      <c r="BA30" s="7"/>
+      <c r="BF30" s="7"/>
+      <c r="BK30" s="7"/>
+    </row>
+    <row r="31" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>2008</v>
       </c>
@@ -3106,36 +3171,37 @@
       <c r="R31" s="5"/>
       <c r="S31" s="5"/>
       <c r="T31" s="5"/>
-      <c r="U31" s="7"/>
+      <c r="U31" s="5"/>
       <c r="V31" s="7"/>
       <c r="W31" s="7"/>
       <c r="X31" s="7"/>
       <c r="Y31" s="7"/>
-      <c r="Z31" s="8"/>
+      <c r="Z31" s="7"/>
       <c r="AA31" s="8"/>
       <c r="AB31" s="8"/>
       <c r="AC31" s="8"/>
       <c r="AD31" s="8"/>
-      <c r="AE31" s="7"/>
+      <c r="AE31" s="8"/>
       <c r="AF31" s="7"/>
       <c r="AG31" s="7"/>
       <c r="AH31" s="7"/>
       <c r="AI31" s="7"/>
       <c r="AJ31" s="7"/>
-      <c r="AM31" s="7"/>
+      <c r="AK31" s="7"/>
       <c r="AN31" s="7"/>
       <c r="AO31" s="7"/>
       <c r="AP31" s="7"/>
       <c r="AQ31" s="7"/>
       <c r="AR31" s="7"/>
-      <c r="AT31" s="7"/>
-      <c r="AV31" s="7"/>
-      <c r="AX31" s="7"/>
-      <c r="AZ31" s="7"/>
-      <c r="BE31" s="7"/>
-      <c r="BJ31" s="7"/>
-    </row>
-    <row r="32" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS31" s="7"/>
+      <c r="AU31" s="7"/>
+      <c r="AW31" s="7"/>
+      <c r="AY31" s="7"/>
+      <c r="BA31" s="7"/>
+      <c r="BF31" s="7"/>
+      <c r="BK31" s="7"/>
+    </row>
+    <row r="32" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
         <v>2009</v>
       </c>
@@ -3180,36 +3246,37 @@
       <c r="R32" s="5"/>
       <c r="S32" s="5"/>
       <c r="T32" s="5"/>
-      <c r="U32" s="7"/>
+      <c r="U32" s="5"/>
       <c r="V32" s="7"/>
       <c r="W32" s="7"/>
       <c r="X32" s="7"/>
       <c r="Y32" s="7"/>
-      <c r="Z32" s="8"/>
+      <c r="Z32" s="7"/>
       <c r="AA32" s="8"/>
       <c r="AB32" s="8"/>
       <c r="AC32" s="8"/>
       <c r="AD32" s="8"/>
-      <c r="AE32" s="7"/>
+      <c r="AE32" s="8"/>
       <c r="AF32" s="7"/>
       <c r="AG32" s="7"/>
       <c r="AH32" s="7"/>
       <c r="AI32" s="7"/>
       <c r="AJ32" s="7"/>
-      <c r="AM32" s="7"/>
+      <c r="AK32" s="7"/>
       <c r="AN32" s="7"/>
       <c r="AO32" s="7"/>
       <c r="AP32" s="7"/>
       <c r="AQ32" s="7"/>
       <c r="AR32" s="7"/>
-      <c r="AT32" s="7"/>
-      <c r="AV32" s="7"/>
-      <c r="AX32" s="7"/>
-      <c r="AZ32" s="7"/>
-      <c r="BE32" s="7"/>
-      <c r="BJ32" s="7"/>
-    </row>
-    <row r="33" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS32" s="7"/>
+      <c r="AU32" s="7"/>
+      <c r="AW32" s="7"/>
+      <c r="AY32" s="7"/>
+      <c r="BA32" s="7"/>
+      <c r="BF32" s="7"/>
+      <c r="BK32" s="7"/>
+    </row>
+    <row r="33" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>2010</v>
       </c>
@@ -3224,23 +3291,25 @@
         <v>1043</v>
       </c>
       <c r="E33" s="11">
-        <f t="shared" ref="E33:E45" si="6">SUM(F33:I33)</f>
-        <v>2821</v>
+        <f t="shared" ref="E33:E41" si="6">SUM(F33:I33)</f>
+        <v>2820</v>
       </c>
       <c r="F33" s="11">
-        <v>2351</v>
+        <v>2350</v>
       </c>
       <c r="G33" s="14">
         <f>ROUND(0.2*SUM(F33,H33,I33),0)</f>
         <v>470</v>
       </c>
+      <c r="J33" s="7"/>
+      <c r="K33" s="7"/>
       <c r="L33" s="7">
         <f>SUM(F33,H33,I33)</f>
-        <v>2351</v>
+        <v>2350</v>
       </c>
       <c r="M33" s="23">
-        <f>SUM(J33,K33)</f>
-        <v>0</v>
+        <f>2720-F33</f>
+        <v>370</v>
       </c>
       <c r="N33" s="1">
         <v>124</v>
@@ -3251,42 +3320,45 @@
       <c r="P33" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q33" s="31"/>
+      <c r="Q33" s="34" t="s">
+        <v>51</v>
+      </c>
       <c r="R33" s="5"/>
-      <c r="S33" s="5" t="s">
+      <c r="S33" s="5"/>
+      <c r="T33" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="T33" s="5"/>
-      <c r="U33" s="7"/>
+      <c r="U33" s="5"/>
       <c r="V33" s="7"/>
       <c r="W33" s="7"/>
       <c r="X33" s="7"/>
       <c r="Y33" s="7"/>
-      <c r="Z33" s="8"/>
+      <c r="Z33" s="7"/>
       <c r="AA33" s="8"/>
       <c r="AB33" s="8"/>
       <c r="AC33" s="8"/>
       <c r="AD33" s="8"/>
-      <c r="AE33" s="7"/>
+      <c r="AE33" s="8"/>
       <c r="AF33" s="7"/>
       <c r="AG33" s="7"/>
       <c r="AH33" s="7"/>
       <c r="AI33" s="7"/>
       <c r="AJ33" s="7"/>
-      <c r="AM33" s="7"/>
+      <c r="AK33" s="7"/>
       <c r="AN33" s="7"/>
       <c r="AO33" s="7"/>
       <c r="AP33" s="7"/>
       <c r="AQ33" s="7"/>
       <c r="AR33" s="7"/>
-      <c r="AT33" s="7"/>
-      <c r="AV33" s="7"/>
-      <c r="AX33" s="7"/>
-      <c r="AZ33" s="7"/>
-      <c r="BE33" s="7"/>
-      <c r="BJ33" s="7"/>
-    </row>
-    <row r="34" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS33" s="7"/>
+      <c r="AU33" s="7"/>
+      <c r="AW33" s="7"/>
+      <c r="AY33" s="7"/>
+      <c r="BA33" s="7"/>
+      <c r="BF33" s="7"/>
+      <c r="BK33" s="7"/>
+    </row>
+    <row r="34" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>2011</v>
       </c>
@@ -3312,12 +3384,12 @@
         <v>339</v>
       </c>
       <c r="L34" s="7">
-        <f t="shared" si="5"/>
+        <f>SUM(F34,H34,I34)</f>
         <v>1694</v>
       </c>
       <c r="M34" s="23">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f>2540-F34</f>
+        <v>846</v>
       </c>
       <c r="N34" s="1">
         <v>366</v>
@@ -3328,42 +3400,45 @@
       <c r="P34" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q34" s="31"/>
+      <c r="Q34" s="34" t="s">
+        <v>50</v>
+      </c>
       <c r="R34" s="5"/>
-      <c r="S34" s="5" t="s">
+      <c r="S34" s="5"/>
+      <c r="T34" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="T34" s="5"/>
-      <c r="U34" s="7"/>
+      <c r="U34" s="5"/>
       <c r="V34" s="7"/>
       <c r="W34" s="7"/>
       <c r="X34" s="7"/>
       <c r="Y34" s="7"/>
-      <c r="Z34" s="8"/>
+      <c r="Z34" s="7"/>
       <c r="AA34" s="8"/>
       <c r="AB34" s="8"/>
       <c r="AC34" s="8"/>
       <c r="AD34" s="8"/>
-      <c r="AE34" s="7"/>
+      <c r="AE34" s="8"/>
       <c r="AF34" s="7"/>
       <c r="AG34" s="7"/>
       <c r="AH34" s="7"/>
       <c r="AI34" s="7"/>
       <c r="AJ34" s="7"/>
-      <c r="AM34" s="7"/>
+      <c r="AK34" s="7"/>
       <c r="AN34" s="7"/>
       <c r="AO34" s="7"/>
       <c r="AP34" s="7"/>
       <c r="AQ34" s="7"/>
       <c r="AR34" s="7"/>
-      <c r="AT34" s="7"/>
-      <c r="AV34" s="7"/>
-      <c r="AX34" s="7"/>
-      <c r="AZ34" s="7"/>
-      <c r="BE34" s="7"/>
-      <c r="BJ34" s="7"/>
-    </row>
-    <row r="35" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS34" s="7"/>
+      <c r="AU34" s="7"/>
+      <c r="AW34" s="7"/>
+      <c r="AY34" s="7"/>
+      <c r="BA34" s="7"/>
+      <c r="BF34" s="7"/>
+      <c r="BK34" s="7"/>
+    </row>
+    <row r="35" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>2012</v>
       </c>
@@ -3387,18 +3462,26 @@
         <v>135</v>
       </c>
       <c r="H35" s="1">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="I35" s="1">
-        <v>255</v>
+        <v>256</v>
+      </c>
+      <c r="J35" s="1">
+        <f>571-H35</f>
+        <v>151</v>
+      </c>
+      <c r="K35" s="1">
+        <f>387-I35</f>
+        <v>131</v>
       </c>
       <c r="L35" s="7">
-        <f t="shared" si="5"/>
+        <f>SUM(F35,H35,I35)</f>
         <v>676</v>
       </c>
       <c r="M35" s="23">
-        <f>SUM(J35,K35)</f>
-        <v>0</v>
+        <f t="shared" ref="M35:M45" si="7">SUM(J35,K35)</f>
+        <v>282</v>
       </c>
       <c r="N35" s="1">
         <v>175</v>
@@ -3409,44 +3492,47 @@
       <c r="P35" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q35" s="32"/>
+      <c r="Q35" s="30" t="s">
+        <v>52</v>
+      </c>
       <c r="R35" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S35" s="5" t="s">
+      <c r="S35" s="35"/>
+      <c r="T35" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="T35" s="5"/>
-      <c r="U35" s="7"/>
+      <c r="U35" s="5"/>
       <c r="V35" s="7"/>
       <c r="W35" s="7"/>
       <c r="X35" s="7"/>
       <c r="Y35" s="7"/>
-      <c r="Z35" s="8"/>
+      <c r="Z35" s="7"/>
       <c r="AA35" s="8"/>
       <c r="AB35" s="8"/>
       <c r="AC35" s="8"/>
       <c r="AD35" s="8"/>
-      <c r="AE35" s="7"/>
+      <c r="AE35" s="8"/>
       <c r="AF35" s="7"/>
       <c r="AG35" s="7"/>
       <c r="AH35" s="7"/>
       <c r="AI35" s="7"/>
       <c r="AJ35" s="7"/>
-      <c r="AM35" s="7"/>
+      <c r="AK35" s="7"/>
       <c r="AN35" s="7"/>
       <c r="AO35" s="7"/>
       <c r="AP35" s="7"/>
       <c r="AQ35" s="7"/>
       <c r="AR35" s="7"/>
-      <c r="AT35" s="7"/>
-      <c r="AV35" s="7"/>
-      <c r="AX35" s="7"/>
-      <c r="AZ35" s="7"/>
-      <c r="BE35" s="7"/>
-      <c r="BJ35" s="7"/>
-    </row>
-    <row r="36" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS35" s="7"/>
+      <c r="AU35" s="7"/>
+      <c r="AW35" s="7"/>
+      <c r="AY35" s="7"/>
+      <c r="BA35" s="7"/>
+      <c r="BF35" s="7"/>
+      <c r="BK35" s="7"/>
+    </row>
+    <row r="36" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>2013</v>
       </c>
@@ -3462,32 +3548,34 @@
       </c>
       <c r="E36" s="11">
         <f t="shared" si="6"/>
-        <v>2868</v>
+        <v>2834</v>
       </c>
       <c r="F36" s="4"/>
       <c r="G36" s="14">
         <f>ROUND(0.2*SUM(F36,H36,I36),0)</f>
-        <v>478</v>
+        <v>472</v>
       </c>
       <c r="H36" s="1">
-        <v>1552</v>
+        <v>1530</v>
       </c>
       <c r="I36" s="1">
-        <v>838</v>
+        <v>832</v>
       </c>
       <c r="J36" s="1">
-        <v>583</v>
+        <f>1936-H36</f>
+        <v>406</v>
       </c>
       <c r="K36" s="1">
-        <v>375</v>
+        <f>1202-I36</f>
+        <v>370</v>
       </c>
       <c r="L36" s="7">
-        <f t="shared" si="3"/>
-        <v>2390</v>
+        <f>SUM(F36,H36,I36)</f>
+        <v>2362</v>
       </c>
       <c r="M36" s="23">
-        <f>SUM(J36,K36)</f>
-        <v>958</v>
+        <f t="shared" si="7"/>
+        <v>776</v>
       </c>
       <c r="N36" s="1">
         <v>19</v>
@@ -3498,44 +3586,47 @@
       <c r="P36" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q36" s="32"/>
+      <c r="Q36" s="34" t="s">
+        <v>53</v>
+      </c>
       <c r="R36" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S36" s="5" t="s">
+      <c r="S36" s="35"/>
+      <c r="T36" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="T36" s="5"/>
-      <c r="U36" s="7"/>
+      <c r="U36" s="5"/>
       <c r="V36" s="7"/>
       <c r="W36" s="7"/>
       <c r="X36" s="7"/>
       <c r="Y36" s="7"/>
-      <c r="Z36" s="8"/>
+      <c r="Z36" s="7"/>
       <c r="AA36" s="8"/>
       <c r="AB36" s="8"/>
       <c r="AC36" s="8"/>
       <c r="AD36" s="8"/>
-      <c r="AE36" s="7"/>
+      <c r="AE36" s="8"/>
       <c r="AF36" s="7"/>
       <c r="AG36" s="7"/>
       <c r="AH36" s="7"/>
       <c r="AI36" s="7"/>
       <c r="AJ36" s="7"/>
-      <c r="AM36" s="7"/>
+      <c r="AK36" s="7"/>
       <c r="AN36" s="7"/>
       <c r="AO36" s="7"/>
       <c r="AP36" s="7"/>
       <c r="AQ36" s="7"/>
       <c r="AR36" s="7"/>
-      <c r="AT36" s="7"/>
-      <c r="AV36" s="7"/>
-      <c r="AX36" s="7"/>
-      <c r="AZ36" s="7"/>
-      <c r="BE36" s="7"/>
-      <c r="BJ36" s="7"/>
-    </row>
-    <row r="37" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS36" s="7"/>
+      <c r="AU36" s="7"/>
+      <c r="AW36" s="7"/>
+      <c r="AY36" s="7"/>
+      <c r="BA36" s="7"/>
+      <c r="BF36" s="7"/>
+      <c r="BK36" s="7"/>
+    </row>
+    <row r="37" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>2014</v>
       </c>
@@ -3551,32 +3642,34 @@
       </c>
       <c r="E37" s="11">
         <f t="shared" si="6"/>
-        <v>4638</v>
+        <v>5437</v>
       </c>
       <c r="F37" s="4"/>
       <c r="G37" s="14">
         <f>ROUND(0.2*SUM(F37,H37,I37),0)</f>
-        <v>773</v>
+        <v>906</v>
       </c>
       <c r="H37" s="1">
-        <v>2302</v>
+        <v>2691</v>
       </c>
       <c r="I37" s="1">
-        <v>1563</v>
+        <v>1840</v>
       </c>
       <c r="J37" s="1">
-        <v>178</v>
+        <f>2888-H37</f>
+        <v>197</v>
       </c>
       <c r="K37" s="1">
-        <v>250</v>
+        <f>2116-I37</f>
+        <v>276</v>
       </c>
       <c r="L37" s="7">
         <f>SUM(F37,H37,I37)</f>
-        <v>3865</v>
+        <v>4531</v>
       </c>
       <c r="M37" s="23">
-        <f>SUM(J37,K37)</f>
-        <v>428</v>
+        <f t="shared" si="7"/>
+        <v>473</v>
       </c>
       <c r="N37" s="1">
         <v>149</v>
@@ -3587,44 +3680,47 @@
       <c r="P37" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q37" s="32"/>
+      <c r="Q37" s="34" t="s">
+        <v>54</v>
+      </c>
       <c r="R37" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S37" s="5" t="s">
+      <c r="S37" s="35"/>
+      <c r="T37" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="T37" s="5"/>
-      <c r="U37" s="7"/>
+      <c r="U37" s="5"/>
       <c r="V37" s="7"/>
       <c r="W37" s="7"/>
       <c r="X37" s="7"/>
       <c r="Y37" s="7"/>
-      <c r="Z37" s="8"/>
+      <c r="Z37" s="7"/>
       <c r="AA37" s="8"/>
       <c r="AB37" s="8"/>
       <c r="AC37" s="8"/>
       <c r="AD37" s="8"/>
-      <c r="AE37" s="7"/>
+      <c r="AE37" s="8"/>
       <c r="AF37" s="7"/>
       <c r="AG37" s="7"/>
       <c r="AH37" s="7"/>
       <c r="AI37" s="7"/>
       <c r="AJ37" s="7"/>
-      <c r="AM37" s="7"/>
+      <c r="AK37" s="7"/>
       <c r="AN37" s="7"/>
       <c r="AO37" s="7"/>
       <c r="AP37" s="7"/>
       <c r="AQ37" s="7"/>
       <c r="AR37" s="7"/>
-      <c r="AT37" s="7"/>
-      <c r="AV37" s="7"/>
-      <c r="AX37" s="7"/>
-      <c r="AZ37" s="7"/>
-      <c r="BE37" s="7"/>
-      <c r="BJ37" s="7"/>
-    </row>
-    <row r="38" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS37" s="7"/>
+      <c r="AU37" s="7"/>
+      <c r="AW37" s="7"/>
+      <c r="AY37" s="7"/>
+      <c r="BA37" s="7"/>
+      <c r="BF37" s="7"/>
+      <c r="BK37" s="7"/>
+    </row>
+    <row r="38" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
         <v>2015</v>
       </c>
@@ -3644,7 +3740,7 @@
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="14">
-        <f t="shared" ref="G33:G40" si="7">ROUND(0.2*SUM(F38,H38,I38),0)</f>
+        <f>ROUND(0.2*SUM(F38,H38,I38),0)</f>
         <v>983</v>
       </c>
       <c r="H38" s="1">
@@ -3654,9 +3750,11 @@
         <v>1474</v>
       </c>
       <c r="J38" s="1">
+        <f>3921-H38</f>
         <v>481</v>
       </c>
       <c r="K38" s="1">
+        <f>1577-I38</f>
         <v>103</v>
       </c>
       <c r="L38" s="7">
@@ -3664,7 +3762,7 @@
         <v>4914</v>
       </c>
       <c r="M38" s="23">
-        <f>SUM(J38,K38)</f>
+        <f t="shared" si="7"/>
         <v>584</v>
       </c>
       <c r="N38" s="1">
@@ -3676,44 +3774,47 @@
       <c r="P38" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q38" s="32"/>
+      <c r="Q38" s="34" t="s">
+        <v>55</v>
+      </c>
       <c r="R38" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S38" s="5" t="s">
+      <c r="S38" s="35"/>
+      <c r="T38" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="T38" s="5"/>
-      <c r="U38" s="7"/>
+      <c r="U38" s="5"/>
       <c r="V38" s="7"/>
       <c r="W38" s="7"/>
       <c r="X38" s="7"/>
       <c r="Y38" s="7"/>
-      <c r="Z38" s="8"/>
+      <c r="Z38" s="7"/>
       <c r="AA38" s="8"/>
       <c r="AB38" s="8"/>
       <c r="AC38" s="8"/>
       <c r="AD38" s="8"/>
-      <c r="AE38" s="7"/>
+      <c r="AE38" s="8"/>
       <c r="AF38" s="7"/>
       <c r="AG38" s="7"/>
       <c r="AH38" s="7"/>
       <c r="AI38" s="7"/>
       <c r="AJ38" s="7"/>
-      <c r="AM38" s="7"/>
+      <c r="AK38" s="7"/>
       <c r="AN38" s="7"/>
       <c r="AO38" s="7"/>
       <c r="AP38" s="7"/>
       <c r="AQ38" s="7"/>
       <c r="AR38" s="7"/>
-      <c r="AT38" s="7"/>
-      <c r="AV38" s="7"/>
-      <c r="AX38" s="7"/>
-      <c r="AZ38" s="7"/>
-      <c r="BE38" s="7"/>
-      <c r="BJ38" s="7"/>
-    </row>
-    <row r="39" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS38" s="7"/>
+      <c r="AU38" s="7"/>
+      <c r="AW38" s="7"/>
+      <c r="AY38" s="7"/>
+      <c r="BA38" s="7"/>
+      <c r="BF38" s="7"/>
+      <c r="BK38" s="7"/>
+    </row>
+    <row r="39" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>2016</v>
       </c>
@@ -3729,32 +3830,34 @@
       </c>
       <c r="E39" s="11">
         <f t="shared" si="6"/>
-        <v>3876</v>
+        <v>3833</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="14">
-        <f t="shared" si="7"/>
-        <v>646</v>
+        <f>ROUND(0.2*SUM(F39,H39,I39),0)</f>
+        <v>639</v>
       </c>
       <c r="H39" s="1">
         <v>2246</v>
       </c>
       <c r="I39" s="1">
-        <v>984</v>
+        <v>948</v>
       </c>
       <c r="J39" s="1">
+        <f>3657-H39</f>
         <v>1411</v>
       </c>
       <c r="K39" s="1">
-        <v>204</v>
+        <f>1188-I39</f>
+        <v>240</v>
       </c>
       <c r="L39" s="7">
         <f t="shared" si="3"/>
-        <v>3230</v>
+        <v>3194</v>
       </c>
       <c r="M39" s="23">
-        <f>SUM(J39,K39)</f>
-        <v>1615</v>
+        <f t="shared" si="7"/>
+        <v>1651</v>
       </c>
       <c r="N39" s="1">
         <v>74</v>
@@ -3765,44 +3868,47 @@
       <c r="P39" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q39" s="32"/>
+      <c r="Q39" s="34" t="s">
+        <v>55</v>
+      </c>
       <c r="R39" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S39" s="5" t="s">
+      <c r="S39" s="35"/>
+      <c r="T39" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="T39" s="5"/>
-      <c r="U39" s="7"/>
+      <c r="U39" s="5"/>
       <c r="V39" s="7"/>
       <c r="W39" s="7"/>
       <c r="X39" s="7"/>
       <c r="Y39" s="7"/>
-      <c r="Z39" s="8"/>
+      <c r="Z39" s="7"/>
       <c r="AA39" s="8"/>
       <c r="AB39" s="8"/>
       <c r="AC39" s="8"/>
       <c r="AD39" s="8"/>
-      <c r="AE39" s="7"/>
+      <c r="AE39" s="8"/>
       <c r="AF39" s="7"/>
       <c r="AG39" s="7"/>
       <c r="AH39" s="7"/>
       <c r="AI39" s="7"/>
       <c r="AJ39" s="7"/>
-      <c r="AM39" s="7"/>
+      <c r="AK39" s="7"/>
       <c r="AN39" s="7"/>
       <c r="AO39" s="7"/>
       <c r="AP39" s="7"/>
       <c r="AQ39" s="7"/>
       <c r="AR39" s="7"/>
-      <c r="AT39" s="7"/>
-      <c r="AV39" s="7"/>
-      <c r="AX39" s="7"/>
-      <c r="AZ39" s="7"/>
-      <c r="BE39" s="7"/>
-      <c r="BJ39" s="7"/>
-    </row>
-    <row r="40" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS39" s="7"/>
+      <c r="AU39" s="7"/>
+      <c r="AW39" s="7"/>
+      <c r="AY39" s="7"/>
+      <c r="BA39" s="7"/>
+      <c r="BF39" s="7"/>
+      <c r="BK39" s="7"/>
+    </row>
+    <row r="40" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>2017</v>
       </c>
@@ -3822,7 +3928,7 @@
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="14">
-        <f t="shared" si="7"/>
+        <f>ROUND(0.2*SUM(F40,H40,I40),0)</f>
         <v>248</v>
       </c>
       <c r="H40" s="1">
@@ -3844,7 +3950,7 @@
         <v>1240</v>
       </c>
       <c r="M40" s="23">
-        <f>SUM(J40,K40)</f>
+        <f t="shared" si="7"/>
         <v>909</v>
       </c>
       <c r="N40" s="1">
@@ -3862,40 +3968,41 @@
       <c r="R40" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S40" s="5" t="s">
+      <c r="S40" s="35"/>
+      <c r="T40" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="T40" s="5"/>
-      <c r="U40" s="7"/>
+      <c r="U40" s="5"/>
       <c r="V40" s="7"/>
       <c r="W40" s="7"/>
       <c r="X40" s="7"/>
       <c r="Y40" s="7"/>
-      <c r="Z40" s="8"/>
+      <c r="Z40" s="7"/>
       <c r="AA40" s="8"/>
       <c r="AB40" s="8"/>
       <c r="AC40" s="8"/>
       <c r="AD40" s="8"/>
-      <c r="AE40" s="7"/>
+      <c r="AE40" s="8"/>
       <c r="AF40" s="7"/>
       <c r="AG40" s="7"/>
       <c r="AH40" s="7"/>
       <c r="AI40" s="7"/>
       <c r="AJ40" s="7"/>
-      <c r="AM40" s="7"/>
+      <c r="AK40" s="7"/>
       <c r="AN40" s="7"/>
       <c r="AO40" s="7"/>
       <c r="AP40" s="7"/>
       <c r="AQ40" s="7"/>
       <c r="AR40" s="7"/>
-      <c r="AT40" s="7"/>
-      <c r="AV40" s="7"/>
-      <c r="AX40" s="7"/>
-      <c r="AZ40" s="7"/>
-      <c r="BE40" s="7"/>
-      <c r="BJ40" s="7"/>
-    </row>
-    <row r="41" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS40" s="7"/>
+      <c r="AU40" s="7"/>
+      <c r="AW40" s="7"/>
+      <c r="AY40" s="7"/>
+      <c r="BA40" s="7"/>
+      <c r="BF40" s="7"/>
+      <c r="BK40" s="7"/>
+    </row>
+    <row r="41" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
         <v>2018</v>
       </c>
@@ -3914,7 +4021,8 @@
         <v>0</v>
       </c>
       <c r="F41" s="4"/>
-      <c r="G41" s="4">
+      <c r="G41" s="14">
+        <f t="shared" ref="G38:G48" si="8">ROUND(0.2*SUM(F41,H41,I41),0)</f>
         <v>0</v>
       </c>
       <c r="H41" s="1">
@@ -3934,7 +4042,7 @@
         <v>0</v>
       </c>
       <c r="M41" s="23">
-        <f>SUM(J41,K41)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="N41" s="1">
@@ -3946,42 +4054,45 @@
       <c r="P41" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q41" s="32"/>
+      <c r="Q41" s="34" t="s">
+        <v>48</v>
+      </c>
       <c r="R41" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="S41" s="5"/>
+        <v>48</v>
+      </c>
+      <c r="S41" s="35"/>
       <c r="T41" s="5"/>
-      <c r="U41" s="7"/>
+      <c r="U41" s="5"/>
       <c r="V41" s="7"/>
       <c r="W41" s="7"/>
       <c r="X41" s="7"/>
       <c r="Y41" s="7"/>
-      <c r="Z41" s="8"/>
+      <c r="Z41" s="7"/>
       <c r="AA41" s="8"/>
       <c r="AB41" s="8"/>
       <c r="AC41" s="8"/>
       <c r="AD41" s="8"/>
-      <c r="AE41" s="7"/>
+      <c r="AE41" s="8"/>
       <c r="AF41" s="7"/>
       <c r="AG41" s="7"/>
       <c r="AH41" s="7"/>
       <c r="AI41" s="7"/>
       <c r="AJ41" s="7"/>
-      <c r="AM41" s="7"/>
+      <c r="AK41" s="7"/>
       <c r="AN41" s="7"/>
       <c r="AO41" s="7"/>
       <c r="AP41" s="7"/>
       <c r="AQ41" s="7"/>
       <c r="AR41" s="7"/>
-      <c r="AT41" s="7"/>
-      <c r="AV41" s="7"/>
-      <c r="AX41" s="7"/>
-      <c r="AZ41" s="7"/>
-      <c r="BE41" s="7"/>
-      <c r="BJ41" s="7"/>
-    </row>
-    <row r="42" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS41" s="7"/>
+      <c r="AU41" s="7"/>
+      <c r="AW41" s="7"/>
+      <c r="AY41" s="7"/>
+      <c r="BA41" s="7"/>
+      <c r="BF41" s="7"/>
+      <c r="BK41" s="7"/>
+    </row>
+    <row r="42" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>2019</v>
       </c>
@@ -3997,11 +4108,12 @@
       </c>
       <c r="E42" s="11">
         <f>SUM(F42:I42)</f>
-        <v>762</v>
+        <v>914</v>
       </c>
       <c r="F42" s="4"/>
-      <c r="G42" s="4">
-        <v>0</v>
+      <c r="G42" s="14">
+        <f>ROUND(0.2*SUM(F42,H42,I42),0)</f>
+        <v>152</v>
       </c>
       <c r="H42" s="1">
         <v>516</v>
@@ -4022,7 +4134,7 @@
         <v>762</v>
       </c>
       <c r="M42" s="23">
-        <f>SUM(J42,K42)</f>
+        <f t="shared" si="7"/>
         <v>141</v>
       </c>
       <c r="N42" s="1">
@@ -4040,38 +4152,39 @@
       <c r="R42" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S42" s="5"/>
+      <c r="S42" s="35"/>
       <c r="T42" s="5"/>
-      <c r="U42" s="7"/>
+      <c r="U42" s="5"/>
       <c r="V42" s="7"/>
       <c r="W42" s="7"/>
       <c r="X42" s="7"/>
       <c r="Y42" s="7"/>
-      <c r="Z42" s="8"/>
+      <c r="Z42" s="7"/>
       <c r="AA42" s="8"/>
       <c r="AB42" s="8"/>
       <c r="AC42" s="8"/>
       <c r="AD42" s="8"/>
-      <c r="AE42" s="7"/>
+      <c r="AE42" s="8"/>
       <c r="AF42" s="7"/>
       <c r="AG42" s="7"/>
       <c r="AH42" s="7"/>
       <c r="AI42" s="7"/>
       <c r="AJ42" s="7"/>
-      <c r="AM42" s="7"/>
+      <c r="AK42" s="7"/>
       <c r="AN42" s="7"/>
       <c r="AO42" s="7"/>
       <c r="AP42" s="7"/>
       <c r="AQ42" s="7"/>
       <c r="AR42" s="7"/>
-      <c r="AT42" s="7"/>
-      <c r="AV42" s="7"/>
-      <c r="AX42" s="7"/>
-      <c r="AZ42" s="7"/>
-      <c r="BE42" s="7"/>
-      <c r="BJ42" s="7"/>
-    </row>
-    <row r="43" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AS42" s="7"/>
+      <c r="AU42" s="7"/>
+      <c r="AW42" s="7"/>
+      <c r="AY42" s="7"/>
+      <c r="BA42" s="7"/>
+      <c r="BF42" s="7"/>
+      <c r="BK42" s="7"/>
+    </row>
+    <row r="43" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>2020</v>
       </c>
@@ -4087,11 +4200,12 @@
       </c>
       <c r="E43" s="11">
         <f>SUM(F43:I43)</f>
-        <v>1073</v>
+        <v>1288</v>
       </c>
       <c r="F43" s="4"/>
-      <c r="G43" s="4">
-        <v>0</v>
+      <c r="G43" s="14">
+        <f>ROUND(0.2*SUM(F43,H43,I43),0)</f>
+        <v>215</v>
       </c>
       <c r="H43" s="1">
         <v>535</v>
@@ -4112,7 +4226,7 @@
         <v>1073</v>
       </c>
       <c r="M43" s="23">
-        <f>SUM(J43,K43)</f>
+        <f t="shared" si="7"/>
         <v>452</v>
       </c>
       <c r="N43" s="1">
@@ -4130,38 +4244,39 @@
       <c r="R43" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S43" s="5"/>
+      <c r="S43" s="35"/>
       <c r="T43" s="5"/>
-      <c r="U43" s="7"/>
+      <c r="U43" s="5"/>
       <c r="V43" s="7"/>
       <c r="W43" s="7"/>
       <c r="X43" s="7"/>
       <c r="Y43" s="7"/>
-      <c r="Z43" s="8"/>
+      <c r="Z43" s="7"/>
       <c r="AA43" s="8"/>
       <c r="AB43" s="8"/>
       <c r="AC43" s="8"/>
       <c r="AD43" s="8"/>
-      <c r="AE43" s="7"/>
+      <c r="AE43" s="8"/>
       <c r="AF43" s="7"/>
       <c r="AG43" s="7"/>
       <c r="AH43" s="7"/>
       <c r="AI43" s="7"/>
       <c r="AJ43" s="7"/>
-      <c r="AM43" s="7"/>
+      <c r="AK43" s="7"/>
       <c r="AN43" s="7"/>
       <c r="AO43" s="7"/>
       <c r="AP43" s="7"/>
       <c r="AQ43" s="7"/>
       <c r="AR43" s="7"/>
-      <c r="AT43" s="7"/>
-      <c r="AV43" s="7"/>
-      <c r="AX43" s="7"/>
-      <c r="AZ43" s="7"/>
-      <c r="BE43" s="7"/>
-      <c r="BJ43" s="7"/>
-    </row>
-    <row r="44" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AS43" s="7"/>
+      <c r="AU43" s="7"/>
+      <c r="AW43" s="7"/>
+      <c r="AY43" s="7"/>
+      <c r="BA43" s="7"/>
+      <c r="BF43" s="7"/>
+      <c r="BK43" s="7"/>
+    </row>
+    <row r="44" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>2021</v>
       </c>
@@ -4179,7 +4294,8 @@
         <v>0</v>
       </c>
       <c r="F44" s="11"/>
-      <c r="G44" s="1">
+      <c r="G44" s="14">
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="H44" s="1">
@@ -4197,11 +4313,11 @@
         <v>380</v>
       </c>
       <c r="L44" s="7">
-        <f t="shared" ref="L44:L48" si="8">SUM(F44,H44,I44)</f>
+        <f t="shared" ref="L44:L48" si="9">SUM(F44,H44,I44)</f>
         <v>0</v>
       </c>
       <c r="M44" s="23">
-        <f>SUM(J44,K44)</f>
+        <f t="shared" si="7"/>
         <v>380</v>
       </c>
       <c r="N44" s="7"/>
@@ -4217,38 +4333,39 @@
       <c r="R44" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S44" s="5"/>
+      <c r="S44" s="35"/>
       <c r="T44" s="5"/>
-      <c r="U44" s="7"/>
+      <c r="U44" s="5"/>
       <c r="V44" s="7"/>
       <c r="W44" s="7"/>
       <c r="X44" s="7"/>
       <c r="Y44" s="7"/>
-      <c r="Z44" s="8"/>
+      <c r="Z44" s="7"/>
       <c r="AA44" s="8"/>
       <c r="AB44" s="8"/>
       <c r="AC44" s="8"/>
       <c r="AD44" s="8"/>
-      <c r="AE44" s="7"/>
+      <c r="AE44" s="8"/>
       <c r="AF44" s="7"/>
       <c r="AG44" s="7"/>
       <c r="AH44" s="7"/>
       <c r="AI44" s="7"/>
       <c r="AJ44" s="7"/>
-      <c r="AM44" s="7"/>
+      <c r="AK44" s="7"/>
       <c r="AN44" s="7"/>
       <c r="AO44" s="7"/>
       <c r="AP44" s="7"/>
       <c r="AQ44" s="7"/>
       <c r="AR44" s="7"/>
-      <c r="AT44" s="7"/>
-      <c r="AV44" s="7"/>
-      <c r="AX44" s="7"/>
-      <c r="AZ44" s="7"/>
-      <c r="BE44" s="7"/>
-      <c r="BJ44" s="7"/>
-    </row>
-    <row r="45" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AS44" s="7"/>
+      <c r="AU44" s="7"/>
+      <c r="AW44" s="7"/>
+      <c r="AY44" s="7"/>
+      <c r="BA44" s="7"/>
+      <c r="BF44" s="7"/>
+      <c r="BK44" s="7"/>
+    </row>
+    <row r="45" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>2022</v>
       </c>
@@ -4266,7 +4383,8 @@
         <v>0</v>
       </c>
       <c r="F45" s="11"/>
-      <c r="G45" s="11">
+      <c r="G45" s="14">
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="H45" s="1">
@@ -4284,11 +4402,11 @@
         <v>274</v>
       </c>
       <c r="L45" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="M45" s="23">
-        <f>SUM(J45,K45)</f>
+        <f t="shared" si="7"/>
         <v>347</v>
       </c>
       <c r="N45" s="7"/>
@@ -4304,38 +4422,39 @@
       <c r="R45" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S45" s="5"/>
+      <c r="S45" s="35"/>
       <c r="T45" s="5"/>
-      <c r="U45" s="7"/>
+      <c r="U45" s="5"/>
       <c r="V45" s="7"/>
       <c r="W45" s="7"/>
       <c r="X45" s="7"/>
       <c r="Y45" s="7"/>
-      <c r="Z45" s="8"/>
+      <c r="Z45" s="7"/>
       <c r="AA45" s="8"/>
       <c r="AB45" s="8"/>
       <c r="AC45" s="8"/>
       <c r="AD45" s="8"/>
-      <c r="AE45" s="7"/>
+      <c r="AE45" s="8"/>
       <c r="AF45" s="7"/>
       <c r="AG45" s="7"/>
       <c r="AH45" s="7"/>
       <c r="AI45" s="7"/>
       <c r="AJ45" s="7"/>
-      <c r="AM45" s="7"/>
+      <c r="AK45" s="7"/>
       <c r="AN45" s="7"/>
       <c r="AO45" s="7"/>
       <c r="AP45" s="7"/>
       <c r="AQ45" s="7"/>
       <c r="AR45" s="7"/>
-      <c r="AT45" s="7"/>
-      <c r="AV45" s="7"/>
-      <c r="AX45" s="7"/>
-      <c r="AZ45" s="7"/>
-      <c r="BE45" s="7"/>
-      <c r="BJ45" s="7"/>
-    </row>
-    <row r="46" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AS45" s="7"/>
+      <c r="AU45" s="7"/>
+      <c r="AW45" s="7"/>
+      <c r="AY45" s="7"/>
+      <c r="BA45" s="7"/>
+      <c r="BF45" s="7"/>
+      <c r="BK45" s="7"/>
+    </row>
+    <row r="46" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>2023</v>
       </c>
@@ -4349,12 +4468,13 @@
         <v>646</v>
       </c>
       <c r="E46" s="11">
-        <f t="shared" ref="E46:E48" si="9">SUM(F46:I46)</f>
-        <v>71</v>
+        <f t="shared" ref="E46:E48" si="10">SUM(F46:I46)</f>
+        <v>85</v>
       </c>
       <c r="F46" s="11"/>
-      <c r="G46" s="11">
-        <v>0</v>
+      <c r="G46" s="14">
+        <f>ROUND(0.2*SUM(F46,H46,I46),0)</f>
+        <v>14</v>
       </c>
       <c r="H46" s="1">
         <v>71</v>
@@ -4371,7 +4491,7 @@
         <v>52</v>
       </c>
       <c r="L46" s="7">
-        <f t="shared" si="8"/>
+        <f>SUM(F46,H46,I46)</f>
         <v>71</v>
       </c>
       <c r="M46" s="23">
@@ -4391,38 +4511,39 @@
       <c r="R46" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S46" s="5"/>
+      <c r="S46" s="35"/>
       <c r="T46" s="5"/>
-      <c r="U46" s="7"/>
+      <c r="U46" s="5"/>
       <c r="V46" s="7"/>
       <c r="W46" s="7"/>
       <c r="X46" s="7"/>
       <c r="Y46" s="7"/>
-      <c r="Z46" s="8"/>
+      <c r="Z46" s="7"/>
       <c r="AA46" s="8"/>
       <c r="AB46" s="8"/>
       <c r="AC46" s="8"/>
       <c r="AD46" s="8"/>
-      <c r="AE46" s="7"/>
+      <c r="AE46" s="8"/>
       <c r="AF46" s="7"/>
       <c r="AG46" s="7"/>
       <c r="AH46" s="7"/>
       <c r="AI46" s="7"/>
       <c r="AJ46" s="7"/>
-      <c r="AM46" s="7"/>
+      <c r="AK46" s="7"/>
       <c r="AN46" s="7"/>
       <c r="AO46" s="7"/>
       <c r="AP46" s="7"/>
       <c r="AQ46" s="7"/>
       <c r="AR46" s="7"/>
-      <c r="AT46" s="7"/>
-      <c r="AV46" s="7"/>
-      <c r="AX46" s="7"/>
-      <c r="AZ46" s="7"/>
-      <c r="BE46" s="7"/>
-      <c r="BJ46" s="7"/>
-    </row>
-    <row r="47" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AS46" s="7"/>
+      <c r="AU46" s="7"/>
+      <c r="AW46" s="7"/>
+      <c r="AY46" s="7"/>
+      <c r="BA46" s="7"/>
+      <c r="BF46" s="7"/>
+      <c r="BK46" s="7"/>
+    </row>
+    <row r="47" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>2024</v>
       </c>
@@ -4436,11 +4557,12 @@
         <v>482</v>
       </c>
       <c r="E47" s="11">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1</v>
       </c>
       <c r="F47" s="11"/>
-      <c r="G47" s="11">
+      <c r="G47" s="14">
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="H47" s="1">
@@ -4458,7 +4580,7 @@
         <v>2</v>
       </c>
       <c r="L47" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
       <c r="M47" s="23">
@@ -4478,38 +4600,39 @@
       <c r="R47" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S47" s="5"/>
+      <c r="S47" s="35"/>
       <c r="T47" s="5"/>
-      <c r="U47" s="7"/>
+      <c r="U47" s="5"/>
       <c r="V47" s="7"/>
       <c r="W47" s="7"/>
       <c r="X47" s="7"/>
       <c r="Y47" s="7"/>
-      <c r="Z47" s="8"/>
+      <c r="Z47" s="7"/>
       <c r="AA47" s="8"/>
       <c r="AB47" s="8"/>
       <c r="AC47" s="8"/>
       <c r="AD47" s="8"/>
-      <c r="AE47" s="7"/>
+      <c r="AE47" s="8"/>
       <c r="AF47" s="7"/>
       <c r="AG47" s="7"/>
       <c r="AH47" s="7"/>
       <c r="AI47" s="7"/>
       <c r="AJ47" s="7"/>
-      <c r="AM47" s="7"/>
+      <c r="AK47" s="7"/>
       <c r="AN47" s="7"/>
       <c r="AO47" s="7"/>
       <c r="AP47" s="7"/>
       <c r="AQ47" s="7"/>
       <c r="AR47" s="7"/>
-      <c r="AT47" s="7"/>
-      <c r="AV47" s="7"/>
-      <c r="AX47" s="7"/>
-      <c r="AZ47" s="7"/>
-      <c r="BE47" s="7"/>
-      <c r="BJ47" s="7"/>
-    </row>
-    <row r="48" spans="1:62" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AS47" s="7"/>
+      <c r="AU47" s="7"/>
+      <c r="AW47" s="7"/>
+      <c r="AY47" s="7"/>
+      <c r="BA47" s="7"/>
+      <c r="BF47" s="7"/>
+      <c r="BK47" s="7"/>
+    </row>
+    <row r="48" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>2025</v>
       </c>
@@ -4517,12 +4640,13 @@
       <c r="C48" s="19"/>
       <c r="D48" s="19"/>
       <c r="E48" s="11">
-        <f t="shared" si="9"/>
-        <v>19</v>
+        <f t="shared" si="10"/>
+        <v>23</v>
       </c>
       <c r="F48" s="4"/>
-      <c r="G48" s="4">
-        <v>0</v>
+      <c r="G48" s="14">
+        <f>ROUND(0.2*SUM(F48,H48,I48),0)</f>
+        <v>4</v>
       </c>
       <c r="H48" s="1">
         <v>14</v>
@@ -4539,7 +4663,7 @@
         <v>21</v>
       </c>
       <c r="L48" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>19</v>
       </c>
       <c r="M48" s="23">
@@ -4559,693 +4683,740 @@
       <c r="R48" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S48" s="5"/>
+      <c r="S48" s="35"/>
       <c r="T48" s="5"/>
       <c r="U48" s="5"/>
       <c r="V48" s="5"/>
       <c r="W48" s="5"/>
       <c r="X48" s="5"/>
       <c r="Y48" s="5"/>
-      <c r="Z48" s="8"/>
+      <c r="Z48" s="5"/>
       <c r="AA48" s="8"/>
       <c r="AB48" s="8"/>
       <c r="AC48" s="8"/>
       <c r="AD48" s="8"/>
-      <c r="AM48" s="7"/>
+      <c r="AE48" s="8"/>
       <c r="AN48" s="7"/>
       <c r="AO48" s="7"/>
       <c r="AP48" s="7"/>
       <c r="AQ48" s="7"/>
       <c r="AR48" s="7"/>
-      <c r="AT48" s="7"/>
-      <c r="AV48" s="7"/>
-      <c r="AX48" s="7"/>
-      <c r="AZ48" s="7"/>
-      <c r="BE48" s="7"/>
-      <c r="BJ48" s="7"/>
-    </row>
-    <row r="49" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="A49" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D49" s="27" t="s">
-        <v>14</v>
-      </c>
-      <c r="E49" s="15" t="s">
-        <v>13</v>
-      </c>
+      <c r="AS48" s="7"/>
+      <c r="AU48" s="7"/>
+      <c r="AW48" s="7"/>
+      <c r="AY48" s="7"/>
+      <c r="BA48" s="7"/>
+      <c r="BF48" s="7"/>
+      <c r="BK48" s="7"/>
+    </row>
+    <row r="49" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="1">
+        <v>2026</v>
+      </c>
+      <c r="B49" s="19"/>
+      <c r="C49" s="19"/>
+      <c r="D49" s="19"/>
+      <c r="E49" s="11"/>
       <c r="F49" s="4"/>
-      <c r="G49" s="4"/>
-      <c r="N49" s="13" t="s">
-        <v>20</v>
-      </c>
+      <c r="G49" s="14"/>
+      <c r="L49" s="7"/>
+      <c r="M49" s="23"/>
+      <c r="N49" s="7"/>
+      <c r="O49"/>
+      <c r="P49" s="5"/>
+      <c r="Q49" s="33"/>
       <c r="R49" s="5"/>
-      <c r="AM49" s="7"/>
+      <c r="S49" s="35"/>
+      <c r="T49" s="5"/>
+      <c r="U49" s="5"/>
+      <c r="V49" s="5"/>
+      <c r="W49" s="5"/>
+      <c r="X49" s="5"/>
+      <c r="Y49" s="5"/>
+      <c r="Z49" s="5"/>
+      <c r="AA49" s="8"/>
+      <c r="AB49" s="8"/>
+      <c r="AC49" s="8"/>
+      <c r="AD49" s="8"/>
+      <c r="AE49" s="8"/>
       <c r="AN49" s="7"/>
       <c r="AO49" s="7"/>
       <c r="AP49" s="7"/>
       <c r="AQ49" s="7"/>
       <c r="AR49" s="7"/>
-      <c r="AT49" s="7"/>
-      <c r="AV49" s="7"/>
-      <c r="AX49" s="7"/>
-      <c r="AZ49" s="7"/>
-      <c r="BE49" s="7"/>
-      <c r="BJ49" s="7"/>
-    </row>
-    <row r="50" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="E50" s="16" t="s">
-        <v>18</v>
+      <c r="AS49" s="7"/>
+      <c r="AU49" s="7"/>
+      <c r="AW49" s="7"/>
+      <c r="AY49" s="7"/>
+      <c r="BA49" s="7"/>
+      <c r="BF49" s="7"/>
+      <c r="BK49" s="7"/>
+    </row>
+    <row r="50" spans="1:63" x14ac:dyDescent="0.2">
+      <c r="A50" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D50" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="E50" s="15" t="s">
+        <v>13</v>
       </c>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
+      <c r="N50" s="13" t="s">
+        <v>20</v>
+      </c>
       <c r="R50" s="5"/>
-      <c r="AM50" s="7"/>
+      <c r="S50" s="5"/>
       <c r="AN50" s="7"/>
       <c r="AO50" s="7"/>
       <c r="AP50" s="7"/>
       <c r="AQ50" s="7"/>
       <c r="AR50" s="7"/>
-      <c r="AT50" s="7"/>
-      <c r="AV50" s="7"/>
-      <c r="AX50" s="7"/>
-      <c r="AZ50" s="7"/>
-      <c r="BE50" s="7"/>
-      <c r="BJ50" s="7"/>
-    </row>
-    <row r="51" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="B51" s="27"/>
-      <c r="C51" s="27"/>
-      <c r="D51" s="27"/>
-      <c r="E51" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="AM51" s="7"/>
+      <c r="AS50" s="7"/>
+      <c r="AU50" s="7"/>
+      <c r="AW50" s="7"/>
+      <c r="AY50" s="7"/>
+      <c r="BA50" s="7"/>
+      <c r="BF50" s="7"/>
+      <c r="BK50" s="7"/>
+    </row>
+    <row r="51" spans="1:63" x14ac:dyDescent="0.2">
+      <c r="E51" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="F51" s="4"/>
+      <c r="G51" s="4"/>
+      <c r="R51" s="5"/>
+      <c r="S51" s="5"/>
       <c r="AN51" s="7"/>
       <c r="AO51" s="7"/>
       <c r="AP51" s="7"/>
       <c r="AQ51" s="7"/>
       <c r="AR51" s="7"/>
-      <c r="AT51" s="7"/>
-      <c r="AV51" s="7"/>
-      <c r="AX51" s="7"/>
-      <c r="AZ51" s="7"/>
-      <c r="BE51" s="7"/>
-      <c r="BJ51" s="7"/>
-    </row>
-    <row r="52" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="E52" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="AM52" s="7"/>
+      <c r="AS51" s="7"/>
+      <c r="AU51" s="7"/>
+      <c r="AW51" s="7"/>
+      <c r="AY51" s="7"/>
+      <c r="BA51" s="7"/>
+      <c r="BF51" s="7"/>
+      <c r="BK51" s="7"/>
+    </row>
+    <row r="52" spans="1:63" x14ac:dyDescent="0.2">
+      <c r="B52" s="27"/>
+      <c r="C52" s="27"/>
+      <c r="D52" s="27"/>
+      <c r="E52" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="S52" s="35"/>
       <c r="AN52" s="7"/>
       <c r="AO52" s="7"/>
       <c r="AP52" s="7"/>
       <c r="AQ52" s="7"/>
       <c r="AR52" s="7"/>
-      <c r="AT52" s="7"/>
-      <c r="AV52" s="7"/>
-      <c r="AX52" s="7"/>
-      <c r="AZ52" s="7"/>
-      <c r="BE52" s="7"/>
-      <c r="BJ52" s="7"/>
-    </row>
-    <row r="53" spans="1:62" x14ac:dyDescent="0.2">
+      <c r="AS52" s="7"/>
+      <c r="AU52" s="7"/>
+      <c r="AW52" s="7"/>
+      <c r="AY52" s="7"/>
+      <c r="BA52" s="7"/>
+      <c r="BF52" s="7"/>
+      <c r="BK52" s="7"/>
+    </row>
+    <row r="53" spans="1:63" x14ac:dyDescent="0.2">
       <c r="E53" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="AN53" s="7"/>
+      <c r="AO53" s="7"/>
+      <c r="AP53" s="7"/>
+      <c r="AQ53" s="7"/>
+      <c r="AR53" s="7"/>
+      <c r="AS53" s="7"/>
+      <c r="AU53" s="7"/>
+      <c r="AW53" s="7"/>
+      <c r="AY53" s="7"/>
+      <c r="BA53" s="7"/>
+      <c r="BF53" s="7"/>
+      <c r="BK53" s="7"/>
+    </row>
+    <row r="54" spans="1:63" x14ac:dyDescent="0.2">
+      <c r="E54" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="BE53" s="7"/>
-      <c r="BJ53" s="7"/>
-    </row>
-    <row r="54" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="E54" s="1" t="s">
+      <c r="BF54" s="7"/>
+      <c r="BK54" s="7"/>
+    </row>
+    <row r="55" spans="1:63" x14ac:dyDescent="0.2">
+      <c r="E55" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="BE54" s="7"/>
-      <c r="BJ54" s="7"/>
-    </row>
-    <row r="55" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="E55" s="1" t="s">
+      <c r="BF55" s="7"/>
+      <c r="BK55" s="7"/>
+    </row>
+    <row r="56" spans="1:63" x14ac:dyDescent="0.2">
+      <c r="E56" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="BE55" s="7"/>
-      <c r="BJ55" s="7"/>
-    </row>
-    <row r="56" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="E56" s="1" t="s">
+      <c r="BF56" s="7"/>
+      <c r="BK56" s="7"/>
+    </row>
+    <row r="57" spans="1:63" x14ac:dyDescent="0.2">
+      <c r="E57" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="BE56" s="7"/>
-      <c r="BJ56" s="7"/>
-    </row>
-    <row r="57" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="E57" s="1" t="s">
+      <c r="BF57" s="7"/>
+      <c r="BK57" s="7"/>
+    </row>
+    <row r="58" spans="1:63" x14ac:dyDescent="0.2">
+      <c r="E58" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="BE57" s="7"/>
-      <c r="BJ57" s="7"/>
-    </row>
-    <row r="58" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="E58" s="17" t="s">
+      <c r="BF58" s="7"/>
+      <c r="BK58" s="7"/>
+    </row>
+    <row r="59" spans="1:63" x14ac:dyDescent="0.2">
+      <c r="E59" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="BE58" s="7"/>
-      <c r="BJ58" s="7"/>
-    </row>
-    <row r="59" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="E59" s="22" t="s">
+      <c r="BF59" s="7"/>
+      <c r="BK59" s="7"/>
+    </row>
+    <row r="60" spans="1:63" x14ac:dyDescent="0.2">
+      <c r="E60" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="BE59" s="7"/>
-      <c r="BJ59" s="7"/>
-    </row>
-    <row r="60" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="E60" s="1" t="s">
+      <c r="BF60" s="7"/>
+      <c r="BK60" s="7"/>
+    </row>
+    <row r="61" spans="1:63" x14ac:dyDescent="0.2">
+      <c r="E61" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="BE60" s="7"/>
-      <c r="BJ60" s="7"/>
-    </row>
-    <row r="61" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="E61" s="1" t="s">
+      <c r="BF61" s="7"/>
+      <c r="BK61" s="7"/>
+    </row>
+    <row r="62" spans="1:63" x14ac:dyDescent="0.2">
+      <c r="E62" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="BE61" s="7"/>
-      <c r="BJ61" s="7"/>
-    </row>
-    <row r="62" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="BE62" s="7"/>
-      <c r="BJ62" s="7"/>
-    </row>
-    <row r="63" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="BE63" s="7"/>
-      <c r="BJ63" s="7"/>
-    </row>
-    <row r="64" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="BE64" s="7"/>
-      <c r="BJ64" s="7"/>
-    </row>
-    <row r="65" spans="2:62" x14ac:dyDescent="0.2">
-      <c r="B65" s="2"/>
-      <c r="C65" s="2"/>
-      <c r="D65" s="2"/>
-      <c r="E65" s="2"/>
-      <c r="F65" s="2"/>
-      <c r="G65" s="2"/>
-      <c r="H65" s="2"/>
-      <c r="I65" s="2"/>
-      <c r="J65" s="2"/>
-      <c r="K65" s="2"/>
-      <c r="L65" s="2"/>
-      <c r="M65" s="18"/>
-      <c r="N65" s="2"/>
-      <c r="O65" s="2"/>
-      <c r="P65" s="2"/>
-      <c r="Q65" s="2"/>
-      <c r="T65" s="3"/>
-      <c r="U65" s="3"/>
-      <c r="V65" s="3"/>
-      <c r="X65" s="3"/>
-      <c r="AJ65" s="3"/>
-    </row>
-    <row r="66" spans="2:62" x14ac:dyDescent="0.2">
-      <c r="BE66" s="7"/>
-      <c r="BJ66" s="7"/>
-    </row>
-    <row r="67" spans="2:62" x14ac:dyDescent="0.2">
-      <c r="BE67" s="7"/>
-      <c r="BJ67" s="7"/>
-    </row>
-    <row r="68" spans="2:62" x14ac:dyDescent="0.2">
-      <c r="BE68" s="7"/>
-      <c r="BJ68" s="7"/>
-    </row>
-    <row r="69" spans="2:62" x14ac:dyDescent="0.2">
-      <c r="BE69" s="7"/>
-      <c r="BJ69" s="7"/>
-    </row>
-    <row r="70" spans="2:62" x14ac:dyDescent="0.2">
-      <c r="BE70" s="7"/>
-      <c r="BJ70" s="7"/>
-    </row>
-    <row r="71" spans="2:62" x14ac:dyDescent="0.2">
-      <c r="BE71" s="7"/>
-      <c r="BJ71" s="7"/>
-    </row>
-    <row r="72" spans="2:62" x14ac:dyDescent="0.2">
-      <c r="BE72" s="7"/>
-      <c r="BJ72" s="7"/>
-    </row>
-    <row r="73" spans="2:62" x14ac:dyDescent="0.2">
-      <c r="BE73" s="7"/>
-      <c r="BJ73" s="7"/>
-    </row>
-    <row r="74" spans="2:62" x14ac:dyDescent="0.2">
-      <c r="BE74" s="7"/>
-      <c r="BJ74" s="7"/>
-    </row>
-    <row r="75" spans="2:62" x14ac:dyDescent="0.2">
-      <c r="BE75" s="7"/>
-      <c r="BJ75" s="7"/>
-    </row>
-    <row r="76" spans="2:62" x14ac:dyDescent="0.2">
-      <c r="BE76" s="7"/>
-      <c r="BJ76" s="7"/>
-    </row>
-    <row r="77" spans="2:62" x14ac:dyDescent="0.2">
-      <c r="BE77" s="7"/>
-      <c r="BJ77" s="7"/>
-    </row>
-    <row r="78" spans="2:62" x14ac:dyDescent="0.2">
-      <c r="BE78" s="7"/>
-      <c r="BJ78" s="7"/>
-    </row>
-    <row r="79" spans="2:62" x14ac:dyDescent="0.2">
-      <c r="BE79" s="7"/>
-      <c r="BJ79" s="7"/>
-    </row>
-    <row r="80" spans="2:62" x14ac:dyDescent="0.2">
-      <c r="BE80" s="7"/>
-      <c r="BJ80" s="7"/>
-    </row>
-    <row r="81" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE81" s="7"/>
-      <c r="BJ81" s="7"/>
-    </row>
-    <row r="82" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE82" s="7"/>
-      <c r="BJ82" s="7"/>
-    </row>
-    <row r="83" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE83" s="7"/>
-      <c r="BJ83" s="7"/>
-    </row>
-    <row r="84" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE84" s="7"/>
-      <c r="BJ84" s="7"/>
-    </row>
-    <row r="85" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE85" s="7"/>
-      <c r="BJ85" s="7"/>
-    </row>
-    <row r="86" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE86" s="7"/>
-      <c r="BJ86" s="7"/>
-    </row>
-    <row r="87" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE87" s="7"/>
-      <c r="BJ87" s="7"/>
-    </row>
-    <row r="88" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE88" s="7"/>
-      <c r="BJ88" s="7"/>
-    </row>
-    <row r="89" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE89" s="7"/>
-      <c r="BJ89" s="7"/>
-    </row>
-    <row r="90" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE90" s="7"/>
-      <c r="BJ90" s="7"/>
-    </row>
-    <row r="91" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE91" s="7"/>
-      <c r="BJ91" s="7"/>
-    </row>
-    <row r="92" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE92" s="7"/>
-      <c r="BJ92" s="7"/>
-    </row>
-    <row r="93" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE93" s="7"/>
-      <c r="BJ93" s="7"/>
-    </row>
-    <row r="94" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE94" s="7"/>
-      <c r="BJ94" s="7"/>
-    </row>
-    <row r="95" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE95" s="7"/>
-      <c r="BJ95" s="7"/>
-    </row>
-    <row r="96" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE96" s="7"/>
-      <c r="BJ96" s="7"/>
-    </row>
-    <row r="97" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE97" s="7"/>
-      <c r="BJ97" s="7"/>
-    </row>
-    <row r="98" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE98" s="7"/>
-      <c r="BJ98" s="7"/>
-    </row>
-    <row r="99" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE99" s="7"/>
-      <c r="BJ99" s="7"/>
-    </row>
-    <row r="100" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE100" s="7"/>
-      <c r="BJ100" s="7"/>
-    </row>
-    <row r="101" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE101" s="7"/>
-      <c r="BJ101" s="7"/>
-    </row>
-    <row r="102" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE102" s="7"/>
-      <c r="BJ102" s="7"/>
-    </row>
-    <row r="103" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE103" s="7"/>
-      <c r="BJ103" s="7"/>
-    </row>
-    <row r="104" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE104" s="7"/>
-      <c r="BJ104" s="7"/>
-    </row>
-    <row r="105" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE105" s="7"/>
-      <c r="BJ105" s="7"/>
-    </row>
-    <row r="106" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE106" s="7"/>
-      <c r="BJ106" s="7"/>
-    </row>
-    <row r="107" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE107" s="7"/>
-      <c r="BJ107" s="7"/>
-    </row>
-    <row r="108" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE108" s="7"/>
-      <c r="BJ108" s="7"/>
-    </row>
-    <row r="109" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE109" s="7"/>
-      <c r="BJ109" s="7"/>
-    </row>
-    <row r="110" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE110" s="7"/>
-      <c r="BJ110" s="7"/>
-    </row>
-    <row r="111" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE111" s="7"/>
-      <c r="BJ111" s="7"/>
-    </row>
-    <row r="112" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE112" s="7"/>
-      <c r="BJ112" s="7"/>
-    </row>
-    <row r="113" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE113" s="7"/>
-      <c r="BJ113" s="7"/>
-    </row>
-    <row r="114" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE114" s="7"/>
-      <c r="BJ114" s="7"/>
-    </row>
-    <row r="115" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE115" s="7"/>
-      <c r="BJ115" s="7"/>
-    </row>
-    <row r="116" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE116" s="7"/>
-      <c r="BJ116" s="7"/>
-    </row>
-    <row r="117" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE117" s="7"/>
-      <c r="BJ117" s="7"/>
-    </row>
-    <row r="118" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE118" s="7"/>
-      <c r="BJ118" s="7"/>
-    </row>
-    <row r="119" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE119" s="7"/>
-      <c r="BJ119" s="7"/>
-    </row>
-    <row r="120" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE120" s="7"/>
-      <c r="BJ120" s="7"/>
-    </row>
-    <row r="121" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE121" s="7"/>
-      <c r="BJ121" s="7"/>
-    </row>
-    <row r="122" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE122" s="7"/>
-      <c r="BJ122" s="7"/>
-    </row>
-    <row r="123" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE123" s="7"/>
-      <c r="BJ123" s="7"/>
-    </row>
-    <row r="124" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE124" s="7"/>
-      <c r="BJ124" s="7"/>
-    </row>
-    <row r="125" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE125" s="7"/>
-      <c r="BJ125" s="7"/>
-    </row>
-    <row r="126" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE126" s="7"/>
-      <c r="BJ126" s="7"/>
-    </row>
-    <row r="127" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE127" s="7"/>
-      <c r="BJ127" s="7"/>
-    </row>
-    <row r="128" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE128" s="7"/>
-      <c r="BJ128" s="7"/>
-    </row>
-    <row r="129" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE129" s="7"/>
-      <c r="BJ129" s="7"/>
-    </row>
-    <row r="130" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE130" s="7"/>
-      <c r="BJ130" s="7"/>
-    </row>
-    <row r="131" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE131" s="7"/>
-      <c r="BJ131" s="7"/>
-    </row>
-    <row r="132" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE132" s="7"/>
-      <c r="BJ132" s="7"/>
-    </row>
-    <row r="133" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE133" s="7"/>
-      <c r="BJ133" s="7"/>
-    </row>
-    <row r="134" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE134" s="7"/>
-      <c r="BJ134" s="7"/>
-    </row>
-    <row r="135" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE135" s="7"/>
-      <c r="BJ135" s="7"/>
-    </row>
-    <row r="136" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE136" s="7"/>
-      <c r="BJ136" s="7"/>
-    </row>
-    <row r="137" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE137" s="7"/>
-      <c r="BJ137" s="7"/>
-    </row>
-    <row r="138" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE138" s="7"/>
-      <c r="BJ138" s="7"/>
-    </row>
-    <row r="139" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE139" s="7"/>
-      <c r="BJ139" s="7"/>
-    </row>
-    <row r="140" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE140" s="7"/>
-      <c r="BJ140" s="7"/>
-    </row>
-    <row r="141" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE141" s="7"/>
-      <c r="BJ141" s="7"/>
-    </row>
-    <row r="142" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE142" s="7"/>
-      <c r="BJ142" s="7"/>
-    </row>
-    <row r="143" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE143" s="7"/>
-      <c r="BJ143" s="7"/>
-    </row>
-    <row r="144" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE144" s="7"/>
-      <c r="BJ144" s="7"/>
-    </row>
-    <row r="145" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE145" s="7"/>
-      <c r="BJ145" s="7"/>
-    </row>
-    <row r="146" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE146" s="7"/>
-      <c r="BJ146" s="7"/>
-    </row>
-    <row r="147" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE147" s="7"/>
-      <c r="BJ147" s="7"/>
-    </row>
-    <row r="148" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE148" s="7"/>
-      <c r="BJ148" s="7"/>
-    </row>
-    <row r="149" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE149" s="7"/>
-      <c r="BJ149" s="7"/>
-    </row>
-    <row r="150" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE150" s="7"/>
-      <c r="BJ150" s="7"/>
-    </row>
-    <row r="151" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE151" s="7"/>
-      <c r="BJ151" s="7"/>
-    </row>
-    <row r="152" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE152" s="7"/>
-      <c r="BJ152" s="7"/>
-    </row>
-    <row r="153" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE153" s="7"/>
-      <c r="BJ153" s="7"/>
-    </row>
-    <row r="154" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE154" s="7"/>
-      <c r="BJ154" s="7"/>
-    </row>
-    <row r="155" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE155" s="7"/>
-      <c r="BJ155" s="7"/>
-    </row>
-    <row r="156" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE156" s="7"/>
-      <c r="BJ156" s="7"/>
-    </row>
-    <row r="157" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE157" s="7"/>
-      <c r="BJ157" s="7"/>
-    </row>
-    <row r="158" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE158" s="7"/>
-      <c r="BJ158" s="7"/>
-    </row>
-    <row r="159" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE159" s="7"/>
-      <c r="BJ159" s="7"/>
-    </row>
-    <row r="160" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE160" s="7"/>
-      <c r="BJ160" s="7"/>
-    </row>
-    <row r="161" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE161" s="7"/>
-      <c r="BJ161" s="7"/>
-    </row>
-    <row r="162" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE162" s="7"/>
-      <c r="BJ162" s="7"/>
-    </row>
-    <row r="163" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE163" s="7"/>
-      <c r="BJ163" s="7"/>
-    </row>
-    <row r="164" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE164" s="7"/>
-      <c r="BJ164" s="7"/>
-    </row>
-    <row r="165" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE165" s="7"/>
-      <c r="BJ165" s="7"/>
-    </row>
-    <row r="166" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE166" s="7"/>
-      <c r="BJ166" s="7"/>
-    </row>
-    <row r="167" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE167" s="7"/>
-      <c r="BJ167" s="7"/>
-    </row>
-    <row r="168" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE168" s="7"/>
-      <c r="BJ168" s="7"/>
-    </row>
-    <row r="169" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE169" s="7"/>
-      <c r="BJ169" s="7"/>
-    </row>
-    <row r="170" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE170" s="7"/>
-    </row>
-    <row r="171" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE171" s="7"/>
-    </row>
-    <row r="172" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE172" s="7"/>
-    </row>
-    <row r="173" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE173" s="7"/>
-    </row>
-    <row r="174" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE174" s="7"/>
-    </row>
-    <row r="175" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE175" s="7"/>
-    </row>
-    <row r="176" spans="57:62" x14ac:dyDescent="0.2">
-      <c r="BE176" s="7"/>
-    </row>
-    <row r="177" spans="57:57" x14ac:dyDescent="0.2">
-      <c r="BE177" s="7"/>
-    </row>
-    <row r="178" spans="57:57" x14ac:dyDescent="0.2">
-      <c r="BE178" s="7"/>
-    </row>
-    <row r="179" spans="57:57" x14ac:dyDescent="0.2">
-      <c r="BE179" s="7"/>
-    </row>
-    <row r="180" spans="57:57" x14ac:dyDescent="0.2">
-      <c r="BE180" s="7"/>
-    </row>
-    <row r="181" spans="57:57" x14ac:dyDescent="0.2">
-      <c r="BE181" s="7"/>
-    </row>
-    <row r="182" spans="57:57" x14ac:dyDescent="0.2">
-      <c r="BE182" s="7"/>
-    </row>
-    <row r="183" spans="57:57" x14ac:dyDescent="0.2">
-      <c r="BE183" s="7"/>
-    </row>
-    <row r="184" spans="57:57" x14ac:dyDescent="0.2">
-      <c r="BE184" s="7"/>
-    </row>
-    <row r="185" spans="57:57" x14ac:dyDescent="0.2">
-      <c r="BE185" s="7"/>
-    </row>
-    <row r="186" spans="57:57" x14ac:dyDescent="0.2">
-      <c r="BE186" s="7"/>
-    </row>
-    <row r="187" spans="57:57" x14ac:dyDescent="0.2">
-      <c r="BE187" s="7"/>
-    </row>
-    <row r="188" spans="57:57" x14ac:dyDescent="0.2">
-      <c r="BE188" s="7"/>
-    </row>
-    <row r="189" spans="57:57" x14ac:dyDescent="0.2">
-      <c r="BE189" s="7"/>
-    </row>
-    <row r="190" spans="57:57" x14ac:dyDescent="0.2">
-      <c r="BE190" s="7"/>
+      <c r="BF62" s="7"/>
+      <c r="BK62" s="7"/>
+    </row>
+    <row r="63" spans="1:63" x14ac:dyDescent="0.2">
+      <c r="BF63" s="7"/>
+      <c r="BK63" s="7"/>
+    </row>
+    <row r="64" spans="1:63" x14ac:dyDescent="0.2">
+      <c r="BF64" s="7"/>
+      <c r="BK64" s="7"/>
+    </row>
+    <row r="65" spans="2:63" x14ac:dyDescent="0.2">
+      <c r="BF65" s="7"/>
+      <c r="BK65" s="7"/>
+    </row>
+    <row r="66" spans="2:63" x14ac:dyDescent="0.2">
+      <c r="B66" s="2"/>
+      <c r="C66" s="2"/>
+      <c r="D66" s="2"/>
+      <c r="E66" s="2"/>
+      <c r="F66" s="2"/>
+      <c r="G66" s="2"/>
+      <c r="H66" s="2"/>
+      <c r="I66" s="2"/>
+      <c r="J66" s="2"/>
+      <c r="K66" s="2"/>
+      <c r="L66" s="2"/>
+      <c r="M66" s="18"/>
+      <c r="N66" s="2"/>
+      <c r="O66" s="2"/>
+      <c r="P66" s="2"/>
+      <c r="Q66" s="2"/>
+      <c r="U66" s="3"/>
+      <c r="V66" s="3"/>
+      <c r="W66" s="3"/>
+      <c r="Y66" s="3"/>
+      <c r="AK66" s="3"/>
+    </row>
+    <row r="67" spans="2:63" x14ac:dyDescent="0.2">
+      <c r="BF67" s="7"/>
+      <c r="BK67" s="7"/>
+    </row>
+    <row r="68" spans="2:63" x14ac:dyDescent="0.2">
+      <c r="BF68" s="7"/>
+      <c r="BK68" s="7"/>
+    </row>
+    <row r="69" spans="2:63" x14ac:dyDescent="0.2">
+      <c r="BF69" s="7"/>
+      <c r="BK69" s="7"/>
+    </row>
+    <row r="70" spans="2:63" x14ac:dyDescent="0.2">
+      <c r="BF70" s="7"/>
+      <c r="BK70" s="7"/>
+    </row>
+    <row r="71" spans="2:63" x14ac:dyDescent="0.2">
+      <c r="BF71" s="7"/>
+      <c r="BK71" s="7"/>
+    </row>
+    <row r="72" spans="2:63" x14ac:dyDescent="0.2">
+      <c r="BF72" s="7"/>
+      <c r="BK72" s="7"/>
+    </row>
+    <row r="73" spans="2:63" x14ac:dyDescent="0.2">
+      <c r="BF73" s="7"/>
+      <c r="BK73" s="7"/>
+    </row>
+    <row r="74" spans="2:63" x14ac:dyDescent="0.2">
+      <c r="BF74" s="7"/>
+      <c r="BK74" s="7"/>
+    </row>
+    <row r="75" spans="2:63" x14ac:dyDescent="0.2">
+      <c r="BF75" s="7"/>
+      <c r="BK75" s="7"/>
+    </row>
+    <row r="76" spans="2:63" x14ac:dyDescent="0.2">
+      <c r="BF76" s="7"/>
+      <c r="BK76" s="7"/>
+    </row>
+    <row r="77" spans="2:63" x14ac:dyDescent="0.2">
+      <c r="BF77" s="7"/>
+      <c r="BK77" s="7"/>
+    </row>
+    <row r="78" spans="2:63" x14ac:dyDescent="0.2">
+      <c r="BF78" s="7"/>
+      <c r="BK78" s="7"/>
+    </row>
+    <row r="79" spans="2:63" x14ac:dyDescent="0.2">
+      <c r="BF79" s="7"/>
+      <c r="BK79" s="7"/>
+    </row>
+    <row r="80" spans="2:63" x14ac:dyDescent="0.2">
+      <c r="BF80" s="7"/>
+      <c r="BK80" s="7"/>
+    </row>
+    <row r="81" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF81" s="7"/>
+      <c r="BK81" s="7"/>
+    </row>
+    <row r="82" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF82" s="7"/>
+      <c r="BK82" s="7"/>
+    </row>
+    <row r="83" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF83" s="7"/>
+      <c r="BK83" s="7"/>
+    </row>
+    <row r="84" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF84" s="7"/>
+      <c r="BK84" s="7"/>
+    </row>
+    <row r="85" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF85" s="7"/>
+      <c r="BK85" s="7"/>
+    </row>
+    <row r="86" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF86" s="7"/>
+      <c r="BK86" s="7"/>
+    </row>
+    <row r="87" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF87" s="7"/>
+      <c r="BK87" s="7"/>
+    </row>
+    <row r="88" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF88" s="7"/>
+      <c r="BK88" s="7"/>
+    </row>
+    <row r="89" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF89" s="7"/>
+      <c r="BK89" s="7"/>
+    </row>
+    <row r="90" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF90" s="7"/>
+      <c r="BK90" s="7"/>
+    </row>
+    <row r="91" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF91" s="7"/>
+      <c r="BK91" s="7"/>
+    </row>
+    <row r="92" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF92" s="7"/>
+      <c r="BK92" s="7"/>
+    </row>
+    <row r="93" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF93" s="7"/>
+      <c r="BK93" s="7"/>
+    </row>
+    <row r="94" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF94" s="7"/>
+      <c r="BK94" s="7"/>
+    </row>
+    <row r="95" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF95" s="7"/>
+      <c r="BK95" s="7"/>
+    </row>
+    <row r="96" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF96" s="7"/>
+      <c r="BK96" s="7"/>
+    </row>
+    <row r="97" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF97" s="7"/>
+      <c r="BK97" s="7"/>
+    </row>
+    <row r="98" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF98" s="7"/>
+      <c r="BK98" s="7"/>
+    </row>
+    <row r="99" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF99" s="7"/>
+      <c r="BK99" s="7"/>
+    </row>
+    <row r="100" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF100" s="7"/>
+      <c r="BK100" s="7"/>
+    </row>
+    <row r="101" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF101" s="7"/>
+      <c r="BK101" s="7"/>
+    </row>
+    <row r="102" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF102" s="7"/>
+      <c r="BK102" s="7"/>
+    </row>
+    <row r="103" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF103" s="7"/>
+      <c r="BK103" s="7"/>
+    </row>
+    <row r="104" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF104" s="7"/>
+      <c r="BK104" s="7"/>
+    </row>
+    <row r="105" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF105" s="7"/>
+      <c r="BK105" s="7"/>
+    </row>
+    <row r="106" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF106" s="7"/>
+      <c r="BK106" s="7"/>
+    </row>
+    <row r="107" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF107" s="7"/>
+      <c r="BK107" s="7"/>
+    </row>
+    <row r="108" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF108" s="7"/>
+      <c r="BK108" s="7"/>
+    </row>
+    <row r="109" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF109" s="7"/>
+      <c r="BK109" s="7"/>
+    </row>
+    <row r="110" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF110" s="7"/>
+      <c r="BK110" s="7"/>
+    </row>
+    <row r="111" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF111" s="7"/>
+      <c r="BK111" s="7"/>
+    </row>
+    <row r="112" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF112" s="7"/>
+      <c r="BK112" s="7"/>
+    </row>
+    <row r="113" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF113" s="7"/>
+      <c r="BK113" s="7"/>
+    </row>
+    <row r="114" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF114" s="7"/>
+      <c r="BK114" s="7"/>
+    </row>
+    <row r="115" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF115" s="7"/>
+      <c r="BK115" s="7"/>
+    </row>
+    <row r="116" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF116" s="7"/>
+      <c r="BK116" s="7"/>
+    </row>
+    <row r="117" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF117" s="7"/>
+      <c r="BK117" s="7"/>
+    </row>
+    <row r="118" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF118" s="7"/>
+      <c r="BK118" s="7"/>
+    </row>
+    <row r="119" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF119" s="7"/>
+      <c r="BK119" s="7"/>
+    </row>
+    <row r="120" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF120" s="7"/>
+      <c r="BK120" s="7"/>
+    </row>
+    <row r="121" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF121" s="7"/>
+      <c r="BK121" s="7"/>
+    </row>
+    <row r="122" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF122" s="7"/>
+      <c r="BK122" s="7"/>
+    </row>
+    <row r="123" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF123" s="7"/>
+      <c r="BK123" s="7"/>
+    </row>
+    <row r="124" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF124" s="7"/>
+      <c r="BK124" s="7"/>
+    </row>
+    <row r="125" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF125" s="7"/>
+      <c r="BK125" s="7"/>
+    </row>
+    <row r="126" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF126" s="7"/>
+      <c r="BK126" s="7"/>
+    </row>
+    <row r="127" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF127" s="7"/>
+      <c r="BK127" s="7"/>
+    </row>
+    <row r="128" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF128" s="7"/>
+      <c r="BK128" s="7"/>
+    </row>
+    <row r="129" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF129" s="7"/>
+      <c r="BK129" s="7"/>
+    </row>
+    <row r="130" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF130" s="7"/>
+      <c r="BK130" s="7"/>
+    </row>
+    <row r="131" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF131" s="7"/>
+      <c r="BK131" s="7"/>
+    </row>
+    <row r="132" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF132" s="7"/>
+      <c r="BK132" s="7"/>
+    </row>
+    <row r="133" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF133" s="7"/>
+      <c r="BK133" s="7"/>
+    </row>
+    <row r="134" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF134" s="7"/>
+      <c r="BK134" s="7"/>
+    </row>
+    <row r="135" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF135" s="7"/>
+      <c r="BK135" s="7"/>
+    </row>
+    <row r="136" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF136" s="7"/>
+      <c r="BK136" s="7"/>
+    </row>
+    <row r="137" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF137" s="7"/>
+      <c r="BK137" s="7"/>
+    </row>
+    <row r="138" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF138" s="7"/>
+      <c r="BK138" s="7"/>
+    </row>
+    <row r="139" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF139" s="7"/>
+      <c r="BK139" s="7"/>
+    </row>
+    <row r="140" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF140" s="7"/>
+      <c r="BK140" s="7"/>
+    </row>
+    <row r="141" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF141" s="7"/>
+      <c r="BK141" s="7"/>
+    </row>
+    <row r="142" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF142" s="7"/>
+      <c r="BK142" s="7"/>
+    </row>
+    <row r="143" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF143" s="7"/>
+      <c r="BK143" s="7"/>
+    </row>
+    <row r="144" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF144" s="7"/>
+      <c r="BK144" s="7"/>
+    </row>
+    <row r="145" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF145" s="7"/>
+      <c r="BK145" s="7"/>
+    </row>
+    <row r="146" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF146" s="7"/>
+      <c r="BK146" s="7"/>
+    </row>
+    <row r="147" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF147" s="7"/>
+      <c r="BK147" s="7"/>
+    </row>
+    <row r="148" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF148" s="7"/>
+      <c r="BK148" s="7"/>
+    </row>
+    <row r="149" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF149" s="7"/>
+      <c r="BK149" s="7"/>
+    </row>
+    <row r="150" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF150" s="7"/>
+      <c r="BK150" s="7"/>
+    </row>
+    <row r="151" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF151" s="7"/>
+      <c r="BK151" s="7"/>
+    </row>
+    <row r="152" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF152" s="7"/>
+      <c r="BK152" s="7"/>
+    </row>
+    <row r="153" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF153" s="7"/>
+      <c r="BK153" s="7"/>
+    </row>
+    <row r="154" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF154" s="7"/>
+      <c r="BK154" s="7"/>
+    </row>
+    <row r="155" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF155" s="7"/>
+      <c r="BK155" s="7"/>
+    </row>
+    <row r="156" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF156" s="7"/>
+      <c r="BK156" s="7"/>
+    </row>
+    <row r="157" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF157" s="7"/>
+      <c r="BK157" s="7"/>
+    </row>
+    <row r="158" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF158" s="7"/>
+      <c r="BK158" s="7"/>
+    </row>
+    <row r="159" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF159" s="7"/>
+      <c r="BK159" s="7"/>
+    </row>
+    <row r="160" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF160" s="7"/>
+      <c r="BK160" s="7"/>
+    </row>
+    <row r="161" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF161" s="7"/>
+      <c r="BK161" s="7"/>
+    </row>
+    <row r="162" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF162" s="7"/>
+      <c r="BK162" s="7"/>
+    </row>
+    <row r="163" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF163" s="7"/>
+      <c r="BK163" s="7"/>
+    </row>
+    <row r="164" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF164" s="7"/>
+      <c r="BK164" s="7"/>
+    </row>
+    <row r="165" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF165" s="7"/>
+      <c r="BK165" s="7"/>
+    </row>
+    <row r="166" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF166" s="7"/>
+      <c r="BK166" s="7"/>
+    </row>
+    <row r="167" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF167" s="7"/>
+      <c r="BK167" s="7"/>
+    </row>
+    <row r="168" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF168" s="7"/>
+      <c r="BK168" s="7"/>
+    </row>
+    <row r="169" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF169" s="7"/>
+      <c r="BK169" s="7"/>
+    </row>
+    <row r="170" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF170" s="7"/>
+      <c r="BK170" s="7"/>
+    </row>
+    <row r="171" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF171" s="7"/>
+    </row>
+    <row r="172" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF172" s="7"/>
+    </row>
+    <row r="173" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF173" s="7"/>
+    </row>
+    <row r="174" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF174" s="7"/>
+    </row>
+    <row r="175" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF175" s="7"/>
+    </row>
+    <row r="176" spans="58:63" x14ac:dyDescent="0.2">
+      <c r="BF176" s="7"/>
+    </row>
+    <row r="177" spans="58:58" x14ac:dyDescent="0.2">
+      <c r="BF177" s="7"/>
+    </row>
+    <row r="178" spans="58:58" x14ac:dyDescent="0.2">
+      <c r="BF178" s="7"/>
+    </row>
+    <row r="179" spans="58:58" x14ac:dyDescent="0.2">
+      <c r="BF179" s="7"/>
+    </row>
+    <row r="180" spans="58:58" x14ac:dyDescent="0.2">
+      <c r="BF180" s="7"/>
+    </row>
+    <row r="181" spans="58:58" x14ac:dyDescent="0.2">
+      <c r="BF181" s="7"/>
+    </row>
+    <row r="182" spans="58:58" x14ac:dyDescent="0.2">
+      <c r="BF182" s="7"/>
+    </row>
+    <row r="183" spans="58:58" x14ac:dyDescent="0.2">
+      <c r="BF183" s="7"/>
+    </row>
+    <row r="184" spans="58:58" x14ac:dyDescent="0.2">
+      <c r="BF184" s="7"/>
+    </row>
+    <row r="185" spans="58:58" x14ac:dyDescent="0.2">
+      <c r="BF185" s="7"/>
+    </row>
+    <row r="186" spans="58:58" x14ac:dyDescent="0.2">
+      <c r="BF186" s="7"/>
+    </row>
+    <row r="187" spans="58:58" x14ac:dyDescent="0.2">
+      <c r="BF187" s="7"/>
+    </row>
+    <row r="188" spans="58:58" x14ac:dyDescent="0.2">
+      <c r="BF188" s="7"/>
+    </row>
+    <row r="189" spans="58:58" x14ac:dyDescent="0.2">
+      <c r="BF189" s="7"/>
+    </row>
+    <row r="190" spans="58:58" x14ac:dyDescent="0.2">
+      <c r="BF190" s="7"/>
+    </row>
+    <row r="191" spans="58:58" x14ac:dyDescent="0.2">
+      <c r="BF191" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update FSC freshwater catch numbers from LGL report
</commit_message>
<xml_diff>
--- a/data-raw/freshwater-catch.xlsx
+++ b/data-raw/freshwater-catch.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\skrunchy2025\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FCE902D-13F1-481D-8064-DF2B457AEE42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{298FB934-2BA5-44A8-8D7D-60251A83E0E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E0CDEE87-6CC2-4107-81B9-F1AD4EA649A7}"/>
   </bookViews>
@@ -326,7 +326,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -384,7 +384,6 @@
     <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -401,7 +400,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="2" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -421,10 +420,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -899,15 +894,17 @@
         <v>0</v>
       </c>
       <c r="N2" s="7">
-        <v>1343</v>
+        <f>D2</f>
+        <v>525</v>
       </c>
       <c r="O2" s="7">
-        <v>2500</v>
+        <f>E2</f>
+        <v>1410</v>
       </c>
       <c r="P2" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q2" s="30" t="s">
+      <c r="Q2" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R2" s="7"/>
@@ -976,16 +973,18 @@
         <f t="shared" ref="M3:M47" si="4">SUM(J3,K3)</f>
         <v>0</v>
       </c>
-      <c r="N3" s="1">
-        <v>2600</v>
+      <c r="N3" s="7">
+        <f t="shared" ref="N3:O6" si="5">D3</f>
+        <v>341</v>
       </c>
       <c r="O3" s="7">
-        <v>6060</v>
+        <f t="shared" si="5"/>
+        <v>3625</v>
       </c>
       <c r="P3" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q3" s="30" t="s">
+      <c r="Q3" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R3" s="5"/>
@@ -1054,16 +1053,18 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N4" s="1">
-        <v>2280</v>
+      <c r="N4" s="7">
+        <f t="shared" si="5"/>
+        <v>421</v>
       </c>
       <c r="O4" s="7">
-        <v>7621</v>
+        <f t="shared" si="5"/>
+        <v>2210</v>
       </c>
       <c r="P4" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q4" s="30" t="s">
+      <c r="Q4" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R4" s="5"/>
@@ -1132,16 +1133,18 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N5" s="1">
-        <v>2500</v>
+      <c r="N5" s="7">
+        <f t="shared" si="5"/>
+        <v>329</v>
       </c>
       <c r="O5" s="7">
-        <v>9200</v>
+        <f t="shared" si="5"/>
+        <v>2230</v>
       </c>
       <c r="P5" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q5" s="30" t="s">
+      <c r="Q5" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R5" s="5"/>
@@ -1210,16 +1213,18 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N6" s="1">
-        <v>1976</v>
+      <c r="N6" s="7">
+        <f t="shared" si="5"/>
+        <v>453</v>
       </c>
       <c r="O6" s="7">
-        <v>8300</v>
+        <f t="shared" si="5"/>
+        <v>4366</v>
       </c>
       <c r="P6" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q6" s="30" t="s">
+      <c r="Q6" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R6" s="5"/>
@@ -1289,7 +1294,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="7">
         <v>1568</v>
       </c>
       <c r="O7" s="7">
@@ -1298,7 +1303,7 @@
       <c r="P7" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q7" s="30" t="s">
+      <c r="Q7" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R7" s="5"/>
@@ -1368,7 +1373,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="7">
         <v>3130</v>
       </c>
       <c r="O8" s="7">
@@ -1377,7 +1382,7 @@
       <c r="P8" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q8" s="30" t="s">
+      <c r="Q8" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R8" s="5"/>
@@ -1447,7 +1452,7 @@
         <f>SUM(J9,K9)</f>
         <v>0</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="7">
         <v>6236</v>
       </c>
       <c r="O9" s="7">
@@ -1456,7 +1461,7 @@
       <c r="P9" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q9" s="30" t="s">
+      <c r="Q9" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R9" s="5"/>
@@ -1526,7 +1531,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="7">
         <v>4318</v>
       </c>
       <c r="O10" s="7">
@@ -1535,7 +1540,7 @@
       <c r="P10" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q10" s="30" t="s">
+      <c r="Q10" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R10" s="5"/>
@@ -1605,7 +1610,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="7">
         <v>3745</v>
       </c>
       <c r="O11" s="7">
@@ -1614,7 +1619,7 @@
       <c r="P11" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q11" s="30" t="s">
+      <c r="Q11" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R11" s="5"/>
@@ -1684,7 +1689,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="7">
         <v>5414</v>
       </c>
       <c r="O12" s="7">
@@ -1693,7 +1698,7 @@
       <c r="P12" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q12" s="30" t="s">
+      <c r="Q12" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R12" s="5"/>
@@ -1763,7 +1768,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N13" s="1">
+      <c r="N13" s="7">
         <v>5112</v>
       </c>
       <c r="O13" s="7">
@@ -1772,7 +1777,7 @@
       <c r="P13" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q13" s="30" t="s">
+      <c r="Q13" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R13" s="5"/>
@@ -1842,7 +1847,7 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N14" s="1">
+      <c r="N14" s="7">
         <v>3167</v>
       </c>
       <c r="O14" s="7">
@@ -1851,7 +1856,7 @@
       <c r="P14" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q14" s="30" t="s">
+      <c r="Q14" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R14" s="5"/>
@@ -1921,8 +1926,8 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N15" s="36">
-        <v>3405</v>
+      <c r="N15" s="35">
+        <v>3404.5</v>
       </c>
       <c r="O15" s="7">
         <v>11361</v>
@@ -1930,7 +1935,7 @@
       <c r="P15" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q15" s="30" t="s">
+      <c r="Q15" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R15" s="5"/>
@@ -2000,16 +2005,16 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N16" s="1">
-        <v>4306</v>
+      <c r="N16" s="7">
+        <v>3642</v>
       </c>
       <c r="O16" s="7">
-        <v>9569</v>
+        <v>8718</v>
       </c>
       <c r="P16" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q16" s="30" t="s">
+      <c r="Q16" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R16" s="5"/>
@@ -2079,16 +2084,16 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N17" s="1">
-        <v>1638</v>
+      <c r="N17" s="7">
+        <v>2482.7593418310471</v>
       </c>
       <c r="O17" s="7">
-        <v>8140</v>
+        <v>7647</v>
       </c>
       <c r="P17" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q17" s="30" t="s">
+      <c r="Q17" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R17" s="5"/>
@@ -2158,16 +2163,16 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N18" s="1">
-        <v>714</v>
+      <c r="N18" s="7">
+        <v>900.70270925216892</v>
       </c>
       <c r="O18" s="7">
-        <v>5724</v>
+        <v>5104</v>
       </c>
       <c r="P18" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q18" s="30" t="s">
+      <c r="Q18" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R18" s="5"/>
@@ -2237,16 +2242,16 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N19" s="1">
-        <v>1164</v>
+      <c r="N19" s="7">
+        <v>1024.4556050986284</v>
       </c>
       <c r="O19" s="7">
-        <v>4828</v>
+        <v>4318</v>
       </c>
       <c r="P19" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q19" s="30" t="s">
+      <c r="Q19" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R19" s="5"/>
@@ -2315,16 +2320,16 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N20" s="1">
-        <v>1434</v>
+      <c r="N20" s="7">
+        <v>1065.5984587796249</v>
       </c>
       <c r="O20" s="7">
-        <v>6289</v>
+        <v>4383</v>
       </c>
       <c r="P20" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q20" s="31"/>
+      <c r="Q20" s="30"/>
       <c r="R20" s="5"/>
       <c r="S20" s="5"/>
       <c r="T20" s="5"/>
@@ -2390,16 +2395,16 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N21" s="1">
-        <v>1669</v>
+      <c r="N21" s="7">
+        <v>1841.3114670673194</v>
       </c>
       <c r="O21" s="7">
-        <v>9783</v>
+        <v>7537.1691601122393</v>
       </c>
       <c r="P21" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q21" s="31"/>
+      <c r="Q21" s="30"/>
       <c r="R21" s="5"/>
       <c r="S21" s="5"/>
       <c r="T21" s="5"/>
@@ -2465,16 +2470,16 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N22" s="1">
-        <v>1775</v>
+      <c r="N22" s="7">
+        <v>2122.1119808074445</v>
       </c>
       <c r="O22" s="7">
-        <v>15345</v>
+        <v>10750</v>
       </c>
       <c r="P22" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q22" s="31"/>
+      <c r="Q22" s="30"/>
       <c r="R22" s="5"/>
       <c r="S22" s="5"/>
       <c r="T22" s="5"/>
@@ -2540,16 +2545,16 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N23" s="1">
-        <v>991</v>
+      <c r="N23" s="7">
+        <v>1236.7631948819851</v>
       </c>
       <c r="O23" s="7">
-        <v>12296</v>
+        <v>10939</v>
       </c>
       <c r="P23" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q23" s="31"/>
+      <c r="Q23" s="30"/>
       <c r="R23" s="5"/>
       <c r="S23" s="5"/>
       <c r="T23" s="5"/>
@@ -2615,16 +2620,16 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N24" s="13">
-        <v>1000</v>
-      </c>
-      <c r="O24" s="23">
-        <v>10354</v>
+      <c r="N24" s="7">
+        <v>2161.4633233170166</v>
+      </c>
+      <c r="O24" s="7">
+        <v>7582</v>
       </c>
       <c r="P24" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q24" s="31"/>
+      <c r="Q24" s="30"/>
       <c r="R24" s="5"/>
       <c r="S24" s="5"/>
       <c r="T24" s="5" t="s">
@@ -2693,16 +2698,16 @@
         <f>SUM(J25,K25)</f>
         <v>0</v>
       </c>
-      <c r="N25" s="1">
-        <v>83</v>
+      <c r="N25" s="7">
+        <v>1640.1634517520476</v>
       </c>
       <c r="O25" s="7">
-        <v>6207</v>
+        <v>3912.8933133262135</v>
       </c>
       <c r="P25" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q25" s="32"/>
+      <c r="Q25" s="31"/>
       <c r="R25" s="5" t="s">
         <v>36</v>
       </c>
@@ -2780,16 +2785,16 @@
         <f>SUM(J26,K26)</f>
         <v>1092</v>
       </c>
-      <c r="N26" s="1">
-        <v>331</v>
+      <c r="N26" s="7">
+        <v>2499.7361750593709</v>
       </c>
       <c r="O26" s="7">
-        <v>10472</v>
+        <v>7642.8082590291433</v>
       </c>
       <c r="P26" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q26" s="32"/>
+      <c r="Q26" s="31"/>
       <c r="R26" s="5" t="s">
         <v>36</v>
       </c>
@@ -2857,16 +2862,16 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N27" s="1">
-        <v>158</v>
+      <c r="N27" s="7">
+        <v>2067.8571463190037</v>
       </c>
       <c r="O27" s="7">
-        <v>10924</v>
+        <v>6472.4001409068924</v>
       </c>
       <c r="P27" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q27" s="31"/>
+      <c r="Q27" s="30"/>
       <c r="R27" s="5"/>
       <c r="S27" s="5"/>
       <c r="T27" s="5"/>
@@ -2925,23 +2930,23 @@
         <v>1000</v>
       </c>
       <c r="L28" s="7">
-        <f t="shared" ref="L28:L32" si="5">SUM(F28,H28,I28)</f>
+        <f t="shared" ref="L28:L32" si="6">SUM(F28,H28,I28)</f>
         <v>2500</v>
       </c>
       <c r="M28" s="23">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N28" s="1">
-        <v>306</v>
+      <c r="N28" s="7">
+        <v>1914.7953763388746</v>
       </c>
       <c r="O28" s="7">
-        <v>6939</v>
+        <v>5498.4100135859335</v>
       </c>
       <c r="P28" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q28" s="31"/>
+      <c r="Q28" s="30"/>
       <c r="R28" s="5"/>
       <c r="S28" s="5"/>
       <c r="T28" s="5"/>
@@ -3000,23 +3005,23 @@
         <v>1000</v>
       </c>
       <c r="L29" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>2500</v>
       </c>
       <c r="M29" s="23">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N29" s="1">
-        <v>73</v>
+      <c r="N29" s="7">
+        <v>1335.9871322638492</v>
       </c>
       <c r="O29" s="7">
-        <v>6235</v>
+        <v>6928.7145708721309</v>
       </c>
       <c r="P29" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q29" s="31"/>
+      <c r="Q29" s="30"/>
       <c r="R29" s="5"/>
       <c r="S29" s="5"/>
       <c r="T29" s="5"/>
@@ -3083,16 +3088,16 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N30" s="1">
-        <v>114</v>
+      <c r="N30" s="7">
+        <v>1352</v>
       </c>
       <c r="O30" s="7">
-        <v>4816</v>
+        <v>4369.4293016087877</v>
       </c>
       <c r="P30" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q30" s="31"/>
+      <c r="Q30" s="30"/>
       <c r="R30" s="5"/>
       <c r="S30" s="5"/>
       <c r="T30" s="5"/>
@@ -3151,23 +3156,23 @@
         <v>1000</v>
       </c>
       <c r="L31" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>2500</v>
       </c>
       <c r="M31" s="23">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N31" s="1">
-        <v>439</v>
+      <c r="N31" s="7">
+        <v>1131</v>
       </c>
       <c r="O31" s="7">
-        <v>7887</v>
+        <v>6642.796308598884</v>
       </c>
       <c r="P31" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q31" s="31"/>
+      <c r="Q31" s="30"/>
       <c r="R31" s="5"/>
       <c r="S31" s="5"/>
       <c r="T31" s="5"/>
@@ -3226,23 +3231,23 @@
         <v>1000</v>
       </c>
       <c r="L32" s="7">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>2500</v>
       </c>
       <c r="M32" s="23">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="N32" s="1">
-        <v>476</v>
+      <c r="N32" s="7">
+        <v>1774.7928076382495</v>
       </c>
       <c r="O32" s="7">
-        <v>5576</v>
+        <v>4339.2319519918001</v>
       </c>
       <c r="P32" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q32" s="31"/>
+      <c r="Q32" s="30"/>
       <c r="R32" s="5"/>
       <c r="S32" s="5"/>
       <c r="T32" s="5"/>
@@ -3291,36 +3296,36 @@
         <v>1043</v>
       </c>
       <c r="E33" s="11">
-        <f t="shared" ref="E33:E41" si="6">SUM(F33:I33)</f>
+        <f t="shared" ref="E33:E41" si="7">SUM(F33:I33)</f>
         <v>2820</v>
       </c>
       <c r="F33" s="11">
         <v>2350</v>
       </c>
       <c r="G33" s="14">
-        <f>ROUND(0.2*SUM(F33,H33,I33),0)</f>
+        <f t="shared" ref="G33:G40" si="8">ROUND(0.2*SUM(F33,H33,I33),0)</f>
         <v>470</v>
       </c>
       <c r="J33" s="7"/>
       <c r="K33" s="7"/>
       <c r="L33" s="7">
-        <f>SUM(F33,H33,I33)</f>
+        <f t="shared" ref="L33:L38" si="9">SUM(F33,H33,I33)</f>
         <v>2350</v>
       </c>
       <c r="M33" s="23">
         <f>2720-F33</f>
         <v>370</v>
       </c>
-      <c r="N33" s="1">
-        <v>124</v>
+      <c r="N33" s="7">
+        <v>433.51609072844474</v>
       </c>
       <c r="O33" s="7">
-        <v>6115</v>
+        <v>5173</v>
       </c>
       <c r="P33" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q33" s="34" t="s">
+      <c r="Q33" s="33" t="s">
         <v>51</v>
       </c>
       <c r="R33" s="5"/>
@@ -3373,34 +3378,34 @@
         <v>1104</v>
       </c>
       <c r="E34" s="11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>2033</v>
       </c>
       <c r="F34" s="11">
         <v>1694</v>
       </c>
       <c r="G34" s="14">
-        <f>ROUND(0.2*SUM(F34,H34,I34),0)</f>
+        <f t="shared" si="8"/>
         <v>339</v>
       </c>
       <c r="L34" s="7">
-        <f>SUM(F34,H34,I34)</f>
+        <f t="shared" si="9"/>
         <v>1694</v>
       </c>
       <c r="M34" s="23">
         <f>2540-F34</f>
         <v>846</v>
       </c>
-      <c r="N34" s="1">
-        <v>366</v>
+      <c r="N34" s="7">
+        <v>1020.5538153344096</v>
       </c>
       <c r="O34" s="7">
-        <v>3764</v>
+        <v>4358</v>
       </c>
       <c r="P34" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q34" s="34" t="s">
+      <c r="Q34" s="33" t="s">
         <v>50</v>
       </c>
       <c r="R34" s="5"/>
@@ -3453,12 +3458,12 @@
         <v>645</v>
       </c>
       <c r="E35" s="11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>811</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="14">
-        <f>ROUND(0.2*SUM(F35,H35,I35),0)</f>
+        <f t="shared" si="8"/>
         <v>135</v>
       </c>
       <c r="H35" s="1">
@@ -3476,29 +3481,29 @@
         <v>131</v>
       </c>
       <c r="L35" s="7">
-        <f>SUM(F35,H35,I35)</f>
+        <f t="shared" si="9"/>
         <v>676</v>
       </c>
       <c r="M35" s="23">
-        <f t="shared" ref="M35:M45" si="7">SUM(J35,K35)</f>
+        <f t="shared" ref="M35:M45" si="10">SUM(J35,K35)</f>
         <v>282</v>
       </c>
-      <c r="N35" s="1">
-        <v>175</v>
+      <c r="N35" s="7">
+        <v>968.17880492663608</v>
       </c>
       <c r="O35" s="7">
-        <v>2533</v>
+        <v>2495</v>
       </c>
       <c r="P35" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q35" s="30" t="s">
+      <c r="Q35" s="29" t="s">
         <v>52</v>
       </c>
       <c r="R35" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S35" s="35"/>
+      <c r="S35" s="34"/>
       <c r="T35" s="5" t="s">
         <v>37</v>
       </c>
@@ -3547,12 +3552,12 @@
         <v>642</v>
       </c>
       <c r="E36" s="11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>2834</v>
       </c>
       <c r="F36" s="4"/>
       <c r="G36" s="14">
-        <f>ROUND(0.2*SUM(F36,H36,I36),0)</f>
+        <f t="shared" si="8"/>
         <v>472</v>
       </c>
       <c r="H36" s="1">
@@ -3570,29 +3575,29 @@
         <v>370</v>
       </c>
       <c r="L36" s="7">
-        <f>SUM(F36,H36,I36)</f>
+        <f t="shared" si="9"/>
         <v>2362</v>
       </c>
       <c r="M36" s="23">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>776</v>
       </c>
-      <c r="N36" s="1">
-        <v>19</v>
+      <c r="N36" s="7">
+        <v>429.76675775798543</v>
       </c>
       <c r="O36" s="7">
-        <v>2142</v>
+        <v>2186</v>
       </c>
       <c r="P36" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q36" s="34" t="s">
+      <c r="Q36" s="33" t="s">
         <v>53</v>
       </c>
       <c r="R36" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S36" s="35"/>
+      <c r="S36" s="34"/>
       <c r="T36" s="5" t="s">
         <v>37</v>
       </c>
@@ -3641,12 +3646,12 @@
         <v>604</v>
       </c>
       <c r="E37" s="11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>5437</v>
       </c>
       <c r="F37" s="4"/>
       <c r="G37" s="14">
-        <f>ROUND(0.2*SUM(F37,H37,I37),0)</f>
+        <f t="shared" si="8"/>
         <v>906</v>
       </c>
       <c r="H37" s="1">
@@ -3664,29 +3669,29 @@
         <v>276</v>
       </c>
       <c r="L37" s="7">
-        <f>SUM(F37,H37,I37)</f>
+        <f t="shared" si="9"/>
         <v>4531</v>
       </c>
       <c r="M37" s="23">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>473</v>
       </c>
-      <c r="N37" s="1">
-        <v>149</v>
+      <c r="N37" s="7">
+        <v>368.54113835565875</v>
       </c>
       <c r="O37" s="7">
-        <v>3365</v>
+        <v>3223</v>
       </c>
       <c r="P37" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q37" s="34" t="s">
+      <c r="Q37" s="33" t="s">
         <v>54</v>
       </c>
       <c r="R37" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S37" s="35"/>
+      <c r="S37" s="34"/>
       <c r="T37" s="5" t="s">
         <v>37</v>
       </c>
@@ -3735,12 +3740,12 @@
         <v>852</v>
       </c>
       <c r="E38" s="11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>5897</v>
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="14">
-        <f>ROUND(0.2*SUM(F38,H38,I38),0)</f>
+        <f t="shared" si="8"/>
         <v>983</v>
       </c>
       <c r="H38" s="1">
@@ -3758,29 +3763,29 @@
         <v>103</v>
       </c>
       <c r="L38" s="7">
-        <f>SUM(F38,H38,I38)</f>
+        <f t="shared" si="9"/>
         <v>4914</v>
       </c>
       <c r="M38" s="23">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>584</v>
       </c>
-      <c r="N38" s="1">
-        <v>515</v>
+      <c r="N38" s="7">
+        <v>913.85765148436599</v>
       </c>
       <c r="O38" s="7">
-        <v>5850</v>
+        <v>5961.1813888125944</v>
       </c>
       <c r="P38" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q38" s="34" t="s">
+      <c r="Q38" s="33" t="s">
         <v>55</v>
       </c>
       <c r="R38" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S38" s="35"/>
+      <c r="S38" s="34"/>
       <c r="T38" s="5" t="s">
         <v>37</v>
       </c>
@@ -3829,12 +3834,12 @@
         <v>499</v>
       </c>
       <c r="E39" s="11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3833</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="14">
-        <f>ROUND(0.2*SUM(F39,H39,I39),0)</f>
+        <f t="shared" si="8"/>
         <v>639</v>
       </c>
       <c r="H39" s="1">
@@ -3856,25 +3861,25 @@
         <v>3194</v>
       </c>
       <c r="M39" s="23">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>1651</v>
       </c>
-      <c r="N39" s="1">
-        <v>74</v>
+      <c r="N39" s="7">
+        <v>271.43748438833984</v>
       </c>
       <c r="O39" s="7">
-        <v>3532</v>
+        <v>3457.1106044664784</v>
       </c>
       <c r="P39" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q39" s="34" t="s">
+      <c r="Q39" s="33" t="s">
         <v>55</v>
       </c>
       <c r="R39" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S39" s="35"/>
+      <c r="S39" s="34"/>
       <c r="T39" s="5" t="s">
         <v>37</v>
       </c>
@@ -3923,12 +3928,12 @@
         <v>538</v>
       </c>
       <c r="E40" s="11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1488</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="14">
-        <f>ROUND(0.2*SUM(F40,H40,I40),0)</f>
+        <f t="shared" si="8"/>
         <v>248</v>
       </c>
       <c r="H40" s="1">
@@ -3950,25 +3955,25 @@
         <v>1240</v>
       </c>
       <c r="M40" s="23">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>909</v>
       </c>
-      <c r="N40" s="1">
-        <v>239</v>
+      <c r="N40" s="7">
+        <v>802.12138508513249</v>
       </c>
       <c r="O40" s="7">
-        <v>4474</v>
+        <v>3814</v>
       </c>
       <c r="P40" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q40" s="31" t="s">
+      <c r="Q40" s="30" t="s">
         <v>40</v>
       </c>
       <c r="R40" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S40" s="35"/>
+      <c r="S40" s="34"/>
       <c r="T40" s="5" t="s">
         <v>37</v>
       </c>
@@ -4017,12 +4022,12 @@
         <v>530</v>
       </c>
       <c r="E41" s="11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="F41" s="4"/>
       <c r="G41" s="14">
-        <f t="shared" ref="G38:G48" si="8">ROUND(0.2*SUM(F41,H41,I41),0)</f>
+        <f t="shared" ref="G41:G47" si="11">ROUND(0.2*SUM(F41,H41,I41),0)</f>
         <v>0</v>
       </c>
       <c r="H41" s="1">
@@ -4042,25 +4047,25 @@
         <v>0</v>
       </c>
       <c r="M41" s="23">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="N41" s="1">
-        <v>509</v>
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="N41" s="7">
+        <v>1029.8845799671176</v>
       </c>
       <c r="O41" s="7">
-        <v>5983</v>
+        <v>4209</v>
       </c>
       <c r="P41" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q41" s="34" t="s">
+      <c r="Q41" s="33" t="s">
         <v>48</v>
       </c>
       <c r="R41" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="S41" s="35"/>
+      <c r="S41" s="34"/>
       <c r="T41" s="5"/>
       <c r="U41" s="5"/>
       <c r="V41" s="7"/>
@@ -4134,25 +4139,25 @@
         <v>762</v>
       </c>
       <c r="M42" s="23">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>141</v>
       </c>
-      <c r="N42" s="1">
-        <v>180</v>
+      <c r="N42" s="7">
+        <v>458.42273579665135</v>
       </c>
       <c r="O42" s="7">
-        <v>4460</v>
+        <v>4671</v>
       </c>
       <c r="P42" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q42" s="31" t="s">
+      <c r="Q42" s="30" t="s">
         <v>39</v>
       </c>
       <c r="R42" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S42" s="35"/>
+      <c r="S42" s="34"/>
       <c r="T42" s="5"/>
       <c r="U42" s="5"/>
       <c r="V42" s="7"/>
@@ -4226,25 +4231,25 @@
         <v>1073</v>
       </c>
       <c r="M43" s="23">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>452</v>
       </c>
-      <c r="N43" s="1">
-        <v>329</v>
+      <c r="N43" s="7">
+        <v>507.8023032558001</v>
       </c>
       <c r="O43" s="7">
-        <v>3904</v>
+        <v>3932</v>
       </c>
       <c r="P43" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="Q43" s="31" t="s">
+      <c r="Q43" s="30" t="s">
         <v>41</v>
       </c>
       <c r="R43" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S43" s="35"/>
+      <c r="S43" s="34"/>
       <c r="T43" s="5"/>
       <c r="U43" s="5"/>
       <c r="V43" s="7"/>
@@ -4276,7 +4281,7 @@
       <c r="BF43" s="7"/>
       <c r="BK43" s="7"/>
     </row>
-    <row r="44" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1">
         <v>2021</v>
       </c>
@@ -4295,7 +4300,7 @@
       </c>
       <c r="F44" s="11"/>
       <c r="G44" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="H44" s="1">
@@ -4313,27 +4318,29 @@
         <v>380</v>
       </c>
       <c r="L44" s="7">
-        <f t="shared" ref="L44:L48" si="9">SUM(F44,H44,I44)</f>
+        <f t="shared" ref="L44:L48" si="12">SUM(F44,H44,I44)</f>
         <v>0</v>
       </c>
       <c r="M44" s="23">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>380</v>
       </c>
-      <c r="N44" s="7"/>
-      <c r="O44" s="29">
-        <v>4192</v>
+      <c r="N44" s="7">
+        <v>256.38768738652419</v>
+      </c>
+      <c r="O44" s="7">
+        <v>3801.7564016744309</v>
       </c>
       <c r="P44" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="Q44" s="33" t="s">
+      <c r="Q44" s="32" t="s">
         <v>42</v>
       </c>
       <c r="R44" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S44" s="35"/>
+      <c r="S44" s="34"/>
       <c r="T44" s="5"/>
       <c r="U44" s="5"/>
       <c r="V44" s="7"/>
@@ -4365,7 +4372,7 @@
       <c r="BF44" s="7"/>
       <c r="BK44" s="7"/>
     </row>
-    <row r="45" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="1">
         <v>2022</v>
       </c>
@@ -4384,7 +4391,7 @@
       </c>
       <c r="F45" s="11"/>
       <c r="G45" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="H45" s="1">
@@ -4402,27 +4409,29 @@
         <v>274</v>
       </c>
       <c r="L45" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="M45" s="23">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>347</v>
       </c>
-      <c r="N45" s="7"/>
-      <c r="O45" s="29">
-        <v>2959</v>
+      <c r="N45" s="7">
+        <v>360.96238288924758</v>
+      </c>
+      <c r="O45" s="7">
+        <v>2959.9180100198664</v>
       </c>
       <c r="P45" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="Q45" s="33" t="s">
+      <c r="Q45" s="32" t="s">
         <v>44</v>
       </c>
       <c r="R45" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S45" s="35"/>
+      <c r="S45" s="34"/>
       <c r="T45" s="5"/>
       <c r="U45" s="5"/>
       <c r="V45" s="7"/>
@@ -4454,7 +4463,7 @@
       <c r="BF45" s="7"/>
       <c r="BK45" s="7"/>
     </row>
-    <row r="46" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
         <v>2023</v>
       </c>
@@ -4468,7 +4477,7 @@
         <v>646</v>
       </c>
       <c r="E46" s="11">
-        <f t="shared" ref="E46:E48" si="10">SUM(F46:I46)</f>
+        <f t="shared" ref="E46:E48" si="13">SUM(F46:I46)</f>
         <v>85</v>
       </c>
       <c r="F46" s="11"/>
@@ -4498,20 +4507,22 @@
         <f t="shared" si="4"/>
         <v>258</v>
       </c>
-      <c r="N46" s="7"/>
-      <c r="O46" s="29">
-        <v>3369</v>
+      <c r="N46" s="7">
+        <v>377.52232980028259</v>
+      </c>
+      <c r="O46" s="7">
+        <v>3713</v>
       </c>
       <c r="P46" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="Q46" s="33" t="s">
+      <c r="Q46" s="32" t="s">
         <v>43</v>
       </c>
       <c r="R46" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S46" s="35"/>
+      <c r="S46" s="34"/>
       <c r="T46" s="5"/>
       <c r="U46" s="5"/>
       <c r="V46" s="7"/>
@@ -4543,7 +4554,7 @@
       <c r="BF46" s="7"/>
       <c r="BK46" s="7"/>
     </row>
-    <row r="47" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:63" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1">
         <v>2024</v>
       </c>
@@ -4557,12 +4568,12 @@
         <v>482</v>
       </c>
       <c r="E47" s="11">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>1</v>
       </c>
       <c r="F47" s="11"/>
       <c r="G47" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="H47" s="1">
@@ -4580,27 +4591,29 @@
         <v>2</v>
       </c>
       <c r="L47" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>1</v>
       </c>
       <c r="M47" s="23">
         <f t="shared" si="4"/>
         <v>18</v>
       </c>
-      <c r="N47" s="7"/>
-      <c r="O47" s="29">
-        <v>1860</v>
+      <c r="N47" s="7">
+        <v>528.62413335868473</v>
+      </c>
+      <c r="O47" s="7">
+        <v>1927</v>
       </c>
       <c r="P47" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="Q47" s="33" t="s">
+      <c r="Q47" s="32" t="s">
         <v>45</v>
       </c>
       <c r="R47" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S47" s="35"/>
+      <c r="S47" s="34"/>
       <c r="T47" s="5"/>
       <c r="U47" s="5"/>
       <c r="V47" s="7"/>
@@ -4640,7 +4653,7 @@
       <c r="C48" s="19"/>
       <c r="D48" s="19"/>
       <c r="E48" s="11">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>23</v>
       </c>
       <c r="F48" s="4"/>
@@ -4663,7 +4676,7 @@
         <v>21</v>
       </c>
       <c r="L48" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>19</v>
       </c>
       <c r="M48" s="23">
@@ -4677,13 +4690,13 @@
       <c r="P48" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="Q48" s="33" t="s">
+      <c r="Q48" s="32" t="s">
         <v>46</v>
       </c>
       <c r="R48" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="S48" s="35"/>
+      <c r="S48" s="34"/>
       <c r="T48" s="5"/>
       <c r="U48" s="5"/>
       <c r="V48" s="5"/>
@@ -4724,9 +4737,9 @@
       <c r="N49" s="7"/>
       <c r="O49"/>
       <c r="P49" s="5"/>
-      <c r="Q49" s="33"/>
+      <c r="Q49" s="32"/>
       <c r="R49" s="5"/>
-      <c r="S49" s="35"/>
+      <c r="S49" s="34"/>
       <c r="T49" s="5"/>
       <c r="U49" s="5"/>
       <c r="V49" s="5"/>
@@ -4810,7 +4823,7 @@
       <c r="E52" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="S52" s="35"/>
+      <c r="S52" s="34"/>
       <c r="AN52" s="7"/>
       <c r="AO52" s="7"/>
       <c r="AP52" s="7"/>

</xml_diff>

<commit_message>
Update run reconstruction with new FSC catch numbers from LGL report
</commit_message>
<xml_diff>
--- a/data-raw/freshwater-catch.xlsx
+++ b/data-raw/freshwater-catch.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\skrunchy2025\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D32B37B-05F2-40D6-B03F-1D4AE51D0B6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C265F36-B12C-4570-B6DD-5C5FEACD6897}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E0CDEE87-6CC2-4107-81B9-F1AD4EA649A7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="56">
   <si>
     <t>Year</t>
   </si>
@@ -125,9 +125,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>Source</t>
-  </si>
-  <si>
     <t>Winther et al. 2024</t>
   </si>
   <si>
@@ -135,9 +132,6 @@
   </si>
   <si>
     <t>LW: Double check rec catch above Terrace for 2002, 2003, 2007</t>
-  </si>
-  <si>
-    <t>LW, FN catch above Terrace from AFS</t>
   </si>
   <si>
     <t>Creel survey?</t>
@@ -207,6 +201,9 @@
   </si>
   <si>
     <t>AFS</t>
+  </si>
+  <si>
+    <t>General source</t>
   </si>
 </sst>
 </file>
@@ -731,7 +728,7 @@
     <col min="5" max="12" width="8.7109375" style="1"/>
     <col min="13" max="13" width="8.42578125" style="19" customWidth="1"/>
     <col min="14" max="15" width="7.5703125" style="1" customWidth="1"/>
-    <col min="16" max="16" width="34.42578125" style="1" customWidth="1"/>
+    <col min="16" max="16" width="24.5703125" style="1" customWidth="1"/>
     <col min="17" max="17" width="37.7109375" style="3" customWidth="1"/>
     <col min="18" max="18" width="32.5703125" style="1" customWidth="1"/>
     <col min="19" max="19" width="20.140625" style="1" customWidth="1"/>
@@ -807,19 +804,19 @@
         <v>12</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="Q1" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="R1" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="S1" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="R1" s="18" t="s">
-        <v>34</v>
-      </c>
-      <c r="S1" s="18" t="s">
-        <v>48</v>
-      </c>
       <c r="T1" s="18" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="U1" s="18"/>
       <c r="V1" s="20"/>
@@ -904,14 +901,14 @@
         <v>2500</v>
       </c>
       <c r="P2" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q2" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R2" s="7"/>
       <c r="S2" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T2" s="7"/>
       <c r="U2" s="7"/>
@@ -984,14 +981,14 @@
         <v>6060</v>
       </c>
       <c r="P3" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q3" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R3" s="5"/>
       <c r="S3" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T3" s="5"/>
       <c r="U3" s="5"/>
@@ -1064,14 +1061,14 @@
         <v>7621</v>
       </c>
       <c r="P4" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q4" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R4" s="5"/>
       <c r="S4" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T4" s="5"/>
       <c r="U4" s="5"/>
@@ -1144,14 +1141,14 @@
         <v>9200</v>
       </c>
       <c r="P5" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q5" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R5" s="5"/>
       <c r="S5" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T5" s="5"/>
       <c r="U5" s="5"/>
@@ -1224,14 +1221,14 @@
         <v>8300</v>
       </c>
       <c r="P6" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q6" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R6" s="5"/>
       <c r="S6" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T6" s="5"/>
       <c r="U6" s="5"/>
@@ -1305,14 +1302,14 @@
         <v>7900</v>
       </c>
       <c r="P7" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q7" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R7" s="5"/>
       <c r="S7" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T7" s="5"/>
       <c r="U7" s="5"/>
@@ -1386,14 +1383,14 @@
         <v>10300</v>
       </c>
       <c r="P8" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q8" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R8" s="5"/>
       <c r="S8" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T8" s="5"/>
       <c r="U8" s="5"/>
@@ -1467,14 +1464,14 @@
         <v>10653</v>
       </c>
       <c r="P9" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q9" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R9" s="5"/>
       <c r="S9" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T9" s="5"/>
       <c r="U9" s="5"/>
@@ -1548,14 +1545,14 @@
         <v>7900</v>
       </c>
       <c r="P10" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q10" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R10" s="5"/>
       <c r="S10" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T10" s="5"/>
       <c r="U10" s="5"/>
@@ -1629,14 +1626,14 @@
         <v>13700</v>
       </c>
       <c r="P11" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q11" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R11" s="5"/>
       <c r="S11" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T11" s="5"/>
       <c r="U11" s="5"/>
@@ -1710,14 +1707,14 @@
         <v>9400</v>
       </c>
       <c r="P12" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q12" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R12" s="5"/>
       <c r="S12" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T12" s="5"/>
       <c r="U12" s="5"/>
@@ -1791,14 +1788,14 @@
         <v>17855</v>
       </c>
       <c r="P13" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q13" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R13" s="5"/>
       <c r="S13" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T13" s="5"/>
       <c r="U13" s="5"/>
@@ -1872,14 +1869,14 @@
         <v>11700</v>
       </c>
       <c r="P14" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q14" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R14" s="5"/>
       <c r="S14" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T14" s="5"/>
       <c r="U14" s="5"/>
@@ -1953,14 +1950,14 @@
         <v>11361</v>
       </c>
       <c r="P15" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q15" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R15" s="5"/>
       <c r="S15" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T15" s="5"/>
       <c r="U15" s="5"/>
@@ -2034,14 +2031,14 @@
         <v>8718</v>
       </c>
       <c r="P16" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q16" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R16" s="5"/>
       <c r="S16" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T16" s="5"/>
       <c r="U16" s="5"/>
@@ -2115,14 +2112,14 @@
         <v>7647</v>
       </c>
       <c r="P17" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q17" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R17" s="5"/>
       <c r="S17" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T17" s="5"/>
       <c r="U17" s="5"/>
@@ -2196,14 +2193,14 @@
         <v>5104</v>
       </c>
       <c r="P18" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q18" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R18" s="5"/>
       <c r="S18" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T18" s="5"/>
       <c r="U18" s="5"/>
@@ -2277,14 +2274,14 @@
         <v>4318</v>
       </c>
       <c r="P19" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q19" s="29" t="s">
         <v>27</v>
       </c>
       <c r="R19" s="5"/>
       <c r="S19" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T19" s="5"/>
       <c r="U19" s="5"/>
@@ -2357,12 +2354,12 @@
         <v>4383</v>
       </c>
       <c r="P20" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q20" s="30"/>
       <c r="R20" s="5"/>
       <c r="S20" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T20" s="5"/>
       <c r="U20" s="5"/>
@@ -2434,12 +2431,12 @@
         <v>7537.1691601122393</v>
       </c>
       <c r="P21" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q21" s="30"/>
       <c r="R21" s="5"/>
       <c r="S21" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T21" s="5"/>
       <c r="U21" s="5"/>
@@ -2511,12 +2508,12 @@
         <v>10750</v>
       </c>
       <c r="P22" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q22" s="30"/>
       <c r="R22" s="5"/>
       <c r="S22" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T22" s="5"/>
       <c r="U22" s="5"/>
@@ -2588,12 +2585,12 @@
         <v>10939</v>
       </c>
       <c r="P23" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q23" s="30"/>
       <c r="R23" s="5"/>
       <c r="S23" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T23" s="5"/>
       <c r="U23" s="5"/>
@@ -2665,12 +2662,12 @@
         <v>7582</v>
       </c>
       <c r="P24" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q24" s="30"/>
       <c r="R24" s="5"/>
       <c r="S24" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T24" s="5"/>
       <c r="U24" s="5"/>
@@ -2743,14 +2740,14 @@
         <v>3912.8933133262135</v>
       </c>
       <c r="P25" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q25" s="31"/>
       <c r="R25" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="S25" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T25" s="5"/>
       <c r="U25" s="5"/>
@@ -2832,14 +2829,14 @@
         <v>7642.8082590291433</v>
       </c>
       <c r="P26" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q26" s="31"/>
       <c r="R26" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="S26" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T26" s="5"/>
       <c r="U26" s="5"/>
@@ -2911,12 +2908,12 @@
         <v>6472.4001409068924</v>
       </c>
       <c r="P27" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q27" s="30"/>
       <c r="R27" s="5"/>
       <c r="S27" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T27" s="5"/>
       <c r="U27" s="5"/>
@@ -2988,12 +2985,12 @@
         <v>5498.4100135859335</v>
       </c>
       <c r="P28" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q28" s="30"/>
       <c r="R28" s="5"/>
       <c r="S28" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T28" s="5"/>
       <c r="U28" s="5"/>
@@ -3065,12 +3062,12 @@
         <v>6928.7145708721309</v>
       </c>
       <c r="P29" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q29" s="30"/>
       <c r="R29" s="5"/>
       <c r="S29" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T29" s="5"/>
       <c r="U29" s="5"/>
@@ -3143,12 +3140,12 @@
         <v>4369.4293016087877</v>
       </c>
       <c r="P30" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q30" s="30"/>
       <c r="R30" s="5"/>
       <c r="S30" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T30" s="5"/>
       <c r="U30" s="5"/>
@@ -3220,12 +3217,12 @@
         <v>6642.796308598884</v>
       </c>
       <c r="P31" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q31" s="30"/>
       <c r="R31" s="5"/>
       <c r="S31" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T31" s="5"/>
       <c r="U31" s="5"/>
@@ -3297,12 +3294,12 @@
         <v>4339.2319519918001</v>
       </c>
       <c r="P32" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q32" s="30"/>
       <c r="R32" s="5"/>
       <c r="S32" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T32" s="5"/>
       <c r="U32" s="5"/>
@@ -3377,17 +3374,17 @@
         <v>5173</v>
       </c>
       <c r="P33" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q33" s="33" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="R33" s="5"/>
       <c r="S33" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T33" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="U33" s="5"/>
       <c r="V33" s="7"/>
@@ -3459,17 +3456,17 @@
         <v>4358</v>
       </c>
       <c r="P34" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q34" s="33" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="R34" s="5"/>
       <c r="S34" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T34" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="U34" s="5"/>
       <c r="V34" s="7"/>
@@ -3553,19 +3550,19 @@
         <v>2495</v>
       </c>
       <c r="P35" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q35" s="29" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="R35" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="S35" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T35" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="U35" s="5"/>
       <c r="V35" s="7"/>
@@ -3649,19 +3646,19 @@
         <v>2186</v>
       </c>
       <c r="P36" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q36" s="33" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="R36" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="S36" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T36" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="U36" s="5"/>
       <c r="V36" s="7"/>
@@ -3745,19 +3742,19 @@
         <v>3223</v>
       </c>
       <c r="P37" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q37" s="33" t="s">
+        <v>51</v>
+      </c>
+      <c r="R37" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="S37" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="R37" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="S37" s="7" t="s">
-        <v>55</v>
-      </c>
       <c r="T37" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="U37" s="5"/>
       <c r="V37" s="7"/>
@@ -3841,19 +3838,19 @@
         <v>5961.1813888125944</v>
       </c>
       <c r="P38" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q38" s="33" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="R38" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="S38" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T38" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="U38" s="5"/>
       <c r="V38" s="7"/>
@@ -3937,19 +3934,19 @@
         <v>3457.1106044664784</v>
       </c>
       <c r="P39" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q39" s="33" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="R39" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="S39" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T39" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="U39" s="5"/>
       <c r="V39" s="7"/>
@@ -4033,19 +4030,19 @@
         <v>3814</v>
       </c>
       <c r="P40" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q40" s="30" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="R40" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="S40" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T40" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="U40" s="5"/>
       <c r="V40" s="7"/>
@@ -4127,16 +4124,16 @@
         <v>4209</v>
       </c>
       <c r="P41" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q41" s="33" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="R41" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="S41" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T41" s="5"/>
       <c r="U41" s="5"/>
@@ -4221,16 +4218,16 @@
         <v>4671</v>
       </c>
       <c r="P42" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q42" s="30" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="R42" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="S42" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T42" s="5"/>
       <c r="U42" s="5"/>
@@ -4315,16 +4312,16 @@
         <v>3932</v>
       </c>
       <c r="P43" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q43" s="30" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="R43" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="S43" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T43" s="5"/>
       <c r="U43" s="5"/>
@@ -4407,17 +4404,15 @@
       <c r="O44" s="7">
         <v>3801.7564016744309</v>
       </c>
-      <c r="P44" s="5" t="s">
+      <c r="P44" s="5"/>
+      <c r="Q44" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="R44" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="Q44" s="32" t="s">
-        <v>41</v>
-      </c>
-      <c r="R44" s="5" t="s">
-        <v>35</v>
-      </c>
       <c r="S44" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T44" s="5"/>
       <c r="U44" s="5"/>
@@ -4500,17 +4495,15 @@
       <c r="O45" s="7">
         <v>2959.9180100198664</v>
       </c>
-      <c r="P45" s="5" t="s">
+      <c r="P45" s="5"/>
+      <c r="Q45" s="32" t="s">
+        <v>41</v>
+      </c>
+      <c r="R45" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="Q45" s="32" t="s">
-        <v>43</v>
-      </c>
-      <c r="R45" s="5" t="s">
-        <v>35</v>
-      </c>
       <c r="S45" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T45" s="5"/>
       <c r="U45" s="5"/>
@@ -4593,17 +4586,15 @@
       <c r="O46" s="7">
         <v>3713</v>
       </c>
-      <c r="P46" s="5" t="s">
+      <c r="P46" s="5"/>
+      <c r="Q46" s="32" t="s">
+        <v>40</v>
+      </c>
+      <c r="R46" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="Q46" s="32" t="s">
-        <v>42</v>
-      </c>
-      <c r="R46" s="5" t="s">
-        <v>35</v>
-      </c>
       <c r="S46" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T46" s="5"/>
       <c r="U46" s="5"/>
@@ -4686,17 +4677,15 @@
       <c r="O47" s="7">
         <v>1927</v>
       </c>
-      <c r="P47" s="5" t="s">
+      <c r="P47" s="5"/>
+      <c r="Q47" s="32" t="s">
+        <v>42</v>
+      </c>
+      <c r="R47" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="Q47" s="32" t="s">
-        <v>44</v>
-      </c>
-      <c r="R47" s="5" t="s">
-        <v>35</v>
-      </c>
       <c r="S47" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="T47" s="5"/>
       <c r="U47" s="5"/>
@@ -4771,17 +4760,15 @@
       <c r="O48">
         <v>3270</v>
       </c>
-      <c r="P48" s="5" t="s">
+      <c r="P48" s="5"/>
+      <c r="Q48" s="32" t="s">
+        <v>43</v>
+      </c>
+      <c r="R48" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="Q48" s="32" t="s">
-        <v>45</v>
-      </c>
-      <c r="R48" s="5" t="s">
-        <v>35</v>
-      </c>
       <c r="S48" s="34" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="T48" s="5"/>
       <c r="U48" s="5"/>
@@ -4991,14 +4978,14 @@
     </row>
     <row r="61" spans="1:63" x14ac:dyDescent="0.2">
       <c r="E61" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="BF61" s="7"/>
       <c r="BK61" s="7"/>
     </row>
     <row r="62" spans="1:63" x14ac:dyDescent="0.2">
       <c r="E62" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="BF62" s="7"/>
       <c r="BK62" s="7"/>

</xml_diff>

<commit_message>
Update raw data readme for freshwater catch
</commit_message>
<xml_diff>
--- a/data-raw/freshwater-catch.xlsx
+++ b/data-raw/freshwater-catch.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\skrunchy2025\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C265F36-B12C-4570-B6DD-5C5FEACD6897}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7480D243-972A-45A9-B176-D78F873E10AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E0CDEE87-6CC2-4107-81B9-F1AD4EA649A7}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E0CDEE87-6CC2-4107-81B9-F1AD4EA649A7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -732,7 +732,7 @@
     <col min="17" max="17" width="37.7109375" style="3" customWidth="1"/>
     <col min="18" max="18" width="32.5703125" style="1" customWidth="1"/>
     <col min="19" max="19" width="20.140625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="24.140625" style="1" customWidth="1"/>
+    <col min="20" max="20" width="51.140625" style="1" customWidth="1"/>
     <col min="21" max="24" width="7.5703125" style="1" customWidth="1"/>
     <col min="25" max="26" width="8.85546875" style="1" customWidth="1"/>
     <col min="27" max="30" width="7.5703125" style="1" customWidth="1"/>
@@ -2898,7 +2898,7 @@
         <v>5000</v>
       </c>
       <c r="M27" s="23">
-        <f t="shared" si="4"/>
+        <f>SUM(J27,K27)</f>
         <v>0</v>
       </c>
       <c r="N27" s="7">
@@ -3360,7 +3360,7 @@
       <c r="J33" s="7"/>
       <c r="K33" s="7"/>
       <c r="L33" s="7">
-        <f t="shared" ref="L33:L38" si="8">SUM(F33,H33,I33)</f>
+        <f>SUM(F33,H33,I33)</f>
         <v>2350</v>
       </c>
       <c r="M33" s="23">
@@ -3442,7 +3442,7 @@
         <v>339</v>
       </c>
       <c r="L34" s="7">
-        <f t="shared" si="8"/>
+        <f>SUM(F34,H34,I34)</f>
         <v>1694</v>
       </c>
       <c r="M34" s="23">
@@ -3536,7 +3536,7 @@
         <v>131</v>
       </c>
       <c r="L35" s="7">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="L33:L38" si="8">SUM(F35,H35,I35)</f>
         <v>676</v>
       </c>
       <c r="M35" s="23">

</xml_diff>